<commit_message>
docs: document Phase 1 S3 and IAM progress
</commit_message>
<xml_diff>
--- a/docs/reference/CloudVault_Command_Notes.xlsx
+++ b/docs/reference/CloudVault_Command_Notes.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git" sheetId="1" r:id="R7df35f5a59a44972"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AWS" sheetId="2" r:id="R7fd2e4ced36945dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PowerShell" sheetId="3" r:id="R5d7cbf5444724718"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git" sheetId="1" r:id="R35df907d7fff4e8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AWS" sheetId="2" r:id="R2f41afc885e44f1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PowerShell" sheetId="3" r:id="R6d889de494064163"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -105,7 +105,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="53">
+  <x:cellXfs count="54">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -205,6 +205,9 @@
     <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1091,8 +1094,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re62dede2510e493c"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43db8b68a8d1429b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c6aa9abc06c480a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58a4cccfc5cc4985"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1101,14 +1104,14 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="44" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="48" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="38" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="40" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="44" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="38" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="28" customHeight="1">
+    <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
       <x:c r="A1" s="40" t="str">
         <x:v>AWS CLI Command Reference</x:v>
       </x:c>
@@ -1117,16 +1120,23 @@
       <x:c r="D1" s="40"/>
       <x:c r="E1" s="40"/>
     </x:row>
-    <x:row r="2" ht="42" customHeight="1">
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="12" t="str">
-        <x:v>AWS CLI commands introduced for CloudVault Phase 0: authentication, identity verification, budgets, IAM, and basic S3 practice.</x:v>
+        <x:v>AWS CLI commands used across CloudVault Phase 0 and Phase 1: temporary authentication, identity verification, budgets, IAM, S3 storage, versioning, and least-privilege validation.</x:v>
       </x:c>
       <x:c r="B2" s="12"/>
       <x:c r="C2" s="12"/>
       <x:c r="D2" s="12"/>
       <x:c r="E2" s="12"/>
     </x:row>
-    <x:row r="4">
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="26"/>
+      <x:c r="B3" s="26"/>
+      <x:c r="C3" s="26"/>
+      <x:c r="D3" s="26"/>
+      <x:c r="E3" s="26"/>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="20" t="str">
         <x:v>Command</x:v>
       </x:c>
@@ -1143,7 +1153,7 @@
         <x:v>Notes / Cautions</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
+    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A5" s="27" t="str">
         <x:v>aws --version</x:v>
       </x:c>
@@ -1160,7 +1170,7 @@
         <x:v>If not recognized, inspect PATH or reopen PowerShell after installation.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A6" s="27" t="str">
         <x:v>aws configure list-profiles</x:v>
       </x:c>
@@ -1177,58 +1187,58 @@
         <x:v>Profiles are usually stored in AWS CLI config/credentials files.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
+    <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A7" s="27" t="str">
-        <x:v>aws configure sso --profile cloudvault</x:v>
+        <x:v>aws login --profile cloudvault</x:v>
       </x:c>
       <x:c r="B7" s="27" t="str">
         <x:v>Authentication</x:v>
       </x:c>
       <x:c r="C7" s="27" t="str">
-        <x:v>Starts interactive configuration of an IAM Identity Center (SSO) profile named cloudvault.</x:v>
+        <x:v>Starts browser-based AWS sign-in for the cloudvault profile and obtains temporary local-development credentials.</x:v>
       </x:c>
       <x:c r="D7" s="27" t="str">
-        <x:v>Use to set up temporary/federated CLI access instead of long-lived access keys.</x:v>
+        <x:v>Use at the beginning of a CloudVault CLI session when the profile is not currently authenticated or its login session has expired.</x:v>
       </x:c>
       <x:c r="E7" s="27" t="str">
-        <x:v>Requires IAM Identity Center details such as the SSO start URL and region.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
+        <x:v>Avoids manually creating/storing long-lived IAM access keys.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A8" s="27" t="str">
-        <x:v>aws sso login --profile cloudvault</x:v>
+        <x:v>aws configure list --profile cloudvault</x:v>
       </x:c>
       <x:c r="B8" s="27" t="str">
-        <x:v>Authentication</x:v>
+        <x:v>Configuration / Inspection</x:v>
       </x:c>
       <x:c r="C8" s="27" t="str">
-        <x:v>Authenticates the cloudvault SSO profile and caches temporary credentials.</x:v>
+        <x:v>Shows the effective profile, credential source, and region for the cloudvault profile.</x:v>
       </x:c>
       <x:c r="D8" s="27" t="str">
-        <x:v>Run when beginning a CLI session or when the SSO session has expired.</x:v>
+        <x:v>Use to verify that the profile is using the intended authentication method and region.</x:v>
       </x:c>
       <x:c r="E8" s="27" t="str">
-        <x:v>Usually opens a browser for authentication.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
+        <x:v>Secret values are masked.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A9" s="27" t="str">
-        <x:v>aws sso logout</x:v>
+        <x:v>aws logout --profile cloudvault</x:v>
       </x:c>
       <x:c r="B9" s="27" t="str">
         <x:v>Authentication</x:v>
       </x:c>
       <x:c r="C9" s="27" t="str">
-        <x:v>Removes cached IAM Identity Center login sessions from the local machine.</x:v>
+        <x:v>Signs the cloudvault profile out and removes cached login credentials.</x:v>
       </x:c>
       <x:c r="D9" s="27" t="str">
-        <x:v>Use when you want to explicitly end cached SSO sessions.</x:v>
+        <x:v>Use when you want to explicitly end the local CloudVault CLI session.</x:v>
       </x:c>
       <x:c r="E9" s="27" t="str">
-        <x:v>You will need to log in again before using an SSO profile.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
+        <x:v>Run aws login --profile cloudvault again before issuing authenticated commands.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A10" s="27" t="str">
         <x:v>aws sts get-caller-identity --profile cloudvault</x:v>
       </x:c>
@@ -1245,7 +1255,7 @@
         <x:v>Avoid exposing account identifiers unnecessarily in public screenshots.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
+    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A11" s="27" t="str">
         <x:v>aws sts get-caller-identity --profile cloudvault --query Account --output text</x:v>
       </x:c>
@@ -1262,7 +1272,7 @@
         <x:v>Often assigned to a PowerShell variable such as $AccountId.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
+    <x:row r="12" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A12" s="27" t="str">
         <x:v>aws budgets create-budget --account-id $AccountId --budget file://budget/budget.json --notifications-with-subscribers file://budget/notifications.json --profile cloudvault</x:v>
       </x:c>
@@ -1279,7 +1289,7 @@
         <x:v>The active identity must have AWS Budgets permissions. Verify your notification email configuration.</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
+    <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A13" s="27" t="str">
         <x:v>aws iam create-role --role-name CloudVaultEC2Role --assume-role-policy-document file://iam/assume-role-policy-ec2.json --profile cloudvault</x:v>
       </x:c>
@@ -1296,7 +1306,7 @@
         <x:v>The trust policy controls WHO can assume the role; it does not itself grant S3 or application permissions.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
+    <x:row r="14" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A14" s="27" t="str">
         <x:v>aws iam create-policy --policy-name CloudVaultS3DocumentAccess --policy-document file://iam/policies/cloudvault-s3-document-access.json --profile cloudvault</x:v>
       </x:c>
@@ -1313,7 +1323,7 @@
         <x:v>Review least privilege carefully before creating/attaching the policy.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
+    <x:row r="15" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A15" s="27" t="str">
         <x:v>aws iam attach-role-policy --role-name CloudVaultEC2Role --policy-arn "arn:aws:iam::$AccountId:policy/CloudVaultS3DocumentAccess" --profile cloudvault</x:v>
       </x:c>
@@ -1330,7 +1340,7 @@
         <x:v>Attaching a policy grants the role the permissions defined by that policy.</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
+    <x:row r="16" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A16" s="27" t="str">
         <x:v>aws s3 cp test.pdf s3://YOUR_BUCKET/documents/test.pdf</x:v>
       </x:c>
@@ -1347,7 +1357,7 @@
         <x:v>Replace YOUR_BUCKET. Ensure the current identity has s3:PutObject permission.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
+    <x:row r="17" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A17" s="27" t="str">
         <x:v>aws s3 cp s3://YOUR_BUCKET/documents/test.pdf .</x:v>
       </x:c>
@@ -1364,7 +1374,14 @@
         <x:v>Requires s3:GetObject permission.</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="26"/>
+      <x:c r="B18" s="26"/>
+      <x:c r="C18" s="26"/>
+      <x:c r="D18" s="26"/>
+      <x:c r="E18" s="26"/>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="36" t="str">
         <x:v>Security reminder: prefer temporary credentials for human access, follow least privilege, and never commit AWS credentials or tokens to Git.</x:v>
       </x:c>
@@ -1373,33 +1390,40 @@
       <x:c r="D19" s="36"/>
       <x:c r="E19" s="36"/>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="44" t="str">
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="26"/>
+      <x:c r="B20" s="26"/>
+      <x:c r="C20" s="26"/>
+      <x:c r="D20" s="26"/>
+      <x:c r="E20" s="26"/>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="53" t="str">
         <x:v>Additional AWS CLI Commands — CloudVault Authentication</x:v>
       </x:c>
-      <x:c r="B21" s="44"/>
-      <x:c r="C21" s="44"/>
-      <x:c r="D21" s="44"/>
-      <x:c r="E21" s="44"/>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="49" t="str">
+      <x:c r="B21" s="53"/>
+      <x:c r="C21" s="53"/>
+      <x:c r="D21" s="53"/>
+      <x:c r="E21" s="53"/>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="20" t="str">
         <x:v>Command</x:v>
       </x:c>
-      <x:c r="B22" s="49" t="str">
+      <x:c r="B22" s="20" t="str">
         <x:v>Category</x:v>
       </x:c>
-      <x:c r="C22" s="49" t="str">
+      <x:c r="C22" s="20" t="str">
         <x:v>What it does</x:v>
       </x:c>
-      <x:c r="D22" s="49" t="str">
+      <x:c r="D22" s="20" t="str">
         <x:v>When / Why to use it</x:v>
       </x:c>
-      <x:c r="E22" s="49" t="str">
+      <x:c r="E22" s="20" t="str">
         <x:v>Notes / Cautions</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
+    <x:row r="23" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A23" s="27" t="str">
         <x:v>aws login --profile cloudvault</x:v>
       </x:c>
@@ -1416,7 +1440,7 @@
         <x:v>Avoids manually creating/storing long-lived IAM access keys. The profile should have a region configured.</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
+    <x:row r="24" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A24" s="27" t="str">
         <x:v>aws configure list --profile cloudvault</x:v>
       </x:c>
@@ -1433,7 +1457,7 @@
         <x:v>A TYPE value such as 'login' indicates credentials supplied by aws login. Secret values are masked.</x:v>
       </x:c>
     </x:row>
-    <x:row r="25">
+    <x:row r="25" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A25" s="27" t="str">
         <x:v>aws logout --profile cloudvault</x:v>
       </x:c>
@@ -1450,16 +1474,30 @@
         <x:v>After logout, run aws login --profile cloudvault again before issuing authenticated commands.</x:v>
       </x:c>
     </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="52" t="str">
+    <x:row r="26" ht="15" hidden="0" customHeight="1">
+      <x:c r="A26" s="26"/>
+      <x:c r="B26" s="26"/>
+      <x:c r="C26" s="26"/>
+      <x:c r="D26" s="26"/>
+      <x:c r="E26" s="26"/>
+    </x:row>
+    <x:row r="27" ht="15" hidden="0" customHeight="1">
+      <x:c r="A27" s="36" t="str">
         <x:v>CloudVault validation sequence: aws login --profile cloudvault → aws sts get-caller-identity --profile cloudvault → aws configure list --profile cloudvault</x:v>
       </x:c>
-      <x:c r="B27" s="52"/>
-      <x:c r="C27" s="52"/>
-      <x:c r="D27" s="52"/>
-      <x:c r="E27" s="52"/>
-    </x:row>
-    <x:row r="29">
+      <x:c r="B27" s="36"/>
+      <x:c r="C27" s="36"/>
+      <x:c r="D27" s="36"/>
+      <x:c r="E27" s="36"/>
+    </x:row>
+    <x:row r="28" ht="15" hidden="0" customHeight="1">
+      <x:c r="A28" s="26"/>
+      <x:c r="B28" s="26"/>
+      <x:c r="C28" s="26"/>
+      <x:c r="D28" s="26"/>
+      <x:c r="E28" s="26"/>
+    </x:row>
+    <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="26" t="str">
         <x:v>Additional AWS CLI Commands — IAM Role Validation</x:v>
       </x:c>
@@ -1468,7 +1506,7 @@
       <x:c r="D29" s="26"/>
       <x:c r="E29" s="26"/>
     </x:row>
-    <x:row r="30">
+    <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="26" t="str">
         <x:v>Command</x:v>
       </x:c>
@@ -1502,7 +1540,7 @@
         <x:v>For Phase 0, verify that ec2.amazonaws.com is the trusted service and sts:AssumeRole is the trust action. Avoid publishing account-specific ARN details.</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="32" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A32" s="26" t="str">
         <x:v>aws iam list-attached-role-policies --role-name CloudVaultEC2Role --profile cloudvault</x:v>
       </x:c>
@@ -1516,10 +1554,10 @@
         <x:v>Use to verify whether the role currently receives permissions from managed policies.</x:v>
       </x:c>
       <x:c r="E32" s="26" t="str">
-        <x:v>For Phase 0, AttachedPolicies: [] is expected because the S3 permissions policy is intentionally deferred until the bucket exists.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>At the end of Phase 0, AttachedPolicies: [] was expected. During Phase 1, CloudVaultS3DocumentAccess was intentionally attached after the real S3 bucket existed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A33" s="26" t="str">
         <x:v>aws iam list-role-policies --role-name CloudVaultEC2Role --profile cloudvault</x:v>
       </x:c>
@@ -1536,7 +1574,7 @@
         <x:v>For the completed Phase 0 validation, PolicyNames: [] is the expected result.</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="34" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A34" s="26" t="str">
         <x:v>aws iam list-instance-profiles-for-role --role-name CloudVaultEC2Role --profile cloudvault</x:v>
       </x:c>
@@ -1553,14 +1591,663 @@
         <x:v>For Phase 0, InstanceProfiles: [] is expected. The instance profile will be created later during the EC2 phase.</x:v>
       </x:c>
     </x:row>
-    <x:row r="35">
+    <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="26" t="str">
-        <x:v>Phase 0 IAM validation result: trust policy verified; no managed policies, no inline policies, and no EC2 instance profile yet — all expected.</x:v>
+        <x:v>Phase 0 IAM validation result: EC2 trust verified; no managed policies, no inline policies, and no EC2 instance profile at the Phase 0 checkpoint. Phase 1 later attached the scoped S3 policy.</x:v>
       </x:c>
       <x:c r="B35" s="26"/>
       <x:c r="C35" s="26"/>
       <x:c r="D35" s="26"/>
       <x:c r="E35" s="26"/>
+    </x:row>
+    <x:row r="36" ht="15" hidden="0" customHeight="1">
+      <x:c r="A36" s="26"/>
+      <x:c r="B36" s="26"/>
+      <x:c r="C36" s="26"/>
+      <x:c r="D36" s="26"/>
+      <x:c r="E36" s="26"/>
+    </x:row>
+    <x:row r="37" ht="15" hidden="0" customHeight="1">
+      <x:c r="A37" s="26" t="str">
+        <x:v>Additional AWS CLI Commands — CloudVault Phase 1 S3 &amp; IAM</x:v>
+      </x:c>
+      <x:c r="B37" s="26"/>
+      <x:c r="C37" s="26"/>
+      <x:c r="D37" s="26"/>
+      <x:c r="E37" s="26"/>
+    </x:row>
+    <x:row r="38" ht="15" hidden="0" customHeight="1">
+      <x:c r="A38" s="26" t="str">
+        <x:v>Command</x:v>
+      </x:c>
+      <x:c r="B38" s="26" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="C38" s="26" t="str">
+        <x:v>What it does</x:v>
+      </x:c>
+      <x:c r="D38" s="26" t="str">
+        <x:v>When / Why to use it</x:v>
+      </x:c>
+      <x:c r="E38" s="26" t="str">
+        <x:v>Notes / Cautions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A39" s="26" t="str">
+        <x:v>aws s3api create-bucket --bucket cloudvault-documents-dev01 --region ap-southeast-1 --create-bucket-configuration LocationConstraint=ap-southeast-1 --object-ownership BucketOwnerEnforced --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B39" s="26" t="str">
+        <x:v>S3 / Provisioning</x:v>
+      </x:c>
+      <x:c r="C39" s="26" t="str">
+        <x:v>Creates the CloudVault S3 bucket in Singapore with bucket-owner-enforced object ownership.</x:v>
+      </x:c>
+      <x:c r="D39" s="26" t="str">
+        <x:v>Use once when creating the project document bucket through the CLI.</x:v>
+      </x:c>
+      <x:c r="E39" s="26" t="str">
+        <x:v>S3 bucket names are globally unique. BucketOwnerEnforced disables ACL-based ownership.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A40" s="26" t="str">
+        <x:v>aws s3api head-bucket --bucket cloudvault-documents-dev01 --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B40" s="26" t="str">
+        <x:v>S3 / Validation</x:v>
+      </x:c>
+      <x:c r="C40" s="26" t="str">
+        <x:v>Checks that the bucket exists and returns metadata such as bucket region when authorized.</x:v>
+      </x:c>
+      <x:c r="D40" s="26" t="str">
+        <x:v>Use immediately after bucket creation or when troubleshooting a bucket/region issue.</x:v>
+      </x:c>
+      <x:c r="E40" s="26" t="str">
+        <x:v>The --bucket option is required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="66" hidden="0" customHeight="1">
+      <x:c r="A41" s="26" t="str">
+        <x:v>aws s3api put-public-access-block --bucket cloudvault-documents-dev01 --public-access-block-configuration BlockPublicAcls=true,IgnorePublicAcls=true,BlockPublicPolicy=true,RestrictPublicBuckets=true --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B41" s="26" t="str">
+        <x:v>S3 / Security</x:v>
+      </x:c>
+      <x:c r="C41" s="26" t="str">
+        <x:v>Enables all four S3 Block Public Access controls on the CloudVault bucket.</x:v>
+      </x:c>
+      <x:c r="D41" s="26" t="str">
+        <x:v>Use to explicitly enforce the private-bucket design.</x:v>
+      </x:c>
+      <x:c r="E41" s="26" t="str">
+        <x:v>CloudVault does not require public bucket access.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A42" s="26" t="str">
+        <x:v>aws s3api get-public-access-block --bucket cloudvault-documents-dev01 --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B42" s="26" t="str">
+        <x:v>S3 / Validation</x:v>
+      </x:c>
+      <x:c r="C42" s="26" t="str">
+        <x:v>Retrieves the current Block Public Access configuration.</x:v>
+      </x:c>
+      <x:c r="D42" s="26" t="str">
+        <x:v>Use to verify that all four public-access protections remain enabled.</x:v>
+      </x:c>
+      <x:c r="E42" s="26" t="str">
+        <x:v>Expected values are true for all four controls.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A43" s="26" t="str">
+        <x:v>aws s3api put-bucket-versioning --bucket cloudvault-documents-dev01 --versioning-configuration Status=Enabled --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B43" s="26" t="str">
+        <x:v>S3 / Versioning</x:v>
+      </x:c>
+      <x:c r="C43" s="26" t="str">
+        <x:v>Enables object versioning on the CloudVault document bucket.</x:v>
+      </x:c>
+      <x:c r="D43" s="26" t="str">
+        <x:v>Use so overwrites and normal deletes preserve recoverable historical versions.</x:v>
+      </x:c>
+      <x:c r="E43" s="26" t="str">
+        <x:v>Old versions continue to consume storage until deleted or expired by lifecycle rules.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A44" s="26" t="str">
+        <x:v>aws s3api get-bucket-versioning --bucket cloudvault-documents-dev01 --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B44" s="26" t="str">
+        <x:v>S3 / Validation</x:v>
+      </x:c>
+      <x:c r="C44" s="26" t="str">
+        <x:v>Retrieves the bucket versioning status.</x:v>
+      </x:c>
+      <x:c r="D44" s="26" t="str">
+        <x:v>Use to confirm versioning is enabled before testing object history.</x:v>
+      </x:c>
+      <x:c r="E44" s="26" t="str">
+        <x:v>Expected Status: Enabled.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A45" s="26" t="str">
+        <x:v>aws s3api put-bucket-encryption --bucket cloudvault-documents-dev01 --server-side-encryption-configuration file://s3/config/bucket_encryption.json --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B45" s="26" t="str">
+        <x:v>S3 / Encryption</x:v>
+      </x:c>
+      <x:c r="C45" s="26" t="str">
+        <x:v>Applies the project's default S3 server-side encryption configuration from a JSON file.</x:v>
+      </x:c>
+      <x:c r="D45" s="26" t="str">
+        <x:v>Use to explicitly document and apply SSE-S3 for CloudVault.</x:v>
+      </x:c>
+      <x:c r="E45" s="26" t="str">
+        <x:v>Run from the repository root so the relative file:// path resolves correctly.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A46" s="26" t="str">
+        <x:v>aws s3api get-bucket-encryption --bucket cloudvault-documents-dev01 --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B46" s="26" t="str">
+        <x:v>S3 / Validation</x:v>
+      </x:c>
+      <x:c r="C46" s="26" t="str">
+        <x:v>Returns the bucket's default encryption configuration.</x:v>
+      </x:c>
+      <x:c r="D46" s="26" t="str">
+        <x:v>Use to confirm SSE-S3 is configured.</x:v>
+      </x:c>
+      <x:c r="E46" s="26" t="str">
+        <x:v>AES256 identifies SSE-S3.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A47" s="26" t="str">
+        <x:v>aws s3api put-bucket-tagging --bucket cloudvault-documents-dev01 --tagging file://s3/config/bucket-tags.json --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B47" s="26" t="str">
+        <x:v>S3 / Tagging</x:v>
+      </x:c>
+      <x:c r="C47" s="26" t="str">
+        <x:v>Applies the CloudVault project/environment tags from a local JSON file.</x:v>
+      </x:c>
+      <x:c r="D47" s="26" t="str">
+        <x:v>Use to keep project resources identifiable for organization and future cost tracking.</x:v>
+      </x:c>
+      <x:c r="E47" s="26" t="str">
+        <x:v>Keep examples free of account-specific identifiers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A48" s="26" t="str">
+        <x:v>aws s3api get-bucket-tagging --bucket cloudvault-documents-dev01 --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B48" s="26" t="str">
+        <x:v>S3 / Validation</x:v>
+      </x:c>
+      <x:c r="C48" s="26" t="str">
+        <x:v>Returns tags currently configured on the bucket.</x:v>
+      </x:c>
+      <x:c r="D48" s="26" t="str">
+        <x:v>Use to verify Project=CloudVault and Environment=Learning.</x:v>
+      </x:c>
+      <x:c r="E48" s="26" t="str">
+        <x:v>Useful after updates to confirm the desired tag set.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A49" s="26" t="str">
+        <x:v>aws s3api get-bucket-ownership-controls --bucket cloudvault-documents-dev01 --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B49" s="26" t="str">
+        <x:v>S3 / Security</x:v>
+      </x:c>
+      <x:c r="C49" s="26" t="str">
+        <x:v>Retrieves S3 Object Ownership configuration.</x:v>
+      </x:c>
+      <x:c r="D49" s="26" t="str">
+        <x:v>Use to verify BucketOwnerEnforced remains active.</x:v>
+      </x:c>
+      <x:c r="E49" s="26" t="str">
+        <x:v>With BucketOwnerEnforced, ACLs are disabled.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A50" s="26" t="str">
+        <x:v>aws s3 cp .\test-data\sample.txt s3://cloudvault-documents-dev01/documents/sample.txt --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B50" s="26" t="str">
+        <x:v>S3 / Objects</x:v>
+      </x:c>
+      <x:c r="C50" s="26" t="str">
+        <x:v>Uploads a local test file to the documents/ prefix.</x:v>
+      </x:c>
+      <x:c r="D50" s="26" t="str">
+        <x:v>Use for basic object-write testing.</x:v>
+      </x:c>
+      <x:c r="E50" s="26" t="str">
+        <x:v>The documents/ prefix matches the least-privilege IAM policy scope.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A51" s="26" t="str">
+        <x:v>aws s3 ls s3://cloudvault-documents-dev01 --recursive --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B51" s="26" t="str">
+        <x:v>S3 / Objects</x:v>
+      </x:c>
+      <x:c r="C51" s="26" t="str">
+        <x:v>Lists currently visible objects recursively.</x:v>
+      </x:c>
+      <x:c r="D51" s="26" t="str">
+        <x:v>Use to confirm the current object is present.</x:v>
+      </x:c>
+      <x:c r="E51" s="26" t="str">
+        <x:v>This high-level listing does not show historical versions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A52" s="26" t="str">
+        <x:v>aws s3api head-object --bucket cloudvault-documents-dev01 --key documents/sample.txt --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B52" s="26" t="str">
+        <x:v>S3 / Metadata</x:v>
+      </x:c>
+      <x:c r="C52" s="26" t="str">
+        <x:v>Returns metadata for the current object version.</x:v>
+      </x:c>
+      <x:c r="D52" s="26" t="str">
+        <x:v>Use to inspect content length, VersionId, content type, ETag, and encryption.</x:v>
+      </x:c>
+      <x:c r="E52" s="26" t="str">
+        <x:v>A VersionId confirms versioning is active; AES256 confirms SSE-S3.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A53" s="26" t="str">
+        <x:v>aws s3api list-object-versions --bucket cloudvault-documents-dev01 --prefix documents/sample.txt --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B53" s="26" t="str">
+        <x:v>S3 / Versioning</x:v>
+      </x:c>
+      <x:c r="C53" s="26" t="str">
+        <x:v>Lists data versions and delete markers for the specified key prefix.</x:v>
+      </x:c>
+      <x:c r="D53" s="26" t="str">
+        <x:v>Use to inspect versioning behavior after overwrites or deletes.</x:v>
+      </x:c>
+      <x:c r="E53" s="26" t="str">
+        <x:v>The command name is plural: list-object-versions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A54" s="26" t="str">
+        <x:v>aws s3api get-object --bucket cloudvault-documents-dev01 --key documents/sample.txt --version-id "VERSION_ID" .\test-data\restored-version.txt --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B54" s="26" t="str">
+        <x:v>S3 / Versioning</x:v>
+      </x:c>
+      <x:c r="C54" s="26" t="str">
+        <x:v>Downloads a specific historical object version by VersionId.</x:v>
+      </x:c>
+      <x:c r="D54" s="26" t="str">
+        <x:v>Use for point-in-time inspection or restoration testing.</x:v>
+      </x:c>
+      <x:c r="E54" s="26" t="str">
+        <x:v>Replace VERSION_ID with a real value only during the lab; avoid publishing real version IDs unnecessarily.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A55" s="26" t="str">
+        <x:v>aws s3 rm s3://cloudvault-documents-dev01/documents/sample.txt --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B55" s="26" t="str">
+        <x:v>S3 / Versioning</x:v>
+      </x:c>
+      <x:c r="C55" s="26" t="str">
+        <x:v>Deletes the current key without specifying a version ID.</x:v>
+      </x:c>
+      <x:c r="D55" s="26" t="str">
+        <x:v>Use to demonstrate delete-marker behavior in a versioned bucket.</x:v>
+      </x:c>
+      <x:c r="E55" s="26" t="str">
+        <x:v>A normal delete creates a delete marker rather than permanently deleting historical versions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A56" s="26" t="str">
+        <x:v>aws s3api delete-object --bucket cloudvault-documents-dev01 --key documents/sample.txt --version-id "DELETE_MARKER_VERSION_ID" --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B56" s="26" t="str">
+        <x:v>S3 / Recovery</x:v>
+      </x:c>
+      <x:c r="C56" s="26" t="str">
+        <x:v>Deletes a specific version or delete marker.</x:v>
+      </x:c>
+      <x:c r="D56" s="26" t="str">
+        <x:v>Use in the lab to remove the current delete marker and reveal the previous object version.</x:v>
+      </x:c>
+      <x:c r="E56" s="26" t="str">
+        <x:v>Targeting a data-version ID permanently deletes that historical version if permissions allow it.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A57" s="26" t="str">
+        <x:v>aws accessanalyzer validate-policy --policy-document file://iam/policies/cloudvault-s3-document-access.json --policy-type IDENTITY_POLICY --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B57" s="26" t="str">
+        <x:v>IAM / Validation</x:v>
+      </x:c>
+      <x:c r="C57" s="26" t="str">
+        <x:v>Validates the local IAM identity policy using IAM Access Analyzer.</x:v>
+      </x:c>
+      <x:c r="D57" s="26" t="str">
+        <x:v>Use before creating or updating the managed policy.</x:v>
+      </x:c>
+      <x:c r="E57" s="26" t="str">
+        <x:v>A clean validation returns findings: []. Use file://, not files://.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A58" s="26" t="str">
+        <x:v>aws iam create-policy --policy-name CloudVaultS3DocumentAccess --description "Least-privilege S3 access to the CloudVault documents prefix" --policy-document file://iam/policies/cloudvault-s3-document-access.json --tags Key=Project,Value=CloudVault Key=Environment,Value=Learning --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B58" s="26" t="str">
+        <x:v>IAM</x:v>
+      </x:c>
+      <x:c r="C58" s="26" t="str">
+        <x:v>Creates the customer-managed CloudVault S3 policy from the validated local JSON.</x:v>
+      </x:c>
+      <x:c r="D58" s="26" t="str">
+        <x:v>Use after the real bucket ARN has replaced the Phase 0 placeholder.</x:v>
+      </x:c>
+      <x:c r="E58" s="26" t="str">
+        <x:v>Avoid Resource: * and keep the policy scoped to the CloudVault bucket/documents prefix.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A59" s="26" t="str">
+        <x:v>aws iam get-policy-version --policy-arn $PolicyArn --version-id $DefaultVersionId --query "PolicyVersion.Document" --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B59" s="26" t="str">
+        <x:v>IAM / Validation</x:v>
+      </x:c>
+      <x:c r="C59" s="26" t="str">
+        <x:v>Retrieves the actual JSON document stored for a managed policy version.</x:v>
+      </x:c>
+      <x:c r="D59" s="26" t="str">
+        <x:v>Use to compare the AWS-stored policy with the local source file.</x:v>
+      </x:c>
+      <x:c r="E59" s="26" t="str">
+        <x:v>get-policy returns metadata; get-policy-version returns the policy document.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A60" s="26" t="str">
+        <x:v>aws iam list-entities-for-policy --policy-arn $PolicyArn --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B60" s="26" t="str">
+        <x:v>IAM / Validation</x:v>
+      </x:c>
+      <x:c r="C60" s="26" t="str">
+        <x:v>Lists users, groups, and roles attached to the customer-managed policy.</x:v>
+      </x:c>
+      <x:c r="D60" s="26" t="str">
+        <x:v>Use to confirm the policy is attached only to the intended role.</x:v>
+      </x:c>
+      <x:c r="E60" s="26" t="str">
+        <x:v>PolicyUsers and PolicyGroups should remain empty.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A61" s="26" t="str">
+        <x:v>aws iam simulate-principal-policy --policy-source-arn $RoleArn --action-names s3:GetObject --resource-arns arn:aws:s3:::cloudvault-documents-dev01/documents/sample.txt --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B61" s="26" t="str">
+        <x:v>IAM / Simulation</x:v>
+      </x:c>
+      <x:c r="C61" s="26" t="str">
+        <x:v>Simulates whether the role is allowed to perform a requested action on a resource.</x:v>
+      </x:c>
+      <x:c r="D61" s="26" t="str">
+        <x:v>Use to validate both positive and negative least-privilege cases before runtime EC2 testing.</x:v>
+      </x:c>
+      <x:c r="E61" s="26" t="str">
+        <x:v>Simulation is not a replacement for a later real workload/instance-profile test.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A62" s="26" t="str">
+        <x:v>Phase 1 reminder: validate both allowed and denied actions. Keep public screenshots free of AWS account IDs, account-specific ARNs, role IDs, canonical owner IDs, and object version IDs.</x:v>
+      </x:c>
+      <x:c r="B62" s="26"/>
+      <x:c r="C62" s="26"/>
+      <x:c r="D62" s="26"/>
+      <x:c r="E62" s="26"/>
+    </x:row>
+    <x:row r="63" ht="66" hidden="0" customHeight="1">
+      <x:c r="A63" s="26" t="str">
+        <x:v>aws iam simulate-principal-policy --policy-source-arn $RoleArn --action-names s3:ListBucket --resource-arns arn:aws:s3:::cloudvault-documents-dev01 --context-entries ContextKeyName=s3:prefix,ContextKeyValues=private/,ContextKeyType=string --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B63" s="26" t="str">
+        <x:v>IAM / Simulation</x:v>
+      </x:c>
+      <x:c r="C63" s="26" t="str">
+        <x:v>Simulates listing an unapproved private/ prefix.</x:v>
+      </x:c>
+      <x:c r="D63" s="26" t="str">
+        <x:v>Use to prove the s3:prefix condition rejects unrelated paths.</x:v>
+      </x:c>
+      <x:c r="E63" s="26" t="str">
+        <x:v>Expected: implicitDeny.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A64" s="26" t="str">
+        <x:v>aws iam simulate-principal-policy --policy-source-arn $RoleArn --action-names s3:DeleteObjectVersion --resource-arns arn:aws:s3:::cloudvault-documents-dev01/documents/sample.txt --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B64" s="26" t="str">
+        <x:v>IAM / Simulation</x:v>
+      </x:c>
+      <x:c r="C64" s="26" t="str">
+        <x:v>Simulates permanent deletion of a historical object version.</x:v>
+      </x:c>
+      <x:c r="D64" s="26" t="str">
+        <x:v>Use to prove version deletion is not granted by the current policy.</x:v>
+      </x:c>
+      <x:c r="E64" s="26" t="str">
+        <x:v>Expected: implicitDeny.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="15" hidden="0" customHeight="1">
+      <x:c r="A65" s="26"/>
+      <x:c r="B65" s="26"/>
+      <x:c r="C65" s="26"/>
+      <x:c r="D65" s="26"/>
+      <x:c r="E65" s="26"/>
+    </x:row>
+    <x:row r="66" ht="15" hidden="0" customHeight="1">
+      <x:c r="A66" s="26"/>
+      <x:c r="B66" s="26"/>
+      <x:c r="C66" s="26"/>
+      <x:c r="D66" s="26"/>
+      <x:c r="E66" s="26"/>
+    </x:row>
+    <x:row r="67" ht="15" hidden="0" customHeight="1">
+      <x:c r="A67" s="26"/>
+      <x:c r="B67" s="26"/>
+      <x:c r="C67" s="26"/>
+      <x:c r="D67" s="26"/>
+      <x:c r="E67" s="26"/>
+    </x:row>
+    <x:row r="68" ht="15" hidden="0" customHeight="1">
+      <x:c r="A68" s="26"/>
+      <x:c r="B68" s="26"/>
+      <x:c r="C68" s="26"/>
+      <x:c r="D68" s="26"/>
+      <x:c r="E68" s="26"/>
+    </x:row>
+    <x:row r="69" ht="15" hidden="0" customHeight="1">
+      <x:c r="A69" s="26"/>
+      <x:c r="B69" s="26"/>
+      <x:c r="C69" s="26"/>
+      <x:c r="D69" s="26"/>
+      <x:c r="E69" s="26"/>
+    </x:row>
+    <x:row r="70" ht="15" hidden="0" customHeight="1">
+      <x:c r="A70" s="26"/>
+      <x:c r="B70" s="26"/>
+      <x:c r="C70" s="26"/>
+      <x:c r="D70" s="26"/>
+      <x:c r="E70" s="26"/>
+    </x:row>
+    <x:row r="71" ht="15" hidden="0" customHeight="1">
+      <x:c r="A71" s="26"/>
+      <x:c r="B71" s="26"/>
+      <x:c r="C71" s="26"/>
+      <x:c r="D71" s="26"/>
+      <x:c r="E71" s="26"/>
+    </x:row>
+    <x:row r="72" ht="15" hidden="0" customHeight="1">
+      <x:c r="A72" s="26"/>
+      <x:c r="B72" s="26"/>
+      <x:c r="C72" s="26"/>
+      <x:c r="D72" s="26"/>
+      <x:c r="E72" s="26"/>
+    </x:row>
+    <x:row r="73" ht="15" hidden="0" customHeight="1">
+      <x:c r="A73" s="26"/>
+      <x:c r="B73" s="26"/>
+      <x:c r="C73" s="26"/>
+      <x:c r="D73" s="26"/>
+      <x:c r="E73" s="26"/>
+    </x:row>
+    <x:row r="74" ht="15" hidden="0" customHeight="1">
+      <x:c r="A74" s="26"/>
+      <x:c r="B74" s="26"/>
+      <x:c r="C74" s="26"/>
+      <x:c r="D74" s="26"/>
+      <x:c r="E74" s="26"/>
+    </x:row>
+    <x:row r="75" ht="15" hidden="0" customHeight="1">
+      <x:c r="A75" s="26"/>
+      <x:c r="B75" s="26"/>
+      <x:c r="C75" s="26"/>
+      <x:c r="D75" s="26"/>
+      <x:c r="E75" s="26"/>
+    </x:row>
+    <x:row r="76" ht="15" hidden="0" customHeight="1">
+      <x:c r="A76" s="26"/>
+      <x:c r="B76" s="26"/>
+      <x:c r="C76" s="26"/>
+      <x:c r="D76" s="26"/>
+      <x:c r="E76" s="26"/>
+    </x:row>
+    <x:row r="77" ht="15" hidden="0" customHeight="1">
+      <x:c r="A77" s="26"/>
+      <x:c r="B77" s="26"/>
+      <x:c r="C77" s="26"/>
+      <x:c r="D77" s="26"/>
+      <x:c r="E77" s="26"/>
+    </x:row>
+    <x:row r="78" ht="15" hidden="0" customHeight="1">
+      <x:c r="A78" s="26"/>
+      <x:c r="B78" s="26"/>
+      <x:c r="C78" s="26"/>
+      <x:c r="D78" s="26"/>
+      <x:c r="E78" s="26"/>
+    </x:row>
+    <x:row r="79" ht="15" hidden="0" customHeight="1">
+      <x:c r="A79" s="26"/>
+      <x:c r="B79" s="26"/>
+      <x:c r="C79" s="26"/>
+      <x:c r="D79" s="26"/>
+      <x:c r="E79" s="26"/>
+    </x:row>
+    <x:row r="80" ht="15" hidden="0" customHeight="1">
+      <x:c r="A80" s="26"/>
+      <x:c r="B80" s="26"/>
+      <x:c r="C80" s="26"/>
+      <x:c r="D80" s="26"/>
+      <x:c r="E80" s="26"/>
+    </x:row>
+    <x:row r="81" ht="15" hidden="0" customHeight="1">
+      <x:c r="A81" s="26"/>
+      <x:c r="B81" s="26"/>
+      <x:c r="C81" s="26"/>
+      <x:c r="D81" s="26"/>
+      <x:c r="E81" s="26"/>
+    </x:row>
+    <x:row r="82" ht="15" hidden="0" customHeight="1">
+      <x:c r="A82" s="26"/>
+      <x:c r="B82" s="26"/>
+      <x:c r="C82" s="26"/>
+      <x:c r="D82" s="26"/>
+      <x:c r="E82" s="26"/>
+    </x:row>
+    <x:row r="83" ht="15" hidden="0" customHeight="1">
+      <x:c r="A83" s="26"/>
+      <x:c r="B83" s="26"/>
+      <x:c r="C83" s="26"/>
+      <x:c r="D83" s="26"/>
+      <x:c r="E83" s="26"/>
+    </x:row>
+    <x:row r="84" ht="15" hidden="0" customHeight="1">
+      <x:c r="A84" s="26"/>
+      <x:c r="B84" s="26"/>
+      <x:c r="C84" s="26"/>
+      <x:c r="D84" s="26"/>
+      <x:c r="E84" s="26"/>
+    </x:row>
+    <x:row r="85" ht="15" hidden="0" customHeight="1">
+      <x:c r="A85" s="26"/>
+      <x:c r="B85" s="26"/>
+      <x:c r="C85" s="26"/>
+      <x:c r="D85" s="26"/>
+      <x:c r="E85" s="26"/>
+    </x:row>
+    <x:row r="86" ht="15" hidden="0" customHeight="1">
+      <x:c r="A86" s="26"/>
+      <x:c r="B86" s="26"/>
+      <x:c r="C86" s="26"/>
+      <x:c r="D86" s="26"/>
+      <x:c r="E86" s="26"/>
+    </x:row>
+    <x:row r="87" ht="15" hidden="0" customHeight="1">
+      <x:c r="A87" s="26"/>
+      <x:c r="B87" s="26"/>
+      <x:c r="C87" s="26"/>
+      <x:c r="D87" s="26"/>
+      <x:c r="E87" s="26"/>
+    </x:row>
+    <x:row r="88" ht="15" hidden="0" customHeight="1">
+      <x:c r="A88" s="26"/>
+      <x:c r="B88" s="26"/>
+      <x:c r="C88" s="26"/>
+      <x:c r="D88" s="26"/>
+      <x:c r="E88" s="26"/>
+    </x:row>
+    <x:row r="89" ht="15" hidden="0" customHeight="1">
+      <x:c r="A89" s="26"/>
+      <x:c r="B89" s="26"/>
+      <x:c r="C89" s="26"/>
+      <x:c r="D89" s="26"/>
+      <x:c r="E89" s="26"/>
+    </x:row>
+    <x:row r="90" ht="15" hidden="0" customHeight="1">
+      <x:c r="A90" s="26"/>
+      <x:c r="B90" s="26"/>
+      <x:c r="C90" s="26"/>
+      <x:c r="D90" s="26"/>
+      <x:c r="E90" s="26"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1574,7 +2261,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d68998e50294f2f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26d6e1466150435f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1583,14 +2270,14 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="44" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="48" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="38" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="40" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="44" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="38" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="28" customHeight="1">
+    <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
       <x:c r="A1" s="40" t="str">
         <x:v>PowerShell Command Reference</x:v>
       </x:c>
@@ -1599,7 +2286,7 @@
       <x:c r="D1" s="40"/>
       <x:c r="E1" s="40"/>
     </x:row>
-    <x:row r="2" ht="42" customHeight="1">
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="12" t="str">
         <x:v>PowerShell and Windows shell commands used while installing/troubleshooting AWS CLI and Git and managing the CloudVault project.</x:v>
       </x:c>
@@ -1608,7 +2295,14 @@
       <x:c r="D2" s="12"/>
       <x:c r="E2" s="12"/>
     </x:row>
-    <x:row r="4">
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="26"/>
+      <x:c r="B3" s="26"/>
+      <x:c r="C3" s="26"/>
+      <x:c r="D3" s="26"/>
+      <x:c r="E3" s="26"/>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="20" t="str">
         <x:v>Command</x:v>
       </x:c>
@@ -1625,7 +2319,7 @@
         <x:v>Notes / Cautions</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
+    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A5" s="27" t="str">
         <x:v>$env:PATH</x:v>
       </x:c>
@@ -1642,7 +2336,7 @@
         <x:v>In PowerShell, environment variables use the $env:NAME syntax.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A6" s="27" t="str">
         <x:v>$env:PATH -split ';'</x:v>
       </x:c>
@@ -1659,7 +2353,7 @@
         <x:v>Useful for AWS CLI/Git PATH troubleshooting.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
+    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A7" s="27" t="str">
         <x:v>echo $PATH</x:v>
       </x:c>
@@ -1676,7 +2370,7 @@
         <x:v>For Windows PATH in PowerShell, use $env:PATH instead.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
+    <x:row r="8" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A8" s="27" t="str">
         <x:v>Test-Path "C:\Users\YourUser\AppData\Local\Programs\Amazon\AWSCLIV2\aws.exe"</x:v>
       </x:c>
@@ -1693,7 +2387,7 @@
         <x:v>Does not run the executable.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
+    <x:row r="9" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A9" s="27" t="str">
         <x:v>&amp; "C:\Users\YourUser\AppData\Local\Programs\Amazon\AWSCLIV2\aws.exe" --version</x:v>
       </x:c>
@@ -1710,7 +2404,7 @@
         <x:v>If this works but aws --version does not, PATH is the likely issue.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
+    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A10" s="27" t="str">
         <x:v>[Environment]::GetEnvironmentVariable("Path", "User") -split ';'</x:v>
       </x:c>
@@ -1727,7 +2421,7 @@
         <x:v>Different from the current process PATH, which may be stale until PowerShell is reopened.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
+    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A11" s="27" t="str">
         <x:v>Get-Command aws -ErrorAction SilentlyContinue</x:v>
       </x:c>
@@ -1744,7 +2438,7 @@
         <x:v>An empty result generally means it is not available through the current command-resolution path.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
+    <x:row r="12" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A12" s="27" t="str">
         <x:v>$env:PATH += ";C:\Users\YourUser\AppData\Local\Programs\Amazon\AWSCLIV2"</x:v>
       </x:c>
@@ -1761,7 +2455,7 @@
         <x:v>This does not permanently update Windows PATH.</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
+    <x:row r="13" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A13" s="27" t="str">
         <x:v>where.exe git</x:v>
       </x:c>
@@ -1778,7 +2472,7 @@
         <x:v>No output usually means Git is not currently resolvable through PATH.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
+    <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A14" s="27" t="str">
         <x:v>Get-Command git -ErrorAction SilentlyContinue</x:v>
       </x:c>
@@ -1795,7 +2489,7 @@
         <x:v>If empty, Git may be missing or PATH may not be refreshed.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
+    <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A15" s="27" t="str">
         <x:v>winget install --id Git.Git -e --source winget</x:v>
       </x:c>
@@ -1812,7 +2506,7 @@
         <x:v>Close and reopen PowerShell after installation so PATH changes are picked up.</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
+    <x:row r="16" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A16" s="27" t="str">
         <x:v>cd C:\Projects\aws-cloudvault</x:v>
       </x:c>
@@ -1829,7 +2523,7 @@
         <x:v>cd is an alias for Set-Location in PowerShell.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
+    <x:row r="17" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A17" s="27" t="str">
         <x:v>Get-ChildItem</x:v>
       </x:c>
@@ -1846,7 +2540,7 @@
         <x:v>Aliases include dir and ls.</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
+    <x:row r="18" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A18" s="27" t="str">
         <x:v>mkdir backend</x:v>
       </x:c>
@@ -1863,7 +2557,7 @@
         <x:v>mkdir is an alias for New-Item -ItemType Directory.</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
+    <x:row r="19" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A19" s="27" t="str">
         <x:v>mkdir frontend</x:v>
       </x:c>
@@ -1880,7 +2574,7 @@
         <x:v>Git will not track it while it is empty.</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
+    <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A20" s="27" t="str">
         <x:v>mkdir infrastructure</x:v>
       </x:c>
@@ -1897,7 +2591,7 @@
         <x:v>Git will not track it while it is empty.</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
+    <x:row r="21" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A21" s="27" t="str">
         <x:v>New-Item backend\.gitkeep -ItemType File</x:v>
       </x:c>
@@ -1914,7 +2608,7 @@
         <x:v>.gitkeep is a convention, not a special Git feature.</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
+    <x:row r="22" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A22" s="27" t="str">
         <x:v>New-Item frontend\.gitkeep -ItemType File</x:v>
       </x:c>
@@ -1931,7 +2625,7 @@
         <x:v>.gitkeep is only a naming convention.</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
+    <x:row r="23" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A23" s="27" t="str">
         <x:v>New-Item infrastructure\.gitkeep -ItemType File</x:v>
       </x:c>
@@ -1948,7 +2642,7 @@
         <x:v>.gitkeep is only a naming convention.</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
+    <x:row r="24" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A24" s="27" t="str">
         <x:v>Get-Content .gitignore</x:v>
       </x:c>
@@ -1965,7 +2659,7 @@
         <x:v>Important for checking that secrets, .env files, keys, and local AWS files are excluded.</x:v>
       </x:c>
     </x:row>
-    <x:row r="25">
+    <x:row r="25" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A25" s="27" t="str">
         <x:v>$AccountId = aws sts get-caller-identity --profile cloudvault --query Account --output text</x:v>
       </x:c>
@@ -1982,7 +2676,14 @@
         <x:v>The variable exists only for the current PowerShell session unless persisted elsewhere.</x:v>
       </x:c>
     </x:row>
-    <x:row r="27">
+    <x:row r="26" ht="15" hidden="0" customHeight="1">
+      <x:c r="A26" s="26"/>
+      <x:c r="B26" s="26"/>
+      <x:c r="C26" s="26"/>
+      <x:c r="D26" s="26"/>
+      <x:c r="E26" s="26"/>
+    </x:row>
+    <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="36" t="str">
         <x:v>PowerShell tip: after an installer changes PATH, close and reopen PowerShell/Windows Terminal before assuming the installation failed.</x:v>
       </x:c>
@@ -1991,33 +2692,40 @@
       <x:c r="D27" s="36"/>
       <x:c r="E27" s="36"/>
     </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="44" t="str">
+    <x:row r="28" ht="15" hidden="0" customHeight="1">
+      <x:c r="A28" s="26"/>
+      <x:c r="B28" s="26"/>
+      <x:c r="C28" s="26"/>
+      <x:c r="D28" s="26"/>
+      <x:c r="E28" s="26"/>
+    </x:row>
+    <x:row r="29" ht="15" hidden="0" customHeight="1">
+      <x:c r="A29" s="53" t="str">
         <x:v>Additional PowerShell Commands — AWS CLI Inspection</x:v>
       </x:c>
-      <x:c r="B29" s="44"/>
-      <x:c r="C29" s="44"/>
-      <x:c r="D29" s="44"/>
-      <x:c r="E29" s="44"/>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="49" t="str">
+      <x:c r="B29" s="53"/>
+      <x:c r="C29" s="53"/>
+      <x:c r="D29" s="53"/>
+      <x:c r="E29" s="53"/>
+    </x:row>
+    <x:row r="30" ht="15" hidden="0" customHeight="1">
+      <x:c r="A30" s="20" t="str">
         <x:v>Command</x:v>
       </x:c>
-      <x:c r="B30" s="49" t="str">
+      <x:c r="B30" s="20" t="str">
         <x:v>Category</x:v>
       </x:c>
-      <x:c r="C30" s="49" t="str">
+      <x:c r="C30" s="20" t="str">
         <x:v>What it does</x:v>
       </x:c>
-      <x:c r="D30" s="49" t="str">
+      <x:c r="D30" s="20" t="str">
         <x:v>When / Why to use it</x:v>
       </x:c>
-      <x:c r="E30" s="49" t="str">
+      <x:c r="E30" s="20" t="str">
         <x:v>Notes / Cautions</x:v>
       </x:c>
     </x:row>
-    <x:row r="31">
+    <x:row r="31" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A31" s="27" t="str">
         <x:v>Get-Content $HOME\.aws\config</x:v>
       </x:c>
@@ -2034,7 +2742,7 @@
         <x:v>Review contents before sharing screenshots publicly. Do not expose credential files or secrets.</x:v>
       </x:c>
     </x:row>
-    <x:row r="32">
+    <x:row r="32" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A32" s="27" t="str">
         <x:v>cd C:\Users\YourUser\.aws</x:v>
       </x:c>
@@ -2050,6 +2758,486 @@
       <x:c r="E32" s="27" t="str">
         <x:v>For normal CloudVault Git work, return to the project repository directory before running Git commands.</x:v>
       </x:c>
+    </x:row>
+    <x:row r="33" ht="15" hidden="0" customHeight="1">
+      <x:c r="A33" s="26"/>
+      <x:c r="B33" s="26"/>
+      <x:c r="C33" s="26"/>
+      <x:c r="D33" s="26"/>
+      <x:c r="E33" s="26"/>
+    </x:row>
+    <x:row r="34" ht="15" hidden="0" customHeight="1">
+      <x:c r="A34" s="26"/>
+      <x:c r="B34" s="26"/>
+      <x:c r="C34" s="26"/>
+      <x:c r="D34" s="26"/>
+      <x:c r="E34" s="26"/>
+    </x:row>
+    <x:row r="35" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A35" s="26" t="str">
+        <x:v>Additional PowerShell Commands — CloudVault Phase 1 Validation</x:v>
+      </x:c>
+      <x:c r="B35" s="26"/>
+      <x:c r="C35" s="26"/>
+      <x:c r="D35" s="26"/>
+      <x:c r="E35" s="26"/>
+    </x:row>
+    <x:row r="36" ht="15" hidden="0" customHeight="1">
+      <x:c r="A36" s="26" t="str">
+        <x:v>Command</x:v>
+      </x:c>
+      <x:c r="B36" s="26" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="C36" s="26" t="str">
+        <x:v>What it does</x:v>
+      </x:c>
+      <x:c r="D36" s="26" t="str">
+        <x:v>When / Why to use it</x:v>
+      </x:c>
+      <x:c r="E36" s="26" t="str">
+        <x:v>Notes / Cautions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A37" s="26" t="str">
+        <x:v>Get-Content .\iam\policies\cloudvault-s3-document-access.json -Raw | ConvertFrom-Json | Out-Null</x:v>
+      </x:c>
+      <x:c r="B37" s="26" t="str">
+        <x:v>JSON Validation</x:v>
+      </x:c>
+      <x:c r="C37" s="26" t="str">
+        <x:v>Parses the IAM policy JSON and discards the parsed object when valid.</x:v>
+      </x:c>
+      <x:c r="D37" s="26" t="str">
+        <x:v>Use before sending a local JSON policy to AWS.</x:v>
+      </x:c>
+      <x:c r="E37" s="26" t="str">
+        <x:v>No output means parsing succeeded; syntax errors are thrown if the JSON is invalid.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A38" s="26" t="str">
+        <x:v>try { Get-Content .\iam\policies\cloudvault-s3-document-access.json -Raw | ConvertFrom-Json | Out-Null; Write-Host "Policy JSON is valid." } catch { Write-Host "Policy JSON is invalid."; Write-Host $_ }</x:v>
+      </x:c>
+      <x:c r="B38" s="26" t="str">
+        <x:v>JSON Validation</x:v>
+      </x:c>
+      <x:c r="C38" s="26" t="str">
+        <x:v>Validates the policy JSON and prints an explicit success/failure message.</x:v>
+      </x:c>
+      <x:c r="D38" s="26" t="str">
+        <x:v>Use when you want a readable validation result during a manual lab.</x:v>
+      </x:c>
+      <x:c r="E38" s="26" t="str">
+        <x:v>Separate multiple PowerShell statements on one line with semicolons.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A39" s="26" t="str">
+        <x:v>Select-String -Path .\iam\policies\cloudvault-s3-document-access.json -Pattern '"Resource"\s*:\s*"\*"'</x:v>
+      </x:c>
+      <x:c r="B39" s="26" t="str">
+        <x:v>File Inspection / IAM</x:v>
+      </x:c>
+      <x:c r="C39" s="26" t="str">
+        <x:v>Searches the policy file for an unrestricted Resource: * statement.</x:v>
+      </x:c>
+      <x:c r="D39" s="26" t="str">
+        <x:v>Use as an additional least-privilege check before creating the managed policy.</x:v>
+      </x:c>
+      <x:c r="E39" s="26" t="str">
+        <x:v>No output is the desired result for the CloudVault S3 policy.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A40" s="26" t="str">
+        <x:v>$PolicyArn = aws iam list-policies --scope Local --query "Policies[?PolicyName==\'CloudVaultS3DocumentAccess\'].Arn | [0]" --output text --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B40" s="26" t="str">
+        <x:v>Variables / AWS</x:v>
+      </x:c>
+      <x:c r="C40" s="26" t="str">
+        <x:v>Stores the CloudVault managed-policy ARN in a PowerShell variable.</x:v>
+      </x:c>
+      <x:c r="D40" s="26" t="str">
+        <x:v>Use to avoid repeatedly copying an account-specific ARN into later commands.</x:v>
+      </x:c>
+      <x:c r="E40" s="26" t="str">
+        <x:v>The variable lasts only for the current PowerShell session.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A41" s="26" t="str">
+        <x:v>$DefaultVersionId = aws iam get-policy --policy-arn $PolicyArn --query "Policy.DefaultVersionId" --output text --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B41" s="26" t="str">
+        <x:v>Variables / AWS</x:v>
+      </x:c>
+      <x:c r="C41" s="26" t="str">
+        <x:v>Stores the managed policy's current default version ID.</x:v>
+      </x:c>
+      <x:c r="D41" s="26" t="str">
+        <x:v>Use before retrieving the policy document with get-policy-version.</x:v>
+      </x:c>
+      <x:c r="E41" s="26" t="str">
+        <x:v>A newly created managed policy usually starts at v1.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A42" s="26" t="str">
+        <x:v>$RoleArn = aws iam get-role --role-name CloudVaultEC2Role --query "Role.Arn" --output text --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B42" s="26" t="str">
+        <x:v>Variables / AWS</x:v>
+      </x:c>
+      <x:c r="C42" s="26" t="str">
+        <x:v>Stores the CloudVault EC2 role ARN in a PowerShell variable.</x:v>
+      </x:c>
+      <x:c r="D42" s="26" t="str">
+        <x:v>Use with IAM policy simulation commands.</x:v>
+      </x:c>
+      <x:c r="E42" s="26" t="str">
+        <x:v>Avoid publishing the account-specific ARN in screenshots.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A43" s="26" t="str">
+        <x:v>PowerShell lab note: run CloudVault commands from the repository root so relative file:// paths such as file://s3/config/bucket_encryption.json resolve correctly.</x:v>
+      </x:c>
+      <x:c r="B43" s="26"/>
+      <x:c r="C43" s="26"/>
+      <x:c r="D43" s="26"/>
+      <x:c r="E43" s="26"/>
+    </x:row>
+    <x:row r="44" ht="15" hidden="0" customHeight="1">
+      <x:c r="A44" s="26"/>
+      <x:c r="B44" s="26"/>
+      <x:c r="C44" s="26"/>
+      <x:c r="D44" s="26"/>
+      <x:c r="E44" s="26"/>
+    </x:row>
+    <x:row r="45" ht="15" hidden="0" customHeight="1">
+      <x:c r="A45" s="26"/>
+      <x:c r="B45" s="26"/>
+      <x:c r="C45" s="26"/>
+      <x:c r="D45" s="26"/>
+      <x:c r="E45" s="26"/>
+    </x:row>
+    <x:row r="46" ht="15" hidden="0" customHeight="1">
+      <x:c r="A46" s="26"/>
+      <x:c r="B46" s="26"/>
+      <x:c r="C46" s="26"/>
+      <x:c r="D46" s="26"/>
+      <x:c r="E46" s="26"/>
+    </x:row>
+    <x:row r="47" ht="15" hidden="0" customHeight="1">
+      <x:c r="A47" s="26"/>
+      <x:c r="B47" s="26"/>
+      <x:c r="C47" s="26"/>
+      <x:c r="D47" s="26"/>
+      <x:c r="E47" s="26"/>
+    </x:row>
+    <x:row r="48" ht="15" hidden="0" customHeight="1">
+      <x:c r="A48" s="26"/>
+      <x:c r="B48" s="26"/>
+      <x:c r="C48" s="26"/>
+      <x:c r="D48" s="26"/>
+      <x:c r="E48" s="26"/>
+    </x:row>
+    <x:row r="49" ht="15" hidden="0" customHeight="1">
+      <x:c r="A49" s="26"/>
+      <x:c r="B49" s="26"/>
+      <x:c r="C49" s="26"/>
+      <x:c r="D49" s="26"/>
+      <x:c r="E49" s="26"/>
+    </x:row>
+    <x:row r="50" ht="15" hidden="0" customHeight="1">
+      <x:c r="A50" s="26"/>
+      <x:c r="B50" s="26"/>
+      <x:c r="C50" s="26"/>
+      <x:c r="D50" s="26"/>
+      <x:c r="E50" s="26"/>
+    </x:row>
+    <x:row r="51" ht="15" hidden="0" customHeight="1">
+      <x:c r="A51" s="26"/>
+      <x:c r="B51" s="26"/>
+      <x:c r="C51" s="26"/>
+      <x:c r="D51" s="26"/>
+      <x:c r="E51" s="26"/>
+    </x:row>
+    <x:row r="52" ht="15" hidden="0" customHeight="1">
+      <x:c r="A52" s="26"/>
+      <x:c r="B52" s="26"/>
+      <x:c r="C52" s="26"/>
+      <x:c r="D52" s="26"/>
+      <x:c r="E52" s="26"/>
+    </x:row>
+    <x:row r="53" ht="15" hidden="0" customHeight="1">
+      <x:c r="A53" s="26"/>
+      <x:c r="B53" s="26"/>
+      <x:c r="C53" s="26"/>
+      <x:c r="D53" s="26"/>
+      <x:c r="E53" s="26"/>
+    </x:row>
+    <x:row r="54" ht="15" hidden="0" customHeight="1">
+      <x:c r="A54" s="26"/>
+      <x:c r="B54" s="26"/>
+      <x:c r="C54" s="26"/>
+      <x:c r="D54" s="26"/>
+      <x:c r="E54" s="26"/>
+    </x:row>
+    <x:row r="55" ht="15" hidden="0" customHeight="1">
+      <x:c r="A55" s="26"/>
+      <x:c r="B55" s="26"/>
+      <x:c r="C55" s="26"/>
+      <x:c r="D55" s="26"/>
+      <x:c r="E55" s="26"/>
+    </x:row>
+    <x:row r="56" ht="15" hidden="0" customHeight="1">
+      <x:c r="A56" s="26"/>
+      <x:c r="B56" s="26"/>
+      <x:c r="C56" s="26"/>
+      <x:c r="D56" s="26"/>
+      <x:c r="E56" s="26"/>
+    </x:row>
+    <x:row r="57" ht="15" hidden="0" customHeight="1">
+      <x:c r="A57" s="26"/>
+      <x:c r="B57" s="26"/>
+      <x:c r="C57" s="26"/>
+      <x:c r="D57" s="26"/>
+      <x:c r="E57" s="26"/>
+    </x:row>
+    <x:row r="58" ht="15" hidden="0" customHeight="1">
+      <x:c r="A58" s="26"/>
+      <x:c r="B58" s="26"/>
+      <x:c r="C58" s="26"/>
+      <x:c r="D58" s="26"/>
+      <x:c r="E58" s="26"/>
+    </x:row>
+    <x:row r="59" ht="15" hidden="0" customHeight="1">
+      <x:c r="A59" s="26"/>
+      <x:c r="B59" s="26"/>
+      <x:c r="C59" s="26"/>
+      <x:c r="D59" s="26"/>
+      <x:c r="E59" s="26"/>
+    </x:row>
+    <x:row r="60" ht="15" hidden="0" customHeight="1">
+      <x:c r="A60" s="26"/>
+      <x:c r="B60" s="26"/>
+      <x:c r="C60" s="26"/>
+      <x:c r="D60" s="26"/>
+      <x:c r="E60" s="26"/>
+    </x:row>
+    <x:row r="61" ht="15" hidden="0" customHeight="1">
+      <x:c r="A61" s="26"/>
+      <x:c r="B61" s="26"/>
+      <x:c r="C61" s="26"/>
+      <x:c r="D61" s="26"/>
+      <x:c r="E61" s="26"/>
+    </x:row>
+    <x:row r="62" ht="15" hidden="0" customHeight="1">
+      <x:c r="A62" s="26"/>
+      <x:c r="B62" s="26"/>
+      <x:c r="C62" s="26"/>
+      <x:c r="D62" s="26"/>
+      <x:c r="E62" s="26"/>
+    </x:row>
+    <x:row r="63" ht="15" hidden="0" customHeight="1">
+      <x:c r="A63" s="26"/>
+      <x:c r="B63" s="26"/>
+      <x:c r="C63" s="26"/>
+      <x:c r="D63" s="26"/>
+      <x:c r="E63" s="26"/>
+    </x:row>
+    <x:row r="64" ht="15" hidden="0" customHeight="1">
+      <x:c r="A64" s="26"/>
+      <x:c r="B64" s="26"/>
+      <x:c r="C64" s="26"/>
+      <x:c r="D64" s="26"/>
+      <x:c r="E64" s="26"/>
+    </x:row>
+    <x:row r="65" ht="15" hidden="0" customHeight="1">
+      <x:c r="A65" s="26"/>
+      <x:c r="B65" s="26"/>
+      <x:c r="C65" s="26"/>
+      <x:c r="D65" s="26"/>
+      <x:c r="E65" s="26"/>
+    </x:row>
+    <x:row r="66" ht="15" hidden="0" customHeight="1">
+      <x:c r="A66" s="26"/>
+      <x:c r="B66" s="26"/>
+      <x:c r="C66" s="26"/>
+      <x:c r="D66" s="26"/>
+      <x:c r="E66" s="26"/>
+    </x:row>
+    <x:row r="67" ht="15" hidden="0" customHeight="1">
+      <x:c r="A67" s="26"/>
+      <x:c r="B67" s="26"/>
+      <x:c r="C67" s="26"/>
+      <x:c r="D67" s="26"/>
+      <x:c r="E67" s="26"/>
+    </x:row>
+    <x:row r="68" ht="15" hidden="0" customHeight="1">
+      <x:c r="A68" s="26"/>
+      <x:c r="B68" s="26"/>
+      <x:c r="C68" s="26"/>
+      <x:c r="D68" s="26"/>
+      <x:c r="E68" s="26"/>
+    </x:row>
+    <x:row r="69" ht="15" hidden="0" customHeight="1">
+      <x:c r="A69" s="26"/>
+      <x:c r="B69" s="26"/>
+      <x:c r="C69" s="26"/>
+      <x:c r="D69" s="26"/>
+      <x:c r="E69" s="26"/>
+    </x:row>
+    <x:row r="70" ht="15" hidden="0" customHeight="1">
+      <x:c r="A70" s="26"/>
+      <x:c r="B70" s="26"/>
+      <x:c r="C70" s="26"/>
+      <x:c r="D70" s="26"/>
+      <x:c r="E70" s="26"/>
+    </x:row>
+    <x:row r="71" ht="15" hidden="0" customHeight="1">
+      <x:c r="A71" s="26"/>
+      <x:c r="B71" s="26"/>
+      <x:c r="C71" s="26"/>
+      <x:c r="D71" s="26"/>
+      <x:c r="E71" s="26"/>
+    </x:row>
+    <x:row r="72" ht="15" hidden="0" customHeight="1">
+      <x:c r="A72" s="26"/>
+      <x:c r="B72" s="26"/>
+      <x:c r="C72" s="26"/>
+      <x:c r="D72" s="26"/>
+      <x:c r="E72" s="26"/>
+    </x:row>
+    <x:row r="73" ht="15" hidden="0" customHeight="1">
+      <x:c r="A73" s="26"/>
+      <x:c r="B73" s="26"/>
+      <x:c r="C73" s="26"/>
+      <x:c r="D73" s="26"/>
+      <x:c r="E73" s="26"/>
+    </x:row>
+    <x:row r="74" ht="15" hidden="0" customHeight="1">
+      <x:c r="A74" s="26"/>
+      <x:c r="B74" s="26"/>
+      <x:c r="C74" s="26"/>
+      <x:c r="D74" s="26"/>
+      <x:c r="E74" s="26"/>
+    </x:row>
+    <x:row r="75" ht="15" hidden="0" customHeight="1">
+      <x:c r="A75" s="26"/>
+      <x:c r="B75" s="26"/>
+      <x:c r="C75" s="26"/>
+      <x:c r="D75" s="26"/>
+      <x:c r="E75" s="26"/>
+    </x:row>
+    <x:row r="76" ht="15" hidden="0" customHeight="1">
+      <x:c r="A76" s="26"/>
+      <x:c r="B76" s="26"/>
+      <x:c r="C76" s="26"/>
+      <x:c r="D76" s="26"/>
+      <x:c r="E76" s="26"/>
+    </x:row>
+    <x:row r="77" ht="15" hidden="0" customHeight="1">
+      <x:c r="A77" s="26"/>
+      <x:c r="B77" s="26"/>
+      <x:c r="C77" s="26"/>
+      <x:c r="D77" s="26"/>
+      <x:c r="E77" s="26"/>
+    </x:row>
+    <x:row r="78" ht="15" hidden="0" customHeight="1">
+      <x:c r="A78" s="26"/>
+      <x:c r="B78" s="26"/>
+      <x:c r="C78" s="26"/>
+      <x:c r="D78" s="26"/>
+      <x:c r="E78" s="26"/>
+    </x:row>
+    <x:row r="79" ht="15" hidden="0" customHeight="1">
+      <x:c r="A79" s="26"/>
+      <x:c r="B79" s="26"/>
+      <x:c r="C79" s="26"/>
+      <x:c r="D79" s="26"/>
+      <x:c r="E79" s="26"/>
+    </x:row>
+    <x:row r="80" ht="15" hidden="0" customHeight="1">
+      <x:c r="A80" s="26"/>
+      <x:c r="B80" s="26"/>
+      <x:c r="C80" s="26"/>
+      <x:c r="D80" s="26"/>
+      <x:c r="E80" s="26"/>
+    </x:row>
+    <x:row r="81" ht="15" hidden="0" customHeight="1">
+      <x:c r="A81" s="26"/>
+      <x:c r="B81" s="26"/>
+      <x:c r="C81" s="26"/>
+      <x:c r="D81" s="26"/>
+      <x:c r="E81" s="26"/>
+    </x:row>
+    <x:row r="82" ht="15" hidden="0" customHeight="1">
+      <x:c r="A82" s="26"/>
+      <x:c r="B82" s="26"/>
+      <x:c r="C82" s="26"/>
+      <x:c r="D82" s="26"/>
+      <x:c r="E82" s="26"/>
+    </x:row>
+    <x:row r="83" ht="15" hidden="0" customHeight="1">
+      <x:c r="A83" s="26"/>
+      <x:c r="B83" s="26"/>
+      <x:c r="C83" s="26"/>
+      <x:c r="D83" s="26"/>
+      <x:c r="E83" s="26"/>
+    </x:row>
+    <x:row r="84" ht="15" hidden="0" customHeight="1">
+      <x:c r="A84" s="26"/>
+      <x:c r="B84" s="26"/>
+      <x:c r="C84" s="26"/>
+      <x:c r="D84" s="26"/>
+      <x:c r="E84" s="26"/>
+    </x:row>
+    <x:row r="85" ht="15" hidden="0" customHeight="1">
+      <x:c r="A85" s="26"/>
+      <x:c r="B85" s="26"/>
+      <x:c r="C85" s="26"/>
+      <x:c r="D85" s="26"/>
+      <x:c r="E85" s="26"/>
+    </x:row>
+    <x:row r="86" ht="15" hidden="0" customHeight="1">
+      <x:c r="A86" s="26"/>
+      <x:c r="B86" s="26"/>
+      <x:c r="C86" s="26"/>
+      <x:c r="D86" s="26"/>
+      <x:c r="E86" s="26"/>
+    </x:row>
+    <x:row r="87" ht="15" hidden="0" customHeight="1">
+      <x:c r="A87" s="26"/>
+      <x:c r="B87" s="26"/>
+      <x:c r="C87" s="26"/>
+      <x:c r="D87" s="26"/>
+      <x:c r="E87" s="26"/>
+    </x:row>
+    <x:row r="88" ht="15" hidden="0" customHeight="1">
+      <x:c r="A88" s="26"/>
+      <x:c r="B88" s="26"/>
+      <x:c r="C88" s="26"/>
+      <x:c r="D88" s="26"/>
+      <x:c r="E88" s="26"/>
+    </x:row>
+    <x:row r="89" ht="15" hidden="0" customHeight="1">
+      <x:c r="A89" s="26"/>
+      <x:c r="B89" s="26"/>
+      <x:c r="C89" s="26"/>
+      <x:c r="D89" s="26"/>
+      <x:c r="E89" s="26"/>
+    </x:row>
+    <x:row r="90" ht="15" hidden="0" customHeight="1">
+      <x:c r="A90" s="26"/>
+      <x:c r="B90" s="26"/>
+      <x:c r="C90" s="26"/>
+      <x:c r="D90" s="26"/>
+      <x:c r="E90" s="26"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2060,7 +3248,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9aadbddcbe9a4c6a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1da958630ed4b56"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add S3 lifecycle and presigned access
</commit_message>
<xml_diff>
--- a/docs/reference/CloudVault_Command_Notes.xlsx
+++ b/docs/reference/CloudVault_Command_Notes.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git" sheetId="1" r:id="R35df907d7fff4e8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AWS" sheetId="2" r:id="R2f41afc885e44f1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PowerShell" sheetId="3" r:id="R6d889de494064163"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git" sheetId="1" r:id="R0d587a18a6124b10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AWS" sheetId="2" r:id="R2f8300b475cb47f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PowerShell" sheetId="3" r:id="Rdff23400cd1e48b3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1094,8 +1094,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c6aa9abc06c480a"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58a4cccfc5cc4985"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b210b7f79e14212"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6afa0b216704490c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2075,74 +2075,166 @@
       <x:c r="E65" s="26"/>
     </x:row>
     <x:row r="66" ht="15" hidden="0" customHeight="1">
-      <x:c r="A66" s="26"/>
+      <x:c r="A66" s="26" t="str">
+        <x:v>Additional AWS CLI Commands — S3 Lifecycle &amp; Presigned Access</x:v>
+      </x:c>
       <x:c r="B66" s="26"/>
       <x:c r="C66" s="26"/>
       <x:c r="D66" s="26"/>
       <x:c r="E66" s="26"/>
     </x:row>
     <x:row r="67" ht="15" hidden="0" customHeight="1">
-      <x:c r="A67" s="26"/>
-      <x:c r="B67" s="26"/>
-      <x:c r="C67" s="26"/>
-      <x:c r="D67" s="26"/>
-      <x:c r="E67" s="26"/>
+      <x:c r="A67" s="26" t="str">
+        <x:v>Command</x:v>
+      </x:c>
+      <x:c r="B67" s="26" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="C67" s="26" t="str">
+        <x:v>What it does</x:v>
+      </x:c>
+      <x:c r="D67" s="26" t="str">
+        <x:v>When / Why to use it</x:v>
+      </x:c>
+      <x:c r="E67" s="26" t="str">
+        <x:v>Notes / Cautions</x:v>
+      </x:c>
     </x:row>
     <x:row r="68" ht="15" hidden="0" customHeight="1">
-      <x:c r="A68" s="26"/>
-      <x:c r="B68" s="26"/>
-      <x:c r="C68" s="26"/>
-      <x:c r="D68" s="26"/>
-      <x:c r="E68" s="26"/>
+      <x:c r="A68" s="26" t="str">
+        <x:v>aws s3api put-bucket-lifecycle-configuration --bucket cloudvault-documents-dev01 --lifecycle-configuration file://s3/config/lifecycle.json --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B68" s="26" t="str">
+        <x:v>S3 / Lifecycle</x:v>
+      </x:c>
+      <x:c r="C68" s="26" t="str">
+        <x:v>Applies the lifecycle configuration stored in s3/config/lifecycle.json to the CloudVault bucket.</x:v>
+      </x:c>
+      <x:c r="D68" s="26" t="str">
+        <x:v>Use after validating the local lifecycle JSON and when intentionally changing lifecycle behavior.</x:v>
+      </x:c>
+      <x:c r="E68" s="26" t="str">
+        <x:v>The current rule expires noncurrent versions under documents/ after 30 days. Lifecycle processing is asynchronous.</x:v>
+      </x:c>
     </x:row>
     <x:row r="69" ht="15" hidden="0" customHeight="1">
-      <x:c r="A69" s="26"/>
-      <x:c r="B69" s="26"/>
-      <x:c r="C69" s="26"/>
-      <x:c r="D69" s="26"/>
-      <x:c r="E69" s="26"/>
+      <x:c r="A69" s="26" t="str">
+        <x:v>aws s3api get-bucket-lifecycle-configuration --bucket cloudvault-documents-dev01 --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B69" s="26" t="str">
+        <x:v>S3 / Lifecycle / Validation</x:v>
+      </x:c>
+      <x:c r="C69" s="26" t="str">
+        <x:v>Retrieves the active lifecycle configuration from S3.</x:v>
+      </x:c>
+      <x:c r="D69" s="26" t="str">
+        <x:v>Use after applying a lifecycle rule to verify AWS stored the intended configuration.</x:v>
+      </x:c>
+      <x:c r="E69" s="26" t="str">
+        <x:v>The returned TransitionDefaultMinimumObjectSize field does not mean a storage-class transition rule was configured.</x:v>
+      </x:c>
     </x:row>
     <x:row r="70" ht="15" hidden="0" customHeight="1">
-      <x:c r="A70" s="26"/>
-      <x:c r="B70" s="26"/>
-      <x:c r="C70" s="26"/>
-      <x:c r="D70" s="26"/>
-      <x:c r="E70" s="26"/>
+      <x:c r="A70" s="26" t="str">
+        <x:v>aws s3api head-object --bucket cloudvault-documents-dev01 --key documents/sample.txt --query "{StorageClass:StorageClass,Size:ContentLength,Encryption:ServerSideEncryption,LastModified:LastModified}" --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B70" s="26" t="str">
+        <x:v>S3 / Storage Class</x:v>
+      </x:c>
+      <x:c r="C70" s="26" t="str">
+        <x:v>Inspects selected object properties including storage class, size, encryption, and modification time.</x:v>
+      </x:c>
+      <x:c r="D70" s="26" t="str">
+        <x:v>Use while reviewing the current storage class without downloading the object.</x:v>
+      </x:c>
+      <x:c r="E70" s="26" t="str">
+        <x:v>StorageClass: null indicates the default S3 Standard storage class for this object.</x:v>
+      </x:c>
     </x:row>
     <x:row r="71" ht="15" hidden="0" customHeight="1">
-      <x:c r="A71" s="26"/>
-      <x:c r="B71" s="26"/>
-      <x:c r="C71" s="26"/>
-      <x:c r="D71" s="26"/>
-      <x:c r="E71" s="26"/>
+      <x:c r="A71" s="26" t="str">
+        <x:v>aws s3 presign s3://cloudvault-documents-dev01/documents/sample.txt --expires-in 300 --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B71" s="26" t="str">
+        <x:v>S3 / Presigned URL</x:v>
+      </x:c>
+      <x:c r="C71" s="26" t="str">
+        <x:v>Generates a temporary presigned GET URL for the private sample object.</x:v>
+      </x:c>
+      <x:c r="D71" s="26" t="str">
+        <x:v>Use to test temporary private download access without making the bucket public.</x:v>
+      </x:c>
+      <x:c r="E71" s="26" t="str">
+        <x:v>Treat the generated URL as sensitive while valid. Do not commit or publish it.</x:v>
+      </x:c>
     </x:row>
     <x:row r="72" ht="15" hidden="0" customHeight="1">
-      <x:c r="A72" s="26"/>
-      <x:c r="B72" s="26"/>
-      <x:c r="C72" s="26"/>
-      <x:c r="D72" s="26"/>
-      <x:c r="E72" s="26"/>
+      <x:c r="A72" s="26" t="str">
+        <x:v>aws s3api get-public-access-block --bucket cloudvault-documents-dev01 --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B72" s="26" t="str">
+        <x:v>S3 / Security / Validation</x:v>
+      </x:c>
+      <x:c r="C72" s="26" t="str">
+        <x:v>Retrieves the bucket's four Block Public Access settings.</x:v>
+      </x:c>
+      <x:c r="D72" s="26" t="str">
+        <x:v>Use after presigned-access tests to confirm the bucket remains private.</x:v>
+      </x:c>
+      <x:c r="E72" s="26" t="str">
+        <x:v>CloudVault expects all four settings to remain true.</x:v>
+      </x:c>
     </x:row>
     <x:row r="73" ht="15" hidden="0" customHeight="1">
-      <x:c r="A73" s="26"/>
-      <x:c r="B73" s="26"/>
-      <x:c r="C73" s="26"/>
-      <x:c r="D73" s="26"/>
-      <x:c r="E73" s="26"/>
+      <x:c r="A73" s="26" t="str">
+        <x:v>aws s3api head-object --bucket cloudvault-documents-dev01 --key documents/presigned-upload-test.txt --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B73" s="26" t="str">
+        <x:v>S3 / Presigned PUT / Validation</x:v>
+      </x:c>
+      <x:c r="C73" s="26" t="str">
+        <x:v>Retrieves metadata for the object uploaded through the presigned PUT URL.</x:v>
+      </x:c>
+      <x:c r="D73" s="26" t="str">
+        <x:v>Use to prove the direct HTTP upload created the expected S3 object.</x:v>
+      </x:c>
+      <x:c r="E73" s="26" t="str">
+        <x:v>The test confirmed text/plain, SSE-S3 AES256, and a version ID.</x:v>
+      </x:c>
     </x:row>
     <x:row r="74" ht="15" hidden="0" customHeight="1">
-      <x:c r="A74" s="26"/>
-      <x:c r="B74" s="26"/>
-      <x:c r="C74" s="26"/>
-      <x:c r="D74" s="26"/>
-      <x:c r="E74" s="26"/>
+      <x:c r="A74" s="26" t="str">
+        <x:v>aws s3api head-object --bucket cloudvault-documents-dev01 --key documents/presigned-upload-test.txt --query "{Size:ContentLength,ContentType:ContentType,Encryption:ServerSideEncryption,StorageClass:StorageClass,VersionId:VersionId,LastModified:LastModified}" --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B74" s="26" t="str">
+        <x:v>S3 / Presigned PUT / Validation</x:v>
+      </x:c>
+      <x:c r="C74" s="26" t="str">
+        <x:v>Returns a concise view of the uploaded object's important properties.</x:v>
+      </x:c>
+      <x:c r="D74" s="26" t="str">
+        <x:v>Use for readable validation output after a presigned PUT upload.</x:v>
+      </x:c>
+      <x:c r="E74" s="26" t="str">
+        <x:v>Do not publish object version IDs unnecessarily.</x:v>
+      </x:c>
     </x:row>
     <x:row r="75" ht="15" hidden="0" customHeight="1">
-      <x:c r="A75" s="26"/>
-      <x:c r="B75" s="26"/>
-      <x:c r="C75" s="26"/>
-      <x:c r="D75" s="26"/>
-      <x:c r="E75" s="26"/>
+      <x:c r="A75" s="26" t="str">
+        <x:v>aws s3 cp s3://cloudvault-documents-dev01/documents/presigned-upload-test.txt .\test-data\presigned-upload-verified.txt --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B75" s="26" t="str">
+        <x:v>S3 / Download / Validation</x:v>
+      </x:c>
+      <x:c r="C75" s="26" t="str">
+        <x:v>Downloads the object uploaded through the presigned PUT workflow.</x:v>
+      </x:c>
+      <x:c r="D75" s="26" t="str">
+        <x:v>Use to verify the uploaded content can be retrieved and compared locally.</x:v>
+      </x:c>
+      <x:c r="E75" s="26" t="str">
+        <x:v>test-data/ is local test material and should remain ignored by Git.</x:v>
+      </x:c>
     </x:row>
     <x:row r="76" ht="15" hidden="0" customHeight="1">
       <x:c r="A76" s="26"/>
@@ -2261,7 +2353,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26d6e1466150435f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62eb351df2524248"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2918,109 +3010,251 @@
       <x:c r="E44" s="26"/>
     </x:row>
     <x:row r="45" ht="15" hidden="0" customHeight="1">
-      <x:c r="A45" s="26"/>
+      <x:c r="A45" s="26" t="str">
+        <x:v>Additional PowerShell Commands — Lifecycle, Python &amp; Presigned PUT</x:v>
+      </x:c>
       <x:c r="B45" s="26"/>
       <x:c r="C45" s="26"/>
       <x:c r="D45" s="26"/>
       <x:c r="E45" s="26"/>
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
-      <x:c r="A46" s="26"/>
-      <x:c r="B46" s="26"/>
-      <x:c r="C46" s="26"/>
-      <x:c r="D46" s="26"/>
-      <x:c r="E46" s="26"/>
+      <x:c r="A46" s="26" t="str">
+        <x:v>Command</x:v>
+      </x:c>
+      <x:c r="B46" s="26" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="C46" s="26" t="str">
+        <x:v>What it does</x:v>
+      </x:c>
+      <x:c r="D46" s="26" t="str">
+        <x:v>When / Why to use it</x:v>
+      </x:c>
+      <x:c r="E46" s="26" t="str">
+        <x:v>Notes / Cautions</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
-      <x:c r="A47" s="26"/>
-      <x:c r="B47" s="26"/>
-      <x:c r="C47" s="26"/>
-      <x:c r="D47" s="26"/>
-      <x:c r="E47" s="26"/>
+      <x:c r="A47" s="26" t="str">
+        <x:v>Get-Content .\s3\config\lifecycle.json -Raw | ConvertFrom-Json | Out-Null; Write-Host "Lifecycle JSON is valid."</x:v>
+      </x:c>
+      <x:c r="B47" s="26" t="str">
+        <x:v>JSON Validation / S3</x:v>
+      </x:c>
+      <x:c r="C47" s="26" t="str">
+        <x:v>Reads the lifecycle configuration as one string, parses it as JSON, and prints a success message when valid.</x:v>
+      </x:c>
+      <x:c r="D47" s="26" t="str">
+        <x:v>Use before applying s3/config/lifecycle.json to AWS.</x:v>
+      </x:c>
+      <x:c r="E47" s="26" t="str">
+        <x:v>A space is required before -Raw; lifecycle.json-Raw is an invalid path.</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
-      <x:c r="A48" s="26"/>
-      <x:c r="B48" s="26"/>
-      <x:c r="C48" s="26"/>
-      <x:c r="D48" s="26"/>
-      <x:c r="E48" s="26"/>
+      <x:c r="A48" s="26" t="str">
+        <x:v>Set-Content -Path .\test-data\presigned-upload-test.txt -Value "CloudVault presigned upload test."</x:v>
+      </x:c>
+      <x:c r="B48" s="26" t="str">
+        <x:v>Test Data</x:v>
+      </x:c>
+      <x:c r="C48" s="26" t="str">
+        <x:v>Creates the local text file used for the presigned PUT exercise.</x:v>
+      </x:c>
+      <x:c r="D48" s="26" t="str">
+        <x:v>Use to create a harmless local object for direct HTTP upload testing.</x:v>
+      </x:c>
+      <x:c r="E48" s="26" t="str">
+        <x:v>The test-data/ directory is ignored by Git.</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
-      <x:c r="A49" s="26"/>
-      <x:c r="B49" s="26"/>
-      <x:c r="C49" s="26"/>
-      <x:c r="D49" s="26"/>
-      <x:c r="E49" s="26"/>
+      <x:c r="A49" s="26" t="str">
+        <x:v>winget install --id Python.Python.3.13 -e</x:v>
+      </x:c>
+      <x:c r="B49" s="26" t="str">
+        <x:v>Package Management / Python</x:v>
+      </x:c>
+      <x:c r="C49" s="26" t="str">
+        <x:v>Installs Python 3.13 through Windows Package Manager using an exact package ID match.</x:v>
+      </x:c>
+      <x:c r="D49" s="26" t="str">
+        <x:v>Used to add Python for the Boto3 presigned PUT exercise.</x:v>
+      </x:c>
+      <x:c r="E49" s="26" t="str">
+        <x:v>Reopen PowerShell after installation if python is not immediately recognized.</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
-      <x:c r="A50" s="26"/>
-      <x:c r="B50" s="26"/>
-      <x:c r="C50" s="26"/>
-      <x:c r="D50" s="26"/>
-      <x:c r="E50" s="26"/>
+      <x:c r="A50" s="26" t="str">
+        <x:v>python --version</x:v>
+      </x:c>
+      <x:c r="B50" s="26" t="str">
+        <x:v>Python / Validation</x:v>
+      </x:c>
+      <x:c r="C50" s="26" t="str">
+        <x:v>Displays the active Python version.</x:v>
+      </x:c>
+      <x:c r="D50" s="26" t="str">
+        <x:v>Use after installation to confirm Python is available.</x:v>
+      </x:c>
+      <x:c r="E50" s="26" t="str">
+        <x:v>The lab used Python 3.13.</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
-      <x:c r="A51" s="26"/>
-      <x:c r="B51" s="26"/>
-      <x:c r="C51" s="26"/>
-      <x:c r="D51" s="26"/>
-      <x:c r="E51" s="26"/>
+      <x:c r="A51" s="26" t="str">
+        <x:v>python -m pip --version</x:v>
+      </x:c>
+      <x:c r="B51" s="26" t="str">
+        <x:v>Python / Validation</x:v>
+      </x:c>
+      <x:c r="C51" s="26" t="str">
+        <x:v>Displays the pip version associated with the active Python interpreter.</x:v>
+      </x:c>
+      <x:c r="D51" s="26" t="str">
+        <x:v>Use before installing Python packages to confirm pip is available for that interpreter.</x:v>
+      </x:c>
+      <x:c r="E51" s="26" t="str">
+        <x:v>Using python -m pip helps avoid ambiguity when multiple Python installations exist.</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
-      <x:c r="A52" s="26"/>
-      <x:c r="B52" s="26"/>
-      <x:c r="C52" s="26"/>
-      <x:c r="D52" s="26"/>
-      <x:c r="E52" s="26"/>
+      <x:c r="A52" s="26" t="str">
+        <x:v>python -m pip install boto3</x:v>
+      </x:c>
+      <x:c r="B52" s="26" t="str">
+        <x:v>Python / AWS SDK</x:v>
+      </x:c>
+      <x:c r="C52" s="26" t="str">
+        <x:v>Installs Boto3, the AWS SDK for Python, and its normal dependencies.</x:v>
+      </x:c>
+      <x:c r="D52" s="26" t="str">
+        <x:v>Required by scripts/presigned_put.py.</x:v>
+      </x:c>
+      <x:c r="E52" s="26" t="str">
+        <x:v>The lab installed packages into the local Python environment; no AWS credentials are embedded in Boto3.</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="15" hidden="0" customHeight="1">
-      <x:c r="A53" s="26"/>
-      <x:c r="B53" s="26"/>
-      <x:c r="C53" s="26"/>
-      <x:c r="D53" s="26"/>
-      <x:c r="E53" s="26"/>
+      <x:c r="A53" s="26" t="str">
+        <x:v>python -m pip install "botocore[crt]"</x:v>
+      </x:c>
+      <x:c r="B53" s="26" t="str">
+        <x:v>Python / AWS Authentication</x:v>
+      </x:c>
+      <x:c r="C53" s="26" t="str">
+        <x:v>Installs Botocore's AWS Common Runtime dependency.</x:v>
+      </x:c>
+      <x:c r="D53" s="26" t="str">
+        <x:v>Required in this environment so Boto3 can use the AWS CLI login credential provider.</x:v>
+      </x:c>
+      <x:c r="E53" s="26" t="str">
+        <x:v>This was needed after MissingDependencyException reported that login credentials require the CRT dependency.</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
-      <x:c r="A54" s="26"/>
-      <x:c r="B54" s="26"/>
-      <x:c r="C54" s="26"/>
-      <x:c r="D54" s="26"/>
-      <x:c r="E54" s="26"/>
+      <x:c r="A54" s="26" t="str">
+        <x:v>python -c "import boto3; print(boto3.__version__)"</x:v>
+      </x:c>
+      <x:c r="B54" s="26" t="str">
+        <x:v>Python / Validation</x:v>
+      </x:c>
+      <x:c r="C54" s="26" t="str">
+        <x:v>Imports Boto3 and prints its installed version.</x:v>
+      </x:c>
+      <x:c r="D54" s="26" t="str">
+        <x:v>Use to confirm Boto3 installed successfully.</x:v>
+      </x:c>
+      <x:c r="E54" s="26" t="str">
+        <x:v>Useful before running a project script that imports boto3.</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="15" hidden="0" customHeight="1">
-      <x:c r="A55" s="26"/>
-      <x:c r="B55" s="26"/>
-      <x:c r="C55" s="26"/>
-      <x:c r="D55" s="26"/>
-      <x:c r="E55" s="26"/>
+      <x:c r="A55" s="26" t="str">
+        <x:v>python -c "import boto3; s=boto3.Session(profile_name='cloudvault'); print(s.region_name); print(s.client('sts').get_caller_identity()['Arn'])"</x:v>
+      </x:c>
+      <x:c r="B55" s="26" t="str">
+        <x:v>Python / AWS Validation</x:v>
+      </x:c>
+      <x:c r="C55" s="26" t="str">
+        <x:v>Creates a Boto3 session from the cloudvault profile and calls STS to prove authentication works.</x:v>
+      </x:c>
+      <x:c r="D55" s="26" t="str">
+        <x:v>Use after installing botocore[crt] to validate the existing login-based profile from Python.</x:v>
+      </x:c>
+      <x:c r="E55" s="26" t="str">
+        <x:v>The returned ARN can contain account-specific information; redact it from public screenshots.</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="15" hidden="0" customHeight="1">
-      <x:c r="A56" s="26"/>
-      <x:c r="B56" s="26"/>
-      <x:c r="C56" s="26"/>
-      <x:c r="D56" s="26"/>
-      <x:c r="E56" s="26"/>
+      <x:c r="A56" s="26" t="str">
+        <x:v>python .\scripts\presigned_put.py</x:v>
+      </x:c>
+      <x:c r="B56" s="26" t="str">
+        <x:v>Python / Presigned URL</x:v>
+      </x:c>
+      <x:c r="C56" s="26" t="str">
+        <x:v>Runs the CloudVault learning script that generates a five-minute presigned PUT URL.</x:v>
+      </x:c>
+      <x:c r="D56" s="26" t="str">
+        <x:v>Use immediately before the direct HTTP upload test.</x:v>
+      </x:c>
+      <x:c r="E56" s="26" t="str">
+        <x:v>Do not commit, log, or publicly share the generated URL while it is valid.</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="15" hidden="0" customHeight="1">
-      <x:c r="A57" s="26"/>
-      <x:c r="B57" s="26"/>
-      <x:c r="C57" s="26"/>
-      <x:c r="D57" s="26"/>
-      <x:c r="E57" s="26"/>
+      <x:c r="A57" s="26" t="str">
+        <x:v>$PresignedUrl = "PASTE_THE_GENERATED_URL_HERE"</x:v>
+      </x:c>
+      <x:c r="B57" s="26" t="str">
+        <x:v>PowerShell Variable / Security</x:v>
+      </x:c>
+      <x:c r="C57" s="26" t="str">
+        <x:v>Stores the temporary presigned URL in a PowerShell variable for the current session.</x:v>
+      </x:c>
+      <x:c r="D57" s="26" t="str">
+        <x:v>Use to avoid repeatedly pasting the long URL into the upload command.</x:v>
+      </x:c>
+      <x:c r="E57" s="26" t="str">
+        <x:v>The URL is a temporary bearer-style credential. Never commit the real value.</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="15" hidden="0" customHeight="1">
-      <x:c r="A58" s="26"/>
-      <x:c r="B58" s="26"/>
-      <x:c r="C58" s="26"/>
-      <x:c r="D58" s="26"/>
-      <x:c r="E58" s="26"/>
+      <x:c r="A58" s="26" t="str">
+        <x:v>Invoke-WebRequest -Uri $PresignedUrl -Method Put -InFile .\test-data\presigned-upload-test.txt -ContentType "text/plain"</x:v>
+      </x:c>
+      <x:c r="B58" s="26" t="str">
+        <x:v>HTTP / S3</x:v>
+      </x:c>
+      <x:c r="C58" s="26" t="str">
+        <x:v>Uploads the local test file directly to S3 using the presigned PUT URL.</x:v>
+      </x:c>
+      <x:c r="D58" s="26" t="str">
+        <x:v>Use to demonstrate that a client can upload without possessing AWS CLI credentials.</x:v>
+      </x:c>
+      <x:c r="E58" s="26" t="str">
+        <x:v>Content-Type must match the value included when the URL was signed. The successful lab returned HTTP 200 OK.</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="15" hidden="0" customHeight="1">
-      <x:c r="A59" s="26"/>
-      <x:c r="B59" s="26"/>
-      <x:c r="C59" s="26"/>
-      <x:c r="D59" s="26"/>
-      <x:c r="E59" s="26"/>
+      <x:c r="A59" s="26" t="str">
+        <x:v>Get-Content .\test-data\presigned-upload-verified.txt</x:v>
+      </x:c>
+      <x:c r="B59" s="26" t="str">
+        <x:v>File Inspection / Validation</x:v>
+      </x:c>
+      <x:c r="C59" s="26" t="str">
+        <x:v>Displays the contents of the object after it has been downloaded back from S3.</x:v>
+      </x:c>
+      <x:c r="D59" s="26" t="str">
+        <x:v>Use as the final content check for the presigned PUT workflow.</x:v>
+      </x:c>
+      <x:c r="E59" s="26" t="str">
+        <x:v>Expected test content: CloudVault presigned upload test.</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="15" hidden="0" customHeight="1">
       <x:c r="A60" s="26"/>
@@ -3248,7 +3482,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1da958630ed4b56"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbda1694b99144895"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: complete Phase 1 S3 documentation
</commit_message>
<xml_diff>
--- a/docs/reference/CloudVault_Command_Notes.xlsx
+++ b/docs/reference/CloudVault_Command_Notes.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git" sheetId="1" r:id="R0d587a18a6124b10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AWS" sheetId="2" r:id="R2f8300b475cb47f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PowerShell" sheetId="3" r:id="Rdff23400cd1e48b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git" sheetId="1" r:id="R5fb0f65387df4b9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AWS" sheetId="2" r:id="R38542316415c4cee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PowerShell" sheetId="3" r:id="R63513dbf896047a8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1085,6 +1085,229 @@
       <x:c r="D42" s="36"/>
       <x:c r="E42" s="36"/>
     </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="26" t="str">
+        <x:v>Additional Git Commands — Protected Branch &amp; Pull Request Workflow</x:v>
+      </x:c>
+      <x:c r="B44" s="26"/>
+      <x:c r="C44" s="26"/>
+      <x:c r="D44" s="26"/>
+      <x:c r="E44" s="26"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="26" t="str">
+        <x:v>Command</x:v>
+      </x:c>
+      <x:c r="B45" s="26" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="C45" s="26" t="str">
+        <x:v>What it does</x:v>
+      </x:c>
+      <x:c r="D45" s="26" t="str">
+        <x:v>When / Why to use it</x:v>
+      </x:c>
+      <x:c r="E45" s="26" t="str">
+        <x:v>Notes / Cautions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="26" t="str">
+        <x:v>git switch -c feat/s3-lifecycle-presigned-access</x:v>
+      </x:c>
+      <x:c r="B46" s="26" t="str">
+        <x:v>Branching</x:v>
+      </x:c>
+      <x:c r="C46" s="26" t="str">
+        <x:v>Creates a new branch and switches to it in one command.</x:v>
+      </x:c>
+      <x:c r="D46" s="26" t="str">
+        <x:v>Use before making Phase 1 changes when main is protected and work must go through a pull request.</x:v>
+      </x:c>
+      <x:c r="E46" s="26" t="str">
+        <x:v>Choose a short descriptive branch name that reflects the work.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="26" t="str">
+        <x:v>git push -u origin feat/s3-lifecycle-presigned-access</x:v>
+      </x:c>
+      <x:c r="B47" s="26" t="str">
+        <x:v>Remote / Branching</x:v>
+      </x:c>
+      <x:c r="C47" s="26" t="str">
+        <x:v>Pushes the feature branch to origin and configures its upstream tracking branch.</x:v>
+      </x:c>
+      <x:c r="D47" s="26" t="str">
+        <x:v>Use after committing work that should be opened as a GitHub pull request.</x:v>
+      </x:c>
+      <x:c r="E47" s="26" t="str">
+        <x:v>After upstream is configured, later pushes from the branch can normally use git push.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="26" t="str">
+        <x:v>git diff --staged</x:v>
+      </x:c>
+      <x:c r="B48" s="26" t="str">
+        <x:v>Inspection</x:v>
+      </x:c>
+      <x:c r="C48" s="26" t="str">
+        <x:v>Shows the exact changes currently staged for the next commit.</x:v>
+      </x:c>
+      <x:c r="D48" s="26" t="str">
+        <x:v>Use after git add and before git commit to review what will actually be committed.</x:v>
+      </x:c>
+      <x:c r="E48" s="26" t="str">
+        <x:v>Especially useful for checking that secrets, generated files, or unrelated changes were not staged.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="26" t="str">
+        <x:v>git switch main</x:v>
+      </x:c>
+      <x:c r="B49" s="26" t="str">
+        <x:v>Branching</x:v>
+      </x:c>
+      <x:c r="C49" s="26" t="str">
+        <x:v>Switches the working tree back to the local main branch.</x:v>
+      </x:c>
+      <x:c r="D49" s="26" t="str">
+        <x:v>Use after a pull request is merged and you are ready to synchronize local main.</x:v>
+      </x:c>
+      <x:c r="E49" s="26" t="str">
+        <x:v>Commit or safely handle outstanding work before switching branches.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="26" t="str">
+        <x:v>git fetch origin</x:v>
+      </x:c>
+      <x:c r="B50" s="26" t="str">
+        <x:v>Remote / Synchronization</x:v>
+      </x:c>
+      <x:c r="C50" s="26" t="str">
+        <x:v>Downloads updated remote references from origin without merging them into the current branch.</x:v>
+      </x:c>
+      <x:c r="D50" s="26" t="str">
+        <x:v>Use after a GitHub pull request is merged so origin/main reflects the latest remote state.</x:v>
+      </x:c>
+      <x:c r="E50" s="26" t="str">
+        <x:v>Unlike git pull, fetch does not integrate changes into the current branch.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="26" t="str">
+        <x:v>git reset --hard origin/main</x:v>
+      </x:c>
+      <x:c r="B51" s="26" t="str">
+        <x:v>Synchronization</x:v>
+      </x:c>
+      <x:c r="C51" s="26" t="str">
+        <x:v>Makes the current local branch and working tree exactly match the origin/main remote-tracking reference.</x:v>
+      </x:c>
+      <x:c r="D51" s="26" t="str">
+        <x:v>Used after the Phase 1 squash merge to synchronize local main with GitHub's new squash commit.</x:v>
+      </x:c>
+      <x:c r="E51" s="26" t="str">
+        <x:v>Destructive to uncommitted/local-only changes. Run git status first and use only when intentionally discarding local divergence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="26" t="str">
+        <x:v>git branch -d feat/s3-lifecycle-presigned-access</x:v>
+      </x:c>
+      <x:c r="B52" s="26" t="str">
+        <x:v>Branch Cleanup</x:v>
+      </x:c>
+      <x:c r="C52" s="26" t="str">
+        <x:v>Deletes the specified local feature branch when Git considers it safely deletable.</x:v>
+      </x:c>
+      <x:c r="D52" s="26" t="str">
+        <x:v>Use after the pull request has been merged and the branch is no longer needed locally.</x:v>
+      </x:c>
+      <x:c r="E52" s="26" t="str">
+        <x:v>Squash merges create a different commit, so Git may warn that the original branch commit is not merged into local main.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="26" t="str">
+        <x:v>git fetch --prune</x:v>
+      </x:c>
+      <x:c r="B53" s="26" t="str">
+        <x:v>Remote / Cleanup</x:v>
+      </x:c>
+      <x:c r="C53" s="26" t="str">
+        <x:v>Fetches remote updates and removes stale remote-tracking references whose remote branches were deleted.</x:v>
+      </x:c>
+      <x:c r="D53" s="26" t="str">
+        <x:v>Use after deleting a merged branch on GitHub to clean up references such as origin/feature-branch.</x:v>
+      </x:c>
+      <x:c r="E53" s="26" t="str">
+        <x:v>This removes stale tracking references, not your local branches.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="26" t="str">
+        <x:v>git branch -v</x:v>
+      </x:c>
+      <x:c r="B54" s="26" t="str">
+        <x:v>Inspection / Branching</x:v>
+      </x:c>
+      <x:c r="C54" s="26" t="str">
+        <x:v>Lists local branches with their latest commit information.</x:v>
+      </x:c>
+      <x:c r="D54" s="26" t="str">
+        <x:v>Use to inspect local branch state after synchronization or cleanup.</x:v>
+      </x:c>
+      <x:c r="E54" s="26" t="str">
+        <x:v>A compact alternative when git branch -vv/--verbose --verbose behaves unexpectedly in a particular environment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="26" t="str">
+        <x:v>git branch --verbose --verbose</x:v>
+      </x:c>
+      <x:c r="B55" s="26" t="str">
+        <x:v>Inspection / Branching</x:v>
+      </x:c>
+      <x:c r="C55" s="26" t="str">
+        <x:v>Shows local branches, latest commits, and upstream tracking information.</x:v>
+      </x:c>
+      <x:c r="D55" s="26" t="str">
+        <x:v>Use to inspect which remote branch a local branch tracks.</x:v>
+      </x:c>
+      <x:c r="E55" s="26" t="str">
+        <x:v>Equivalent intent to git branch -vv; useful as the explicit long-form syntax.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="26" t="str">
+        <x:v>Protected-main workflow used in Phase 1: feature branch → commit → push branch → pull request → squash merge → switch to main → fetch origin → reset local main to origin/main → delete/prune old branch references.</x:v>
+      </x:c>
+      <x:c r="B57" s="26"/>
+      <x:c r="C57" s="26"/>
+      <x:c r="D57" s="26"/>
+      <x:c r="E57" s="26"/>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="26" t="str">
+        <x:v>Git concept: main is the local branch; origin/main is the local remote-tracking reference representing the last fetched state of main on the origin remote.</x:v>
+      </x:c>
+      <x:c r="B58" s="26"/>
+      <x:c r="C58" s="26"/>
+      <x:c r="D58" s="26"/>
+      <x:c r="E58" s="26"/>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="26" t="str">
+        <x:v>GitHub protection lesson: direct pushes to protected main can be rejected by the repository ruleset, requiring changes to flow through a branch and pull request.</x:v>
+      </x:c>
+      <x:c r="B59" s="26"/>
+      <x:c r="C59" s="26"/>
+      <x:c r="D59" s="26"/>
+      <x:c r="E59" s="26"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:E1"/>
@@ -1094,8 +1317,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b210b7f79e14212"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6afa0b216704490c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12418ee50f364b52"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a1216f84d124298"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2244,102 +2467,302 @@
       <x:c r="E76" s="26"/>
     </x:row>
     <x:row r="77" ht="15" hidden="0" customHeight="1">
-      <x:c r="A77" s="26"/>
+      <x:c r="A77" s="26" t="str">
+        <x:v>Additional AWS CLI Commands — Phase 1 Metadata, Monitoring &amp; Final Validation</x:v>
+      </x:c>
       <x:c r="B77" s="26"/>
       <x:c r="C77" s="26"/>
       <x:c r="D77" s="26"/>
       <x:c r="E77" s="26"/>
     </x:row>
     <x:row r="78" ht="15" hidden="0" customHeight="1">
-      <x:c r="A78" s="26"/>
-      <x:c r="B78" s="26"/>
-      <x:c r="C78" s="26"/>
-      <x:c r="D78" s="26"/>
-      <x:c r="E78" s="26"/>
+      <x:c r="A78" s="26" t="str">
+        <x:v>Command</x:v>
+      </x:c>
+      <x:c r="B78" s="26" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="C78" s="26" t="str">
+        <x:v>What it does</x:v>
+      </x:c>
+      <x:c r="D78" s="26" t="str">
+        <x:v>When / Why to use it</x:v>
+      </x:c>
+      <x:c r="E78" s="26" t="str">
+        <x:v>Notes / Cautions</x:v>
+      </x:c>
     </x:row>
     <x:row r="79" ht="15" hidden="0" customHeight="1">
-      <x:c r="A79" s="26"/>
-      <x:c r="B79" s="26"/>
-      <x:c r="C79" s="26"/>
-      <x:c r="D79" s="26"/>
-      <x:c r="E79" s="26"/>
+      <x:c r="A79" s="26" t="str">
+        <x:v>aws s3api put-object --bucket cloudvault-documents-dev01 --key documents/metadata-test.txt --body .\test-data\metadata-test.txt --content-type "text/plain" --metadata "document-type=learning-note,uploaded-by=cloudvault-cli,project=cloudvault" --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B79" s="26" t="str">
+        <x:v>S3 / Metadata</x:v>
+      </x:c>
+      <x:c r="C79" s="26" t="str">
+        <x:v>Uploads an object with user-defined metadata.</x:v>
+      </x:c>
+      <x:c r="D79" s="26" t="str">
+        <x:v>Use to test custom metadata on an S3 object in the versioned documents/ prefix.</x:v>
+      </x:c>
+      <x:c r="E79" s="26" t="str">
+        <x:v>User-defined metadata is returned by head-object. Keep metadata non-sensitive.</x:v>
+      </x:c>
     </x:row>
     <x:row r="80" ht="15" hidden="0" customHeight="1">
-      <x:c r="A80" s="26"/>
-      <x:c r="B80" s="26"/>
-      <x:c r="C80" s="26"/>
-      <x:c r="D80" s="26"/>
-      <x:c r="E80" s="26"/>
+      <x:c r="A80" s="26" t="str">
+        <x:v>aws s3api copy-object --bucket cloudvault-documents-dev01 --key documents/metadata-test.txt --copy-source cloudvault-documents-dev01/documents/metadata-test.txt --metadata-directive REPLACE --content-type "text/plain" --metadata "document-type=project-note,uploaded-by=cloudvault-cli,project=cloudvault" --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B80" s="26" t="str">
+        <x:v>S3 / Metadata / Versioning</x:v>
+      </x:c>
+      <x:c r="C80" s="26" t="str">
+        <x:v>Copies the object onto the same key while replacing its metadata.</x:v>
+      </x:c>
+      <x:c r="D80" s="26" t="str">
+        <x:v>Use to demonstrate how metadata replacement behaves in a versioned bucket.</x:v>
+      </x:c>
+      <x:c r="E80" s="26" t="str">
+        <x:v>This creates a new object version; the historical version retains its original metadata.</x:v>
+      </x:c>
     </x:row>
     <x:row r="81" ht="15" hidden="0" customHeight="1">
-      <x:c r="A81" s="26"/>
-      <x:c r="B81" s="26"/>
-      <x:c r="C81" s="26"/>
-      <x:c r="D81" s="26"/>
-      <x:c r="E81" s="26"/>
+      <x:c r="A81" s="26" t="str">
+        <x:v>aws s3api head-object --bucket cloudvault-documents-dev01 --key documents/metadata-test.txt --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B81" s="26" t="str">
+        <x:v>S3 / Metadata / Validation</x:v>
+      </x:c>
+      <x:c r="C81" s="26" t="str">
+        <x:v>Retrieves the current object's headers and user-defined metadata.</x:v>
+      </x:c>
+      <x:c r="D81" s="26" t="str">
+        <x:v>Use after metadata upload/replacement to confirm the current version's metadata.</x:v>
+      </x:c>
+      <x:c r="E81" s="26" t="str">
+        <x:v>VersionId may appear in output; avoid publishing it.</x:v>
+      </x:c>
     </x:row>
     <x:row r="82" ht="15" hidden="0" customHeight="1">
-      <x:c r="A82" s="26"/>
-      <x:c r="B82" s="26"/>
-      <x:c r="C82" s="26"/>
-      <x:c r="D82" s="26"/>
-      <x:c r="E82" s="26"/>
+      <x:c r="A82" s="26" t="str">
+        <x:v>aws s3api list-bucket-metrics-configurations --bucket cloudvault-documents-dev01 --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B82" s="26" t="str">
+        <x:v>S3 / Monitoring</x:v>
+      </x:c>
+      <x:c r="C82" s="26" t="str">
+        <x:v>Lists optional S3 request-metrics configurations for the bucket.</x:v>
+      </x:c>
+      <x:c r="D82" s="26" t="str">
+        <x:v>Use to check whether request metrics have been explicitly enabled.</x:v>
+      </x:c>
+      <x:c r="E82" s="26" t="str">
+        <x:v>For the Phase 1 lab, no request-metrics configuration was enabled.</x:v>
+      </x:c>
     </x:row>
     <x:row r="83" ht="15" hidden="0" customHeight="1">
-      <x:c r="A83" s="26"/>
-      <x:c r="B83" s="26"/>
-      <x:c r="C83" s="26"/>
-      <x:c r="D83" s="26"/>
-      <x:c r="E83" s="26"/>
+      <x:c r="A83" s="26" t="str">
+        <x:v>aws cloudwatch list-metrics --namespace AWS/S3 --dimensions Name=BucketName,Value=cloudvault-documents-dev01 --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B83" s="26" t="str">
+        <x:v>CloudWatch / S3</x:v>
+      </x:c>
+      <x:c r="C83" s="26" t="str">
+        <x:v>Lists CloudWatch metrics associated with the CloudVault S3 bucket.</x:v>
+      </x:c>
+      <x:c r="D83" s="26" t="str">
+        <x:v>Use to discover the automatic daily S3 storage metrics available for the bucket.</x:v>
+      </x:c>
+      <x:c r="E83" s="26" t="str">
+        <x:v>Phase 1 observed BucketSizeBytes and NumberOfObjects.</x:v>
+      </x:c>
     </x:row>
     <x:row r="84" ht="15" hidden="0" customHeight="1">
-      <x:c r="A84" s="26"/>
-      <x:c r="B84" s="26"/>
-      <x:c r="C84" s="26"/>
-      <x:c r="D84" s="26"/>
-      <x:c r="E84" s="26"/>
+      <x:c r="A84" s="26" t="str">
+        <x:v>aws cloudtrail describe-trails --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B84" s="26" t="str">
+        <x:v>CloudTrail / Validation</x:v>
+      </x:c>
+      <x:c r="C84" s="26" t="str">
+        <x:v>Lists customer-created CloudTrail trails visible to the account.</x:v>
+      </x:c>
+      <x:c r="D84" s="26" t="str">
+        <x:v>Use to determine whether a dedicated trail has been configured.</x:v>
+      </x:c>
+      <x:c r="E84" s="26" t="str">
+        <x:v>Phase 1 intentionally had no customer-created trail.</x:v>
+      </x:c>
     </x:row>
     <x:row r="85" ht="15" hidden="0" customHeight="1">
-      <x:c r="A85" s="26"/>
-      <x:c r="B85" s="26"/>
-      <x:c r="C85" s="26"/>
-      <x:c r="D85" s="26"/>
-      <x:c r="E85" s="26"/>
+      <x:c r="A85" s="26" t="str">
+        <x:v>aws cloudtrail lookup-events --lookup-attributes AttributeKey=EventSource,AttributeValue=s3.amazonaws.com --max-results 10 --query "Events[].{EventName:EventName,EventTime:EventTime}" --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B85" s="26" t="str">
+        <x:v>CloudTrail / Event History</x:v>
+      </x:c>
+      <x:c r="C85" s="26" t="str">
+        <x:v>Looks up recent S3 management events in CloudTrail Event History.</x:v>
+      </x:c>
+      <x:c r="D85" s="26" t="str">
+        <x:v>Use to review bucket-level API activity without creating a dedicated trail.</x:v>
+      </x:c>
+      <x:c r="E85" s="26" t="str">
+        <x:v>S3 object-level data events are separate and were not enabled in Phase 1.</x:v>
+      </x:c>
     </x:row>
     <x:row r="86" ht="15" hidden="0" customHeight="1">
-      <x:c r="A86" s="26"/>
-      <x:c r="B86" s="26"/>
-      <x:c r="C86" s="26"/>
-      <x:c r="D86" s="26"/>
-      <x:c r="E86" s="26"/>
+      <x:c r="A86" s="26" t="str">
+        <x:v>aws s3api list-objects-v2 --bucket cloudvault-documents-dev01 --prefix documents/ --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B86" s="26" t="str">
+        <x:v>S3 / Inventory</x:v>
+      </x:c>
+      <x:c r="C86" s="26" t="str">
+        <x:v>Lists current objects under the documents/ prefix.</x:v>
+      </x:c>
+      <x:c r="D86" s="26" t="str">
+        <x:v>Use during final validation to inventory the current S3 objects.</x:v>
+      </x:c>
+      <x:c r="E86" s="26" t="str">
+        <x:v>This does not include noncurrent versions or delete markers.</x:v>
+      </x:c>
     </x:row>
     <x:row r="87" ht="15" hidden="0" customHeight="1">
-      <x:c r="A87" s="26"/>
-      <x:c r="B87" s="26"/>
-      <x:c r="C87" s="26"/>
-      <x:c r="D87" s="26"/>
-      <x:c r="E87" s="26"/>
+      <x:c r="A87" s="26" t="str">
+        <x:v>aws s3api list-object-versions --bucket cloudvault-documents-dev01 --prefix documents/ --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B87" s="26" t="str">
+        <x:v>S3 / Inventory / Versioning</x:v>
+      </x:c>
+      <x:c r="C87" s="26" t="str">
+        <x:v>Lists current/noncurrent versions and delete markers under documents/.</x:v>
+      </x:c>
+      <x:c r="D87" s="26" t="str">
+        <x:v>Use during final validation to understand versioned storage state.</x:v>
+      </x:c>
+      <x:c r="E87" s="26" t="str">
+        <x:v>Avoid publishing real object version IDs.</x:v>
+      </x:c>
     </x:row>
     <x:row r="88" ht="15" hidden="0" customHeight="1">
-      <x:c r="A88" s="26"/>
-      <x:c r="B88" s="26"/>
-      <x:c r="C88" s="26"/>
-      <x:c r="D88" s="26"/>
-      <x:c r="E88" s="26"/>
+      <x:c r="A88" s="26" t="str">
+        <x:v>aws s3api list-multipart-uploads --bucket cloudvault-documents-dev01 --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B88" s="26" t="str">
+        <x:v>S3 / Inventory / Cleanup</x:v>
+      </x:c>
+      <x:c r="C88" s="26" t="str">
+        <x:v>Lists incomplete multipart uploads for the bucket.</x:v>
+      </x:c>
+      <x:c r="D88" s="26" t="str">
+        <x:v>Use during cost/storage hygiene checks to find abandoned multipart uploads.</x:v>
+      </x:c>
+      <x:c r="E88" s="26" t="str">
+        <x:v>No Uploads array means there are no incomplete multipart uploads.</x:v>
+      </x:c>
     </x:row>
     <x:row r="89" ht="15" hidden="0" customHeight="1">
-      <x:c r="A89" s="26"/>
-      <x:c r="B89" s="26"/>
-      <x:c r="C89" s="26"/>
-      <x:c r="D89" s="26"/>
-      <x:c r="E89" s="26"/>
+      <x:c r="A89" s="26" t="str">
+        <x:v>aws s3api get-bucket-policy --bucket cloudvault-documents-dev01 --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B89" s="26" t="str">
+        <x:v>S3 / Security / Validation</x:v>
+      </x:c>
+      <x:c r="C89" s="26" t="str">
+        <x:v>Retrieves the bucket policy if one exists.</x:v>
+      </x:c>
+      <x:c r="D89" s="26" t="str">
+        <x:v>Use during final security validation to confirm whether access is controlled by a bucket policy.</x:v>
+      </x:c>
+      <x:c r="E89" s="26" t="str">
+        <x:v>NoSuchBucketPolicy was expected for the current IAM identity-policy design.</x:v>
+      </x:c>
     </x:row>
     <x:row r="90" ht="15" hidden="0" customHeight="1">
-      <x:c r="A90" s="26"/>
-      <x:c r="B90" s="26"/>
-      <x:c r="C90" s="26"/>
-      <x:c r="D90" s="26"/>
-      <x:c r="E90" s="26"/>
+      <x:c r="A90" s="26" t="str">
+        <x:v>aws iam get-role --role-name CloudVaultEC2Role --query "Role.{RoleName:RoleName,TrustPolicy:AssumeRolePolicyDocument,Tags:Tags}" --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B90" s="26" t="str">
+        <x:v>IAM / Final Validation</x:v>
+      </x:c>
+      <x:c r="C90" s="26" t="str">
+        <x:v>Returns a privacy-reduced view of the role name, trust policy, and tags.</x:v>
+      </x:c>
+      <x:c r="D90" s="26" t="str">
+        <x:v>Use for final IAM validation without printing the account-specific role ARN.</x:v>
+      </x:c>
+      <x:c r="E90" s="26" t="str">
+        <x:v>Verify EC2 trust and sts:AssumeRole. Runtime EC2 testing remains deferred.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" s="26" t="str">
+        <x:v>aws iam list-attached-role-policies --role-name CloudVaultEC2Role --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B91" s="26" t="str">
+        <x:v>IAM / Final Validation</x:v>
+      </x:c>
+      <x:c r="C91" s="26" t="str">
+        <x:v>Lists managed policies attached to CloudVaultEC2Role.</x:v>
+      </x:c>
+      <x:c r="D91" s="26" t="str">
+        <x:v>Use to confirm CloudVaultS3DocumentAccess is attached at the end of Phase 1.</x:v>
+      </x:c>
+      <x:c r="E91" s="26" t="str">
+        <x:v>Output contains a policy ARN with the AWS account ID; sanitize public screenshots.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" s="26" t="str">
+        <x:v>aws iam list-role-policies --role-name CloudVaultEC2Role --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B92" s="26" t="str">
+        <x:v>IAM / Final Validation</x:v>
+      </x:c>
+      <x:c r="C92" s="26" t="str">
+        <x:v>Lists inline policies embedded in CloudVaultEC2Role.</x:v>
+      </x:c>
+      <x:c r="D92" s="26" t="str">
+        <x:v>Use to confirm there are no unexpected inline permissions.</x:v>
+      </x:c>
+      <x:c r="E92" s="26" t="str">
+        <x:v>Expected Phase 1 result: PolicyNames is empty.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" s="26" t="str">
+        <x:v>aws ce get-cost-and-usage --time-period $TimePeriod --granularity MONTHLY --metrics UnblendedCost --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B93" s="26" t="str">
+        <x:v>Cost Explorer / Validation</x:v>
+      </x:c>
+      <x:c r="C93" s="26" t="str">
+        <x:v>Returns the month-to-date unblended AWS cost for the requested time period.</x:v>
+      </x:c>
+      <x:c r="D93" s="26" t="str">
+        <x:v>Use during the final project cost review against the $10/month guardrail.</x:v>
+      </x:c>
+      <x:c r="E93" s="26" t="str">
+        <x:v>Current-period billing data can be estimated and may change before finalization.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" s="26" t="str">
+        <x:v>aws ce get-cost-and-usage --time-period $TimePeriod --granularity MONTHLY --metrics UnblendedCost --group-by Type=DIMENSION,Key=SERVICE --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B94" s="26" t="str">
+        <x:v>Cost Explorer / Validation</x:v>
+      </x:c>
+      <x:c r="C94" s="26" t="str">
+        <x:v>Breaks month-to-date unblended cost down by AWS service.</x:v>
+      </x:c>
+      <x:c r="D94" s="26" t="str">
+        <x:v>Use to identify which services contributed to project/account cost.</x:v>
+      </x:c>
+      <x:c r="E94" s="26" t="str">
+        <x:v>Phase 1 S3 usage was effectively $0 at the lab's tiny scale; current-period values are estimated.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2353,7 +2776,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62eb351df2524248"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19b013e8bd424d4a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3257,67 +3680,149 @@
       </x:c>
     </x:row>
     <x:row r="60" ht="15" hidden="0" customHeight="1">
-      <x:c r="A60" s="26"/>
+      <x:c r="A60" s="26" t="str">
+        <x:v>Additional PowerShell Commands — Phase 1 Metadata, Monitoring &amp; Cost Review</x:v>
+      </x:c>
       <x:c r="B60" s="26"/>
       <x:c r="C60" s="26"/>
       <x:c r="D60" s="26"/>
       <x:c r="E60" s="26"/>
     </x:row>
     <x:row r="61" ht="15" hidden="0" customHeight="1">
-      <x:c r="A61" s="26"/>
-      <x:c r="B61" s="26"/>
-      <x:c r="C61" s="26"/>
-      <x:c r="D61" s="26"/>
-      <x:c r="E61" s="26"/>
+      <x:c r="A61" s="26" t="str">
+        <x:v>Command</x:v>
+      </x:c>
+      <x:c r="B61" s="26" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="C61" s="26" t="str">
+        <x:v>What it does</x:v>
+      </x:c>
+      <x:c r="D61" s="26" t="str">
+        <x:v>When / Why to use it</x:v>
+      </x:c>
+      <x:c r="E61" s="26" t="str">
+        <x:v>Notes / Cautions</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="15" hidden="0" customHeight="1">
-      <x:c r="A62" s="26"/>
-      <x:c r="B62" s="26"/>
-      <x:c r="C62" s="26"/>
-      <x:c r="D62" s="26"/>
-      <x:c r="E62" s="26"/>
+      <x:c r="A62" s="26" t="str">
+        <x:v>Set-Content -Path .\test-data\metadata-test.txt -Value "CloudVault S3 object metadata test."</x:v>
+      </x:c>
+      <x:c r="B62" s="26" t="str">
+        <x:v>Test Data / S3</x:v>
+      </x:c>
+      <x:c r="C62" s="26" t="str">
+        <x:v>Creates the local text file used for the S3 metadata exercise.</x:v>
+      </x:c>
+      <x:c r="D62" s="26" t="str">
+        <x:v>Use before uploading the metadata-test object to S3.</x:v>
+      </x:c>
+      <x:c r="E62" s="26" t="str">
+        <x:v>test-data/ is ignored by Git and should remain local.</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="15" hidden="0" customHeight="1">
-      <x:c r="A63" s="26"/>
-      <x:c r="B63" s="26"/>
-      <x:c r="C63" s="26"/>
-      <x:c r="D63" s="26"/>
-      <x:c r="E63" s="26"/>
+      <x:c r="A63" s="26" t="str">
+        <x:v>$OldVersionId = aws s3api list-object-versions --bucket cloudvault-documents-dev01 --prefix documents/metadata-test.txt --query "Versions[?Key=='documents/metadata-test.txt' &amp;&amp; IsLatest==``false``].VersionId | [0]" --output text --profile cloudvault</x:v>
+      </x:c>
+      <x:c r="B63" s="26" t="str">
+        <x:v>Variables / AWS / JMESPath</x:v>
+      </x:c>
+      <x:c r="C63" s="26" t="str">
+        <x:v>Stores the first noncurrent metadata-test object version ID in a PowerShell variable.</x:v>
+      </x:c>
+      <x:c r="D63" s="26" t="str">
+        <x:v>Use to inspect historical metadata without manually copying a version ID.</x:v>
+      </x:c>
+      <x:c r="E63" s="26" t="str">
+        <x:v>PowerShell requires escaped backticks around the JMESPath false literal in this command; do not publish the resulting version ID.</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="15" hidden="0" customHeight="1">
-      <x:c r="A64" s="26"/>
-      <x:c r="B64" s="26"/>
-      <x:c r="C64" s="26"/>
-      <x:c r="D64" s="26"/>
-      <x:c r="E64" s="26"/>
+      <x:c r="A64" s="26" t="str">
+        <x:v>$StartTime = (Get-Date).ToUniversalTime().AddHours(-48).ToString("yyyy-MM-ddTHH:mm:ssZ")</x:v>
+      </x:c>
+      <x:c r="B64" s="26" t="str">
+        <x:v>Variables / Time</x:v>
+      </x:c>
+      <x:c r="C64" s="26" t="str">
+        <x:v>Creates a UTC timestamp 48 hours before the current time.</x:v>
+      </x:c>
+      <x:c r="D64" s="26" t="str">
+        <x:v>Use as a CloudWatch metric query start time.</x:v>
+      </x:c>
+      <x:c r="E64" s="26" t="str">
+        <x:v>CloudWatch S3 storage metrics are daily rather than real-time.</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" ht="15" hidden="0" customHeight="1">
-      <x:c r="A65" s="26"/>
-      <x:c r="B65" s="26"/>
-      <x:c r="C65" s="26"/>
-      <x:c r="D65" s="26"/>
-      <x:c r="E65" s="26"/>
+      <x:c r="A65" s="26" t="str">
+        <x:v>$EndTime = (Get-Date).ToUniversalTime().ToString("yyyy-MM-ddTHH:mm:ssZ")</x:v>
+      </x:c>
+      <x:c r="B65" s="26" t="str">
+        <x:v>Variables / Time</x:v>
+      </x:c>
+      <x:c r="C65" s="26" t="str">
+        <x:v>Creates a UTC timestamp for the current time.</x:v>
+      </x:c>
+      <x:c r="D65" s="26" t="str">
+        <x:v>Use as a CloudWatch metric query end time.</x:v>
+      </x:c>
+      <x:c r="E65" s="26" t="str">
+        <x:v>Pairs with $StartTime for a bounded metrics query.</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="15" hidden="0" customHeight="1">
-      <x:c r="A66" s="26"/>
-      <x:c r="B66" s="26"/>
-      <x:c r="C66" s="26"/>
-      <x:c r="D66" s="26"/>
-      <x:c r="E66" s="26"/>
+      <x:c r="A66" s="26" t="str">
+        <x:v>$StartDate = (Get-Date -Day 1).ToString("yyyy-MM-dd")</x:v>
+      </x:c>
+      <x:c r="B66" s="26" t="str">
+        <x:v>Variables / Cost Explorer</x:v>
+      </x:c>
+      <x:c r="C66" s="26" t="str">
+        <x:v>Stores the first day of the current month in AWS Cost Explorer date format.</x:v>
+      </x:c>
+      <x:c r="D66" s="26" t="str">
+        <x:v>Use when building a month-to-date Cost Explorer time period.</x:v>
+      </x:c>
+      <x:c r="E66" s="26" t="str">
+        <x:v>Cost Explorer expects yyyy-MM-dd dates.</x:v>
+      </x:c>
     </x:row>
     <x:row r="67" ht="15" hidden="0" customHeight="1">
-      <x:c r="A67" s="26"/>
-      <x:c r="B67" s="26"/>
-      <x:c r="C67" s="26"/>
-      <x:c r="D67" s="26"/>
-      <x:c r="E67" s="26"/>
+      <x:c r="A67" s="26" t="str">
+        <x:v>$EndDate = (Get-Date).AddDays(1).ToString("yyyy-MM-dd")</x:v>
+      </x:c>
+      <x:c r="B67" s="26" t="str">
+        <x:v>Variables / Cost Explorer</x:v>
+      </x:c>
+      <x:c r="C67" s="26" t="str">
+        <x:v>Stores tomorrow's date in AWS Cost Explorer date format.</x:v>
+      </x:c>
+      <x:c r="D67" s="26" t="str">
+        <x:v>Use as the exclusive end date for a month-to-date Cost Explorer query.</x:v>
+      </x:c>
+      <x:c r="E67" s="26" t="str">
+        <x:v>AWS time-period end dates are exclusive.</x:v>
+      </x:c>
     </x:row>
     <x:row r="68" ht="15" hidden="0" customHeight="1">
-      <x:c r="A68" s="26"/>
-      <x:c r="B68" s="26"/>
-      <x:c r="C68" s="26"/>
-      <x:c r="D68" s="26"/>
-      <x:c r="E68" s="26"/>
+      <x:c r="A68" s="26" t="str">
+        <x:v>$TimePeriod = "Start=$StartDate,End=$EndDate"</x:v>
+      </x:c>
+      <x:c r="B68" s="26" t="str">
+        <x:v>Variables / Cost Explorer</x:v>
+      </x:c>
+      <x:c r="C68" s="26" t="str">
+        <x:v>Builds the Cost Explorer shorthand time-period argument as one PowerShell string.</x:v>
+      </x:c>
+      <x:c r="D68" s="26" t="str">
+        <x:v>Use to avoid PowerShell parsing problems with the comma-separated Start/End shorthand.</x:v>
+      </x:c>
+      <x:c r="E68" s="26" t="str">
+        <x:v>Verify the variable prints as Start=yyyy-MM-dd,End=yyyy-MM-dd before using it.</x:v>
+      </x:c>
     </x:row>
     <x:row r="69" ht="15" hidden="0" customHeight="1">
       <x:c r="A69" s="26"/>
@@ -3482,7 +3987,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbda1694b99144895"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec23640550714bee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(phase-2): document EBS persistence and snapshot recovery
</commit_message>
<xml_diff>
--- a/docs/reference/CloudVault_Command_Notes.xlsx
+++ b/docs/reference/CloudVault_Command_Notes.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git" sheetId="1" r:id="R5fb0f65387df4b9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AWS" sheetId="2" r:id="R38542316415c4cee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PowerShell" sheetId="3" r:id="R63513dbf896047a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git" sheetId="1" r:id="R8beef72692674421"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AWS" sheetId="2" r:id="R886ec38c4a2d4054"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PowerShell" sheetId="3" r:id="Rb66771dc48b44370"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Linux (SSM)" sheetId="4" r:id="Rd0f9613a3de74618"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,7 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="6">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -49,8 +50,35 @@
       <x:color rgb="FF7F6000"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF15314C"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FFA12B22"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="15"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF234560"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -97,6 +125,26 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF163A5F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCE8F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F7FC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF1F8"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -105,7 +153,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="54">
+  <x:cellXfs count="76">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -209,6 +257,56 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -480,9 +578,9 @@
       <x:c r="D1" s="40"/>
       <x:c r="E1" s="40"/>
     </x:row>
-    <x:row r="2" ht="42" customHeight="1">
+    <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="12" t="str">
-        <x:v>Commands used while setting up the CloudVault repository, plus common commit-message standards.</x:v>
+        <x:v>CloudVault Git commands: repository setup, protected-branch workflow, and Phase 2 EBS documentation checkpoint.</x:v>
       </x:c>
       <x:c r="B2" s="12"/>
       <x:c r="C2" s="12"/>
@@ -1307,6 +1405,253 @@
       <x:c r="C59" s="26"/>
       <x:c r="D59" s="26"/>
       <x:c r="E59" s="26"/>
+    </x:row>
+    <x:row r="61" ht="28" customHeight="1">
+      <x:c r="A61" s="56" t="str">
+        <x:v>Phase 2 — EBS Documentation, Branch Review &amp; Pull Request</x:v>
+      </x:c>
+      <x:c r="B61" s="56"/>
+      <x:c r="C61" s="56"/>
+      <x:c r="D61" s="56"/>
+      <x:c r="E61" s="56"/>
+    </x:row>
+    <x:row r="62" ht="26" customHeight="1">
+      <x:c r="A62" s="60" t="str">
+        <x:v>Command</x:v>
+      </x:c>
+      <x:c r="B62" s="60" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="C62" s="60" t="str">
+        <x:v>What it does</x:v>
+      </x:c>
+      <x:c r="D62" s="60" t="str">
+        <x:v>When / Why to use it</x:v>
+      </x:c>
+      <x:c r="E62" s="60" t="str">
+        <x:v>Notes / Cautions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="45" customHeight="1">
+      <x:c r="A63" s="63" t="str">
+        <x:v>git fetch origin</x:v>
+      </x:c>
+      <x:c r="B63" s="63" t="str">
+        <x:v>Sync / Inspection</x:v>
+      </x:c>
+      <x:c r="C63" s="63" t="str">
+        <x:v>Update remote-tracking references without modifying local files.</x:v>
+      </x:c>
+      <x:c r="D63" s="63" t="str">
+        <x:v>Before creating a new documentation branch.</x:v>
+      </x:c>
+      <x:c r="E63" s="63" t="str">
+        <x:v>Fetch first, then check main against origin/main.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="45" customHeight="1">
+      <x:c r="A64" s="64" t="str">
+        <x:v>git pull --ff-only origin main</x:v>
+      </x:c>
+      <x:c r="B64" s="64" t="str">
+        <x:v>Sync / Safe Update</x:v>
+      </x:c>
+      <x:c r="C64" s="64" t="str">
+        <x:v>Fast-forward local main to origin/main without merge commits.</x:v>
+      </x:c>
+      <x:c r="D64" s="64" t="str">
+        <x:v>Use on main if it is behind the remote before branching.</x:v>
+      </x:c>
+      <x:c r="E64" s="64" t="str">
+        <x:v>Fails safely if histories diverged; do not force a merge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="45" customHeight="1">
+      <x:c r="A65" s="63" t="str">
+        <x:v>git switch -c docs/phase-2-ebs-lab</x:v>
+      </x:c>
+      <x:c r="B65" s="63" t="str">
+        <x:v>Branching</x:v>
+      </x:c>
+      <x:c r="C65" s="63" t="str">
+        <x:v>Create and switch to the Phase 2 EBS documentation branch.</x:v>
+      </x:c>
+      <x:c r="D65" s="63" t="str">
+        <x:v>Keep documentation work off protected main.</x:v>
+      </x:c>
+      <x:c r="E65" s="63" t="str">
+        <x:v>Verified feature branch used for this checkpoint.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="45" customHeight="1">
+      <x:c r="A66" s="64" t="str">
+        <x:v>git status --short --branch</x:v>
+      </x:c>
+      <x:c r="B66" s="64" t="str">
+        <x:v>Inspection</x:v>
+      </x:c>
+      <x:c r="C66" s="64" t="str">
+        <x:v>Show current branch and concise working-tree/staging status.</x:v>
+      </x:c>
+      <x:c r="D66" s="64" t="str">
+        <x:v>Before and after editing or staging documentation.</x:v>
+      </x:c>
+      <x:c r="E66" s="64" t="str">
+        <x:v> M means unstaged change; M  means staged change.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="45" customHeight="1">
+      <x:c r="A67" s="63" t="str">
+        <x:v>git branch --show-current</x:v>
+      </x:c>
+      <x:c r="B67" s="63" t="str">
+        <x:v>Inspection</x:v>
+      </x:c>
+      <x:c r="C67" s="63" t="str">
+        <x:v>Print the active local branch name.</x:v>
+      </x:c>
+      <x:c r="D67" s="63" t="str">
+        <x:v>Verify the intended feature branch before committing.</x:v>
+      </x:c>
+      <x:c r="E67" s="63" t="str">
+        <x:v>Expected: docs/phase-2-ebs-lab.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="45" customHeight="1">
+      <x:c r="A68" s="64" t="str">
+        <x:v>git log -1 --format="%h %s"</x:v>
+      </x:c>
+      <x:c r="B68" s="64" t="str">
+        <x:v>Inspection</x:v>
+      </x:c>
+      <x:c r="C68" s="64" t="str">
+        <x:v>Show the latest commit hash and subject.</x:v>
+      </x:c>
+      <x:c r="D68" s="64" t="str">
+        <x:v>Verify the starting main checkpoint.</x:v>
+      </x:c>
+      <x:c r="E68" s="64" t="str">
+        <x:v>Starting checkpoint for this lab: 858378c.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="45" customHeight="1">
+      <x:c r="A69" s="63" t="str">
+        <x:v>git diff --check</x:v>
+      </x:c>
+      <x:c r="B69" s="63" t="str">
+        <x:v>Validation</x:v>
+      </x:c>
+      <x:c r="C69" s="63" t="str">
+        <x:v>Check unstaged changes for whitespace errors.</x:v>
+      </x:c>
+      <x:c r="D69" s="63" t="str">
+        <x:v>After replacing documentation files.</x:v>
+      </x:c>
+      <x:c r="E69" s="63" t="str">
+        <x:v>LF/CRLF conversion warnings on Windows do not by themselves mean errors.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="45" customHeight="1">
+      <x:c r="A70" s="64" t="str">
+        <x:v>git diff --stat</x:v>
+      </x:c>
+      <x:c r="B70" s="64" t="str">
+        <x:v>Review</x:v>
+      </x:c>
+      <x:c r="C70" s="64" t="str">
+        <x:v>Summarize unstaged changes by file.</x:v>
+      </x:c>
+      <x:c r="D70" s="64" t="str">
+        <x:v>Confirm the expected README, diagram, and learning log changed.</x:v>
+      </x:c>
+      <x:c r="E70" s="64" t="str">
+        <x:v>Review actual diffs as needed before staging.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="60" customHeight="1">
+      <x:c r="A71" s="63" t="str">
+        <x:v>git add README.md docs/architecture/cloudvault-current-state.mmd docs/learning-log/phase-2-ec2.md docs/reference/CloudVault_Command_Notes.xlsx</x:v>
+      </x:c>
+      <x:c r="B71" s="63" t="str">
+        <x:v>Staging</x:v>
+      </x:c>
+      <x:c r="C71" s="63" t="str">
+        <x:v>Stage the four Phase 2 documentation/reference files.</x:v>
+      </x:c>
+      <x:c r="D71" s="63" t="str">
+        <x:v>After updating and validating the workbook in the repo.</x:v>
+      </x:c>
+      <x:c r="E71" s="63" t="str">
+        <x:v>Run from repository root; verify the workbook is copied to docs/reference first.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="45" customHeight="1">
+      <x:c r="A72" s="64" t="str">
+        <x:v>git diff --cached --check</x:v>
+      </x:c>
+      <x:c r="B72" s="64" t="str">
+        <x:v>Validation</x:v>
+      </x:c>
+      <x:c r="C72" s="64" t="str">
+        <x:v>Check staged changes for whitespace errors.</x:v>
+      </x:c>
+      <x:c r="D72" s="64" t="str">
+        <x:v>Immediately before committing.</x:v>
+      </x:c>
+      <x:c r="E72" s="64" t="str">
+        <x:v>The --cached flag inspects the staged index.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="45" customHeight="1">
+      <x:c r="A73" s="63" t="str">
+        <x:v>git diff --cached --stat</x:v>
+      </x:c>
+      <x:c r="B73" s="63" t="str">
+        <x:v>Review</x:v>
+      </x:c>
+      <x:c r="C73" s="63" t="str">
+        <x:v>Summarize staged changes by file.</x:v>
+      </x:c>
+      <x:c r="D73" s="63" t="str">
+        <x:v>Confirm the Commands workbook is included with the three documentation files.</x:v>
+      </x:c>
+      <x:c r="E73" s="63" t="str">
+        <x:v>Check git status --short --branch too.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="45" customHeight="1">
+      <x:c r="A74" s="64" t="str">
+        <x:v>git commit -m "docs(phase-2): document EBS persistence and snapshot recovery"</x:v>
+      </x:c>
+      <x:c r="B74" s="64" t="str">
+        <x:v>Commit / Planned</x:v>
+      </x:c>
+      <x:c r="C74" s="64" t="str">
+        <x:v>Commit the reviewed staged changes to the feature branch.</x:v>
+      </x:c>
+      <x:c r="D74" s="64" t="str">
+        <x:v>Only after all four files have been validated.</x:v>
+      </x:c>
+      <x:c r="E74" s="64" t="str">
+        <x:v>Planned next step; not yet executed at this checkpoint.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="45" customHeight="1">
+      <x:c r="A75" s="63" t="str">
+        <x:v>git push -u origin docs/phase-2-ebs-lab</x:v>
+      </x:c>
+      <x:c r="B75" s="63" t="str">
+        <x:v>Remote / Planned</x:v>
+      </x:c>
+      <x:c r="C75" s="63" t="str">
+        <x:v>Push the feature branch and set its upstream.</x:v>
+      </x:c>
+      <x:c r="D75" s="63" t="str">
+        <x:v>After committing, to open a GitHub pull request.</x:v>
+      </x:c>
+      <x:c r="E75" s="63" t="str">
+        <x:v>Planned next step; do not push directly to protected main.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1314,11 +1659,12 @@
     <x:mergeCell ref="A2:E2"/>
     <x:mergeCell ref="A28:E28"/>
     <x:mergeCell ref="A42:E42"/>
+    <x:mergeCell ref="A61:E61"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12418ee50f364b52"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a1216f84d124298"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcfe6e0a3160e4bc0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1070bbf9643f4ef0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1343,9 +1689,9 @@
       <x:c r="D1" s="40"/>
       <x:c r="E1" s="40"/>
     </x:row>
-    <x:row r="2" ht="15" hidden="0" customHeight="1">
+    <x:row r="2" ht="34" hidden="0" customHeight="1">
       <x:c r="A2" s="12" t="str">
-        <x:v>AWS CLI commands used across CloudVault Phase 0 and Phase 1: temporary authentication, identity verification, budgets, IAM, S3 storage, versioning, and least-privilege validation.</x:v>
+        <x:v>CloudVault Phase 0–2 AWS CLI reference: authentication, IAM, S3, EC2, Systems Manager, EBS volumes, snapshots, restoration, and cost control.</x:v>
       </x:c>
       <x:c r="B2" s="12"/>
       <x:c r="C2" s="12"/>
@@ -2762,6 +3108,517 @@
       </x:c>
       <x:c r="E94" s="26" t="str">
         <x:v>Phase 1 S3 usage was effectively $0 at the lab's tiny scale; current-period values are estimated.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="28" customHeight="1">
+      <x:c r="A96" s="56" t="str">
+        <x:v>Phase 2 — EC2 Foundation, Session Manager &amp; Lifecycle</x:v>
+      </x:c>
+      <x:c r="B96" s="56"/>
+      <x:c r="C96" s="56"/>
+      <x:c r="D96" s="56"/>
+      <x:c r="E96" s="56"/>
+    </x:row>
+    <x:row r="97" ht="26" customHeight="1">
+      <x:c r="A97" s="60" t="str">
+        <x:v>Command</x:v>
+      </x:c>
+      <x:c r="B97" s="60" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="C97" s="60" t="str">
+        <x:v>What it does</x:v>
+      </x:c>
+      <x:c r="D97" s="60" t="str">
+        <x:v>When / Why to use it</x:v>
+      </x:c>
+      <x:c r="E97" s="60" t="str">
+        <x:v>Notes / Cautions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="76" customHeight="1">
+      <x:c r="A98" s="63" t="str">
+        <x:v>aws ec2 describe-instances --instance-ids $InstanceId --query "Reservations[].Instances[].{InstanceId:InstanceId,State:State.Name,AZ:Placement.AvailabilityZone,Type:InstanceType}" --output json --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B98" s="63" t="str">
+        <x:v>EC2 / Inventory</x:v>
+      </x:c>
+      <x:c r="C98" s="63" t="str">
+        <x:v>Inspect instance identity, state, type, and Availability Zone.</x:v>
+      </x:c>
+      <x:c r="D98" s="63" t="str">
+        <x:v>Before attaching an EBS volume or starting a lab.</x:v>
+      </x:c>
+      <x:c r="E98" s="63" t="str">
+        <x:v>EBS volumes must be in the same Availability Zone as the EC2 instance.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="60" customHeight="1">
+      <x:c r="A99" s="64" t="str">
+        <x:v>aws ec2 describe-instances --instance-ids $InstanceId --query "Reservations[].Instances[].BlockDeviceMappings" --output json --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B99" s="64" t="str">
+        <x:v>EC2 / Storage</x:v>
+      </x:c>
+      <x:c r="C99" s="64" t="str">
+        <x:v>List the EBS volumes mapped to the instance.</x:v>
+      </x:c>
+      <x:c r="D99" s="64" t="str">
+        <x:v>Distinguish the root volume from the separate data volume.</x:v>
+      </x:c>
+      <x:c r="E99" s="64" t="str">
+        <x:v>Never format or delete the root volume.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="92" customHeight="1">
+      <x:c r="A100" s="63" t="str">
+        <x:v>aws ec2 describe-volumes --volume-ids $DataVolumeId --query "Volumes[].{VolumeId:VolumeId,State:State,Size:Size,Type:VolumeType,Encrypted:Encrypted,AZ:AvailabilityZone,Attachments:Attachments}" --output json --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B100" s="63" t="str">
+        <x:v>EBS / Inspection</x:v>
+      </x:c>
+      <x:c r="C100" s="63" t="str">
+        <x:v>Inspect size, encryption, AZ, state, and attachment information.</x:v>
+      </x:c>
+      <x:c r="D100" s="63" t="str">
+        <x:v>Before and after attaching a data volume.</x:v>
+      </x:c>
+      <x:c r="E100" s="63" t="str">
+        <x:v>Use the exact verified volume ID, not a guessed device name.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="60" customHeight="1">
+      <x:c r="A101" s="64" t="str">
+        <x:v>aws ssm describe-instance-information --filters Key=InstanceIds,Values=$InstanceId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B101" s="64" t="str">
+        <x:v>SSM / Inspection</x:v>
+      </x:c>
+      <x:c r="C101" s="64" t="str">
+        <x:v>Check the instance registration and Session Manager connectivity status.</x:v>
+      </x:c>
+      <x:c r="D101" s="64" t="str">
+        <x:v>Troubleshoot access after an EC2 start.</x:v>
+      </x:c>
+      <x:c r="E101" s="64" t="str">
+        <x:v>The SSM agent needs the instance role and connectivity to Systems Manager endpoints.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="45" customHeight="1">
+      <x:c r="A102" s="63" t="str">
+        <x:v>aws ssm start-session --target $InstanceId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B102" s="63" t="str">
+        <x:v>SSM / Access</x:v>
+      </x:c>
+      <x:c r="C102" s="63" t="str">
+        <x:v>Open a shell on the instance through Systems Manager.</x:v>
+      </x:c>
+      <x:c r="D102" s="63" t="str">
+        <x:v>Perform Linux EBS filesystem commands without SSH.</x:v>
+      </x:c>
+      <x:c r="E102" s="63" t="str">
+        <x:v>Requires Session Manager plugin on Windows; do not open inbound port 22.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="45" customHeight="1">
+      <x:c r="A103" s="64" t="str">
+        <x:v>aws ec2 stop-instances --instance-ids $InstanceId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B103" s="64" t="str">
+        <x:v>EC2 / Cost Control</x:v>
+      </x:c>
+      <x:c r="C103" s="64" t="str">
+        <x:v>Request a normal stop of the instance.</x:v>
+      </x:c>
+      <x:c r="D103" s="64" t="str">
+        <x:v>At the end of the hands-on lab to stop compute charges.</x:v>
+      </x:c>
+      <x:c r="E103" s="64" t="str">
+        <x:v>EBS storage is still billed; do not use force-stop unless troubleshooting requires it.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="45" customHeight="1">
+      <x:c r="A104" s="63" t="str">
+        <x:v>aws ec2 wait instance-stopped --instance-ids $InstanceId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B104" s="63" t="str">
+        <x:v>EC2 / Wait</x:v>
+      </x:c>
+      <x:c r="C104" s="63" t="str">
+        <x:v>Wait until the instance has fully stopped.</x:v>
+      </x:c>
+      <x:c r="D104" s="63" t="str">
+        <x:v>Verify a safe stopping checkpoint before leaving the lab.</x:v>
+      </x:c>
+      <x:c r="E104" s="63" t="str">
+        <x:v>Successful waiter is silent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="45" customHeight="1">
+      <x:c r="A105" s="64" t="str">
+        <x:v>aws ec2 start-instances --instance-ids $InstanceId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B105" s="64" t="str">
+        <x:v>EC2 / Lifecycle</x:v>
+      </x:c>
+      <x:c r="C105" s="64" t="str">
+        <x:v>Start the same existing instance.</x:v>
+      </x:c>
+      <x:c r="D105" s="64" t="str">
+        <x:v>Verify data survives a stop/start cycle.</x:v>
+      </x:c>
+      <x:c r="E105" s="64" t="str">
+        <x:v>Public IPv4 may change; EBS volumes persist.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="45" customHeight="1">
+      <x:c r="A106" s="63" t="str">
+        <x:v>aws ec2 wait instance-running --instance-ids $InstanceId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B106" s="63" t="str">
+        <x:v>EC2 / Wait</x:v>
+      </x:c>
+      <x:c r="C106" s="63" t="str">
+        <x:v>Wait for the instance to reach running state.</x:v>
+      </x:c>
+      <x:c r="D106" s="63" t="str">
+        <x:v>Before reconnecting via Session Manager.</x:v>
+      </x:c>
+      <x:c r="E106" s="63" t="str">
+        <x:v>SSM connectivity may take longer than the EC2 running state.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="92" customHeight="1">
+      <x:c r="A107" s="64" t="str">
+        <x:v>aws ec2 describe-instances --instance-ids $InstanceId --query "Reservations[].Instances[].{InstanceId:InstanceId,State:State.Name,InstanceType:InstanceType,Volumes:BlockDeviceMappings[].Ebs.VolumeId}" --output json --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B107" s="64" t="str">
+        <x:v>EC2 / Final Verification</x:v>
+      </x:c>
+      <x:c r="C107" s="64" t="str">
+        <x:v>Confirm final EC2 state and attached EBS volume IDs.</x:v>
+      </x:c>
+      <x:c r="D107" s="64" t="str">
+        <x:v>Verify the instance is stopped and the original root/data volumes remain.</x:v>
+      </x:c>
+      <x:c r="E107" s="64" t="str">
+        <x:v>Verified end state: stopped t3.micro with an 8 GiB root and 1 GiB data volume.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="28" customHeight="1">
+      <x:c r="A109" s="56" t="str">
+        <x:v>Phase 2 — EBS Provisioning, Snapshot, Recovery &amp; Cleanup</x:v>
+      </x:c>
+      <x:c r="B109" s="56"/>
+      <x:c r="C109" s="56"/>
+      <x:c r="D109" s="56"/>
+      <x:c r="E109" s="56"/>
+    </x:row>
+    <x:row r="110" ht="26" customHeight="1">
+      <x:c r="A110" s="60" t="str">
+        <x:v>Command</x:v>
+      </x:c>
+      <x:c r="B110" s="60" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="C110" s="60" t="str">
+        <x:v>What it does</x:v>
+      </x:c>
+      <x:c r="D110" s="60" t="str">
+        <x:v>When / Why to use it</x:v>
+      </x:c>
+      <x:c r="E110" s="60" t="str">
+        <x:v>Notes / Cautions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="76" customHeight="1">
+      <x:c r="A111" s="63" t="str">
+        <x:v>aws ec2 create-volume --availability-zone ap-southeast-1a --size 1 --volume-type gp3 --encrypted --tag-specifications 'ResourceType=volume,Tags=[{Key=Name,Value=CloudVaultEBSDataDev01}]' --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B111" s="63" t="str">
+        <x:v>EBS / Provisioning</x:v>
+      </x:c>
+      <x:c r="C111" s="63" t="str">
+        <x:v>Create a 1 GiB encrypted gp3 data volume in the EC2 Availability Zone.</x:v>
+      </x:c>
+      <x:c r="D111" s="63" t="str">
+        <x:v>Begin the separate EBS data-volume lab.</x:v>
+      </x:c>
+      <x:c r="E111" s="63" t="str">
+        <x:v>Creating a volume incurs storage cost. Verify the AZ before running; the Name tag is illustrative.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="45" customHeight="1">
+      <x:c r="A112" s="64" t="str">
+        <x:v>aws ec2 wait volume-available --volume-ids $DataVolumeId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B112" s="64" t="str">
+        <x:v>EBS / Wait</x:v>
+      </x:c>
+      <x:c r="C112" s="64" t="str">
+        <x:v>Wait for the newly created volume to be available.</x:v>
+      </x:c>
+      <x:c r="D112" s="64" t="str">
+        <x:v>Before attaching the data volume to EC2.</x:v>
+      </x:c>
+      <x:c r="E112" s="64" t="str">
+        <x:v>Successful waiter is silent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="60" customHeight="1">
+      <x:c r="A113" s="63" t="str">
+        <x:v>aws ec2 attach-volume --volume-id $DataVolumeId --instance-id $InstanceId --device /dev/sdf --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B113" s="63" t="str">
+        <x:v>EBS / Attachment</x:v>
+      </x:c>
+      <x:c r="C113" s="63" t="str">
+        <x:v>Attach the original data volume to the instance.</x:v>
+      </x:c>
+      <x:c r="D113" s="63" t="str">
+        <x:v>Prepare the blank volume for filesystem creation.</x:v>
+      </x:c>
+      <x:c r="E113" s="63" t="str">
+        <x:v>On Nitro instances, the actual Linux name can be /dev/nvme1n1 or another NVMe path; verify SERIAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="45" customHeight="1">
+      <x:c r="A114" s="64" t="str">
+        <x:v>aws ec2 wait volume-in-use --volume-ids $DataVolumeId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B114" s="64" t="str">
+        <x:v>EBS / Wait</x:v>
+      </x:c>
+      <x:c r="C114" s="64" t="str">
+        <x:v>Wait until AWS reports the data volume is attached/in use.</x:v>
+      </x:c>
+      <x:c r="D114" s="64" t="str">
+        <x:v>Before inspecting it inside the Linux instance.</x:v>
+      </x:c>
+      <x:c r="E114" s="64" t="str">
+        <x:v>Do not format until device serial, size, and existing signatures are verified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="60" customHeight="1">
+      <x:c r="A115" s="63" t="str">
+        <x:v>aws ec2 create-snapshot --volume-id $DataVolumeId --description "CloudVault EBS data recovery lab" --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B115" s="63" t="str">
+        <x:v>EBS / Snapshot</x:v>
+      </x:c>
+      <x:c r="C115" s="63" t="str">
+        <x:v>Create a point-in-time EBS snapshot of the original data volume.</x:v>
+      </x:c>
+      <x:c r="D115" s="63" t="str">
+        <x:v>After writing test data and calling sync in Linux.</x:v>
+      </x:c>
+      <x:c r="E115" s="63" t="str">
+        <x:v>Snapshot storage can incur charges; volume remains attached and usable.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="45" customHeight="1">
+      <x:c r="A116" s="64" t="str">
+        <x:v>aws ec2 wait snapshot-completed --snapshot-ids $SnapshotId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B116" s="64" t="str">
+        <x:v>EBS / Wait</x:v>
+      </x:c>
+      <x:c r="C116" s="64" t="str">
+        <x:v>Wait for the snapshot to complete.</x:v>
+      </x:c>
+      <x:c r="D116" s="64" t="str">
+        <x:v>Before creating a restored EBS volume from it.</x:v>
+      </x:c>
+      <x:c r="E116" s="64" t="str">
+        <x:v>Successful waiter is silent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="76" customHeight="1">
+      <x:c r="A117" s="63" t="str">
+        <x:v>aws ec2 describe-snapshots --snapshot-ids $SnapshotId --query "Snapshots[].{SnapshotId:SnapshotId,State:State,Progress:Progress,Encrypted:Encrypted,VolumeId:VolumeId}" --output json --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B117" s="63" t="str">
+        <x:v>EBS / Snapshot Verification</x:v>
+      </x:c>
+      <x:c r="C117" s="63" t="str">
+        <x:v>Verify snapshot status, progress, encryption, and source volume.</x:v>
+      </x:c>
+      <x:c r="D117" s="63" t="str">
+        <x:v>Confirm completed 100% before restoration.</x:v>
+      </x:c>
+      <x:c r="E117" s="63" t="str">
+        <x:v>Snapshot is a backup of EBS blocks, not a mounted filesystem.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="92" customHeight="1">
+      <x:c r="A118" s="64" t="str">
+        <x:v>aws ec2 create-volume --availability-zone ap-southeast-1a --snapshot-id $SnapshotId --volume-type gp3 --encrypted --tag-specifications 'ResourceType=volume,Tags=[{Key=Name,Value=CloudVaultEBSRestoredDev01}]' --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B118" s="64" t="str">
+        <x:v>EBS / Recovery</x:v>
+      </x:c>
+      <x:c r="C118" s="64" t="str">
+        <x:v>Restore the snapshot to a separate encrypted gp3 volume.</x:v>
+      </x:c>
+      <x:c r="D118" s="64" t="str">
+        <x:v>Test recovery without changing the original volume.</x:v>
+      </x:c>
+      <x:c r="E118" s="64" t="str">
+        <x:v>Use the EC2 instance AZ; the restored XFS filesystem initially shares the original UUID.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="45" customHeight="1">
+      <x:c r="A119" s="63" t="str">
+        <x:v>aws ec2 wait volume-available --volume-ids $RestoredVolumeId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B119" s="63" t="str">
+        <x:v>EBS / Wait</x:v>
+      </x:c>
+      <x:c r="C119" s="63" t="str">
+        <x:v>Wait until the restored volume is available.</x:v>
+      </x:c>
+      <x:c r="D119" s="63" t="str">
+        <x:v>Before attaching the restored volume.</x:v>
+      </x:c>
+      <x:c r="E119" s="63" t="str">
+        <x:v>Successful waiter is silent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="60" customHeight="1">
+      <x:c r="A120" s="64" t="str">
+        <x:v>aws ec2 attach-volume --volume-id $RestoredVolumeId --instance-id $InstanceId --device /dev/sdg --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B120" s="64" t="str">
+        <x:v>EBS / Recovery Attachment</x:v>
+      </x:c>
+      <x:c r="C120" s="64" t="str">
+        <x:v>Attach the restored EBS volume alongside the original.</x:v>
+      </x:c>
+      <x:c r="D120" s="64" t="str">
+        <x:v>Compare recovered test data against the source.</x:v>
+      </x:c>
+      <x:c r="E120" s="64" t="str">
+        <x:v>Confirm the new Linux NVMe serial before mounting; do not format the restored volume.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="76" customHeight="1">
+      <x:c r="A121" s="63" t="str">
+        <x:v>aws ec2 describe-volumes --volume-ids $RestoredVolumeId --query "Volumes[].{VolumeId:VolumeId,State:State,Attachments:Attachments}" --output json --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B121" s="63" t="str">
+        <x:v>EBS / Recovery Verification</x:v>
+      </x:c>
+      <x:c r="C121" s="63" t="str">
+        <x:v>Check the restored volume state and attachment.</x:v>
+      </x:c>
+      <x:c r="D121" s="63" t="str">
+        <x:v>Before or after read-only restore validation.</x:v>
+      </x:c>
+      <x:c r="E121" s="63" t="str">
+        <x:v>The restored volume must be unmounted before detachment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="45" customHeight="1">
+      <x:c r="A122" s="64" t="str">
+        <x:v>aws ec2 detach-volume --volume-id $RestoredVolumeId --instance-id $InstanceId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B122" s="64" t="str">
+        <x:v>EBS / Cleanup</x:v>
+      </x:c>
+      <x:c r="C122" s="64" t="str">
+        <x:v>Normally detach the temporary restored volume.</x:v>
+      </x:c>
+      <x:c r="D122" s="64" t="str">
+        <x:v>After sudo umount and verification inside Linux.</x:v>
+      </x:c>
+      <x:c r="E122" s="64" t="str">
+        <x:v>Avoid --force during normal cleanup; verify this is NOT the original data volume.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="45" customHeight="1">
+      <x:c r="A123" s="63" t="str">
+        <x:v>aws ec2 wait volume-available --volume-ids $RestoredVolumeId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B123" s="63" t="str">
+        <x:v>EBS / Cleanup Verification</x:v>
+      </x:c>
+      <x:c r="C123" s="63" t="str">
+        <x:v>Wait until the detached restored volume is available.</x:v>
+      </x:c>
+      <x:c r="D123" s="63" t="str">
+        <x:v>Before deleting the temporary restored volume.</x:v>
+      </x:c>
+      <x:c r="E123" s="63" t="str">
+        <x:v>Successful waiter is silent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="45" customHeight="1">
+      <x:c r="A124" s="64" t="str">
+        <x:v>aws ec2 delete-volume --volume-id $RestoredVolumeId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B124" s="65" t="str">
+        <x:v>EBS / Cleanup — Destructive</x:v>
+      </x:c>
+      <x:c r="C124" s="64" t="str">
+        <x:v>Permanently delete the temporary restored EBS volume.</x:v>
+      </x:c>
+      <x:c r="D124" s="64" t="str">
+        <x:v>After successful data comparison and detachment.</x:v>
+      </x:c>
+      <x:c r="E124" s="64" t="str">
+        <x:v>IRREVERSIBLE. Never substitute $DataVolumeId or the root volume ID.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="45" customHeight="1">
+      <x:c r="A125" s="63" t="str">
+        <x:v>aws ec2 describe-volumes --volume-ids $RestoredVolumeId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B125" s="63" t="str">
+        <x:v>EBS / Cleanup Verification</x:v>
+      </x:c>
+      <x:c r="C125" s="63" t="str">
+        <x:v>Check whether the deleted restored volume still exists.</x:v>
+      </x:c>
+      <x:c r="D125" s="63" t="str">
+        <x:v>Confirm successful deletion.</x:v>
+      </x:c>
+      <x:c r="E125" s="63" t="str">
+        <x:v>InvalidVolume.NotFound is the expected result after deletion.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="45" customHeight="1">
+      <x:c r="A126" s="64" t="str">
+        <x:v>aws ec2 delete-snapshot --snapshot-id $SnapshotId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B126" s="65" t="str">
+        <x:v>EBS / Cleanup — Destructive</x:v>
+      </x:c>
+      <x:c r="C126" s="64" t="str">
+        <x:v>Permanently delete the temporary recovery snapshot.</x:v>
+      </x:c>
+      <x:c r="D126" s="64" t="str">
+        <x:v>After restoring and verifying data and deleting the restored volume.</x:v>
+      </x:c>
+      <x:c r="E126" s="64" t="str">
+        <x:v>IRREVERSIBLE. Deleting a snapshot removes this recovery point; original EBS remains.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127" ht="45" customHeight="1">
+      <x:c r="A127" s="63" t="str">
+        <x:v>aws ec2 describe-snapshots --snapshot-ids $SnapshotId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B127" s="63" t="str">
+        <x:v>EBS / Cleanup Verification</x:v>
+      </x:c>
+      <x:c r="C127" s="63" t="str">
+        <x:v>Check whether the deleted snapshot still exists.</x:v>
+      </x:c>
+      <x:c r="D127" s="63" t="str">
+        <x:v>Confirm successful snapshot cleanup.</x:v>
+      </x:c>
+      <x:c r="E127" s="63" t="str">
+        <x:v>InvalidSnapshot.NotFound is the expected result after deletion.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2773,10 +3630,12 @@
     <x:mergeCell ref="A27:E27"/>
     <x:mergeCell ref="A29:E29"/>
     <x:mergeCell ref="A35:E35"/>
+    <x:mergeCell ref="A96:E96"/>
+    <x:mergeCell ref="A109:E109"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19b013e8bd424d4a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7b2ee5fd39b4d0e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2801,9 +3660,9 @@
       <x:c r="D1" s="40"/>
       <x:c r="E1" s="40"/>
     </x:row>
-    <x:row r="2" ht="15" hidden="0" customHeight="1">
+    <x:row r="2" ht="34" hidden="0" customHeight="1">
       <x:c r="A2" s="12" t="str">
-        <x:v>PowerShell and Windows shell commands used while installing/troubleshooting AWS CLI and Git and managing the CloudVault project.</x:v>
+        <x:v>Windows PowerShell reference for CloudVault setup, validation, Phase 2 EBS resource variables, and documentation.</x:v>
       </x:c>
       <x:c r="B2" s="12"/>
       <x:c r="C2" s="12"/>
@@ -3831,75 +4690,167 @@
       <x:c r="D69" s="26"/>
       <x:c r="E69" s="26"/>
     </x:row>
-    <x:row r="70" ht="15" hidden="0" customHeight="1">
-      <x:c r="A70" s="26"/>
-      <x:c r="B70" s="26"/>
-      <x:c r="C70" s="26"/>
-      <x:c r="D70" s="26"/>
-      <x:c r="E70" s="26"/>
-    </x:row>
-    <x:row r="71" ht="15" hidden="0" customHeight="1">
-      <x:c r="A71" s="26"/>
-      <x:c r="B71" s="26"/>
-      <x:c r="C71" s="26"/>
-      <x:c r="D71" s="26"/>
-      <x:c r="E71" s="26"/>
-    </x:row>
-    <x:row r="72" ht="15" hidden="0" customHeight="1">
-      <x:c r="A72" s="26"/>
-      <x:c r="B72" s="26"/>
-      <x:c r="C72" s="26"/>
-      <x:c r="D72" s="26"/>
-      <x:c r="E72" s="26"/>
-    </x:row>
-    <x:row r="73" ht="15" hidden="0" customHeight="1">
-      <x:c r="A73" s="26"/>
-      <x:c r="B73" s="26"/>
-      <x:c r="C73" s="26"/>
-      <x:c r="D73" s="26"/>
-      <x:c r="E73" s="26"/>
-    </x:row>
-    <x:row r="74" ht="15" hidden="0" customHeight="1">
-      <x:c r="A74" s="26"/>
-      <x:c r="B74" s="26"/>
-      <x:c r="C74" s="26"/>
-      <x:c r="D74" s="26"/>
-      <x:c r="E74" s="26"/>
-    </x:row>
-    <x:row r="75" ht="15" hidden="0" customHeight="1">
-      <x:c r="A75" s="26"/>
-      <x:c r="B75" s="26"/>
-      <x:c r="C75" s="26"/>
-      <x:c r="D75" s="26"/>
-      <x:c r="E75" s="26"/>
-    </x:row>
-    <x:row r="76" ht="15" hidden="0" customHeight="1">
-      <x:c r="A76" s="26"/>
-      <x:c r="B76" s="26"/>
-      <x:c r="C76" s="26"/>
-      <x:c r="D76" s="26"/>
-      <x:c r="E76" s="26"/>
-    </x:row>
-    <x:row r="77" ht="15" hidden="0" customHeight="1">
-      <x:c r="A77" s="26"/>
-      <x:c r="B77" s="26"/>
-      <x:c r="C77" s="26"/>
-      <x:c r="D77" s="26"/>
-      <x:c r="E77" s="26"/>
-    </x:row>
-    <x:row r="78" ht="15" hidden="0" customHeight="1">
-      <x:c r="A78" s="26"/>
-      <x:c r="B78" s="26"/>
-      <x:c r="C78" s="26"/>
-      <x:c r="D78" s="26"/>
-      <x:c r="E78" s="26"/>
-    </x:row>
-    <x:row r="79" ht="15" hidden="0" customHeight="1">
-      <x:c r="A79" s="26"/>
-      <x:c r="B79" s="26"/>
-      <x:c r="C79" s="26"/>
-      <x:c r="D79" s="26"/>
-      <x:c r="E79" s="26"/>
+    <x:row r="70" ht="28" hidden="0" customHeight="1">
+      <x:c r="A70" s="68" t="str">
+        <x:v>Phase 2 — EBS Variables &amp; Documentation Inspection</x:v>
+      </x:c>
+      <x:c r="B70" s="68"/>
+      <x:c r="C70" s="68"/>
+      <x:c r="D70" s="68"/>
+      <x:c r="E70" s="68"/>
+    </x:row>
+    <x:row r="71" ht="26" hidden="0" customHeight="1">
+      <x:c r="A71" s="60" t="str">
+        <x:v>Command</x:v>
+      </x:c>
+      <x:c r="B71" s="60" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="C71" s="60" t="str">
+        <x:v>What it does</x:v>
+      </x:c>
+      <x:c r="D71" s="60" t="str">
+        <x:v>When / Why to use it</x:v>
+      </x:c>
+      <x:c r="E71" s="60" t="str">
+        <x:v>Notes / Cautions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="45" hidden="0" customHeight="1">
+      <x:c r="A72" s="63" t="str">
+        <x:v>$InstanceId = "REPLACE_WITH_VERIFIED_INSTANCE_ID"</x:v>
+      </x:c>
+      <x:c r="B72" s="63" t="str">
+        <x:v>Variables / EC2</x:v>
+      </x:c>
+      <x:c r="C72" s="63" t="str">
+        <x:v>Store the verified EC2 instance ID in the current PowerShell session.</x:v>
+      </x:c>
+      <x:c r="D72" s="63" t="str">
+        <x:v>Before EC2 and SSM commands that use $InstanceId.</x:v>
+      </x:c>
+      <x:c r="E72" s="63" t="str">
+        <x:v>Variables do not persist across new terminal sessions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="45" hidden="0" customHeight="1">
+      <x:c r="A73" s="64" t="str">
+        <x:v>$DataVolumeId = "REPLACE_WITH_ORIGINAL_DATA_VOLUME_ID"</x:v>
+      </x:c>
+      <x:c r="B73" s="64" t="str">
+        <x:v>Variables / EBS</x:v>
+      </x:c>
+      <x:c r="C73" s="64" t="str">
+        <x:v>Store the original data volume ID.</x:v>
+      </x:c>
+      <x:c r="D73" s="64" t="str">
+        <x:v>Before creating snapshots or inspecting the original disk.</x:v>
+      </x:c>
+      <x:c r="E73" s="64" t="str">
+        <x:v>NEVER confuse the original data volume with the disposable restored volume.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="45" hidden="0" customHeight="1">
+      <x:c r="A74" s="63" t="str">
+        <x:v>$SnapshotId = "REPLACE_WITH_SNAPSHOT_ID"</x:v>
+      </x:c>
+      <x:c r="B74" s="63" t="str">
+        <x:v>Variables / EBS</x:v>
+      </x:c>
+      <x:c r="C74" s="63" t="str">
+        <x:v>Store the temporary EBS snapshot ID.</x:v>
+      </x:c>
+      <x:c r="D74" s="63" t="str">
+        <x:v>Before snapshot status, restore, and cleanup commands.</x:v>
+      </x:c>
+      <x:c r="E74" s="63" t="str">
+        <x:v>The snapshot was deleted at the end of the lab.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="45" hidden="0" customHeight="1">
+      <x:c r="A75" s="64" t="str">
+        <x:v>$RestoredVolumeId = "REPLACE_WITH_RESTORED_VOLUME_ID"</x:v>
+      </x:c>
+      <x:c r="B75" s="64" t="str">
+        <x:v>Variables / EBS</x:v>
+      </x:c>
+      <x:c r="C75" s="64" t="str">
+        <x:v>Store the temporary restored EBS volume ID.</x:v>
+      </x:c>
+      <x:c r="D75" s="64" t="str">
+        <x:v>Before inspecting, detaching, or deleting the restored volume.</x:v>
+      </x:c>
+      <x:c r="E75" s="64" t="str">
+        <x:v>The restored volume was deleted at the end of the lab.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="45" hidden="0" customHeight="1">
+      <x:c r="A76" s="63" t="str">
+        <x:v>Get-Content .\docs\learning-log\phase-2-ec2.md</x:v>
+      </x:c>
+      <x:c r="B76" s="63" t="str">
+        <x:v>Documentation / Inspection</x:v>
+      </x:c>
+      <x:c r="C76" s="63" t="str">
+        <x:v>Display the current Phase 2 learning log.</x:v>
+      </x:c>
+      <x:c r="D76" s="63" t="str">
+        <x:v>Before editing or verifying the EBS lab notes.</x:v>
+      </x:c>
+      <x:c r="E76" s="63" t="str">
+        <x:v>Run from the CloudVault repository root.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="45" hidden="0" customHeight="1">
+      <x:c r="A77" s="64" t="str">
+        <x:v>Get-Content .\docs\architecture\cloudvault-current-state.mmd</x:v>
+      </x:c>
+      <x:c r="B77" s="64" t="str">
+        <x:v>Documentation / Inspection</x:v>
+      </x:c>
+      <x:c r="C77" s="64" t="str">
+        <x:v>Display the current Mermaid architecture source.</x:v>
+      </x:c>
+      <x:c r="D77" s="64" t="str">
+        <x:v>Before updating the deployed-resource and recovery-workflow diagram.</x:v>
+      </x:c>
+      <x:c r="E77" s="64" t="str">
+        <x:v>A source-text check does not replace visual Mermaid rendering.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="45" hidden="0" customHeight="1">
+      <x:c r="A78" s="63" t="str">
+        <x:v>Get-Content .\README.md</x:v>
+      </x:c>
+      <x:c r="B78" s="63" t="str">
+        <x:v>Documentation / Inspection</x:v>
+      </x:c>
+      <x:c r="C78" s="63" t="str">
+        <x:v>Display the project README.</x:v>
+      </x:c>
+      <x:c r="D78" s="63" t="str">
+        <x:v>Before updating the Phase 2 progress and resource status.</x:v>
+      </x:c>
+      <x:c r="E78" s="63" t="str">
+        <x:v>Run from the repository root.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="45" hidden="0" customHeight="1">
+      <x:c r="A79" s="64" t="str">
+        <x:v>Copy-Item .\CloudVault_Command_Notes_Phase2_Updated.xlsx .\docs\reference\CloudVault_Command_Notes.xlsx</x:v>
+      </x:c>
+      <x:c r="B79" s="64" t="str">
+        <x:v>Documentation / Workbook</x:v>
+      </x:c>
+      <x:c r="C79" s="64" t="str">
+        <x:v>Copy the updated workbook into the tracked reference location.</x:v>
+      </x:c>
+      <x:c r="D79" s="64" t="str">
+        <x:v>After downloading this updated workbook into the repository root.</x:v>
+      </x:c>
+      <x:c r="E79" s="64" t="str">
+        <x:v>If the downloaded filename or location differs, adjust the source path; overwrites destination.</x:v>
+      </x:c>
     </x:row>
     <x:row r="80" ht="15" hidden="0" customHeight="1">
       <x:c r="A80" s="26"/>
@@ -3984,10 +4935,535 @@
     <x:mergeCell ref="A2:E2"/>
     <x:mergeCell ref="A27:E27"/>
     <x:mergeCell ref="A29:E29"/>
+    <x:mergeCell ref="A70:E70"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec23640550714bee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b49ef0ca5c843f2"/>
   </x:tableParts>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="55" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="42" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="43" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="46" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="71" t="str">
+        <x:v>Linux / SSM Command Reference</x:v>
+      </x:c>
+      <x:c r="B1" s="71"/>
+      <x:c r="C1" s="71"/>
+      <x:c r="D1" s="71"/>
+      <x:c r="E1" s="71"/>
+    </x:row>
+    <x:row r="2" ht="36" customHeight="1">
+      <x:c r="A2" s="75" t="str">
+        <x:v>CloudVault Phase 2 — commands run inside the Amazon Linux 2023 Session Manager shell. Verify NVMe serials before disk operations.</x:v>
+      </x:c>
+      <x:c r="B2" s="75"/>
+      <x:c r="C2" s="75"/>
+      <x:c r="D2" s="75"/>
+      <x:c r="E2" s="75"/>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="A4" s="56" t="str">
+        <x:v>Phase 2 — EC2 Linux Storage, Snapshot Validation &amp; S3 Tests</x:v>
+      </x:c>
+      <x:c r="B4" s="56"/>
+      <x:c r="C4" s="56"/>
+      <x:c r="D4" s="56"/>
+      <x:c r="E4" s="56"/>
+    </x:row>
+    <x:row r="5" ht="26" customHeight="1">
+      <x:c r="A5" s="60" t="str">
+        <x:v>Command</x:v>
+      </x:c>
+      <x:c r="B5" s="60" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="C5" s="60" t="str">
+        <x:v>What it does</x:v>
+      </x:c>
+      <x:c r="D5" s="60" t="str">
+        <x:v>When / Why to use it</x:v>
+      </x:c>
+      <x:c r="E5" s="60" t="str">
+        <x:v>Notes / Cautions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="45" customHeight="1">
+      <x:c r="A6" s="63" t="str">
+        <x:v>lsblk -o NAME,SIZE,TYPE,SERIAL,FSTYPE,MOUNTPOINTS</x:v>
+      </x:c>
+      <x:c r="B6" s="63" t="str">
+        <x:v>Device identification</x:v>
+      </x:c>
+      <x:c r="C6" s="63" t="str">
+        <x:v>List block devices, serials, filesystem types, and mounts.</x:v>
+      </x:c>
+      <x:c r="D6" s="63" t="str">
+        <x:v>Identify original and restored Nitro NVMe EBS devices before touching them.</x:v>
+      </x:c>
+      <x:c r="E6" s="63" t="str">
+        <x:v>Match the EBS volume ID to the NVMe SERIAL; device numbering can change.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="45" customHeight="1">
+      <x:c r="A7" s="64" t="str">
+        <x:v>sudo blkid /dev/nvme1n1</x:v>
+      </x:c>
+      <x:c r="B7" s="64" t="str">
+        <x:v>Filesystem inspection</x:v>
+      </x:c>
+      <x:c r="C7" s="64" t="str">
+        <x:v>Read filesystem UUID and type for the identified original data disk.</x:v>
+      </x:c>
+      <x:c r="D7" s="64" t="str">
+        <x:v>Before adding an /etc/fstab entry.</x:v>
+      </x:c>
+      <x:c r="E7" s="64" t="str">
+        <x:v>Example device path from this lab; verify the actual device first.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="45" customHeight="1">
+      <x:c r="A8" s="63" t="str">
+        <x:v>sudo wipefs -n /dev/nvme1n1</x:v>
+      </x:c>
+      <x:c r="B8" s="63" t="str">
+        <x:v>Non-destructive inspection</x:v>
+      </x:c>
+      <x:c r="C8" s="63" t="str">
+        <x:v>List filesystem signatures without erasing them.</x:v>
+      </x:c>
+      <x:c r="D8" s="63" t="str">
+        <x:v>Before formatting a newly attached blank disk.</x:v>
+      </x:c>
+      <x:c r="E8" s="63" t="str">
+        <x:v>The -n option is a dry run. Never use wipefs to clear an unverified disk.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="45" customHeight="1">
+      <x:c r="A9" s="64" t="str">
+        <x:v>sudo mkfs.xfs /dev/nvme1n1</x:v>
+      </x:c>
+      <x:c r="B9" s="65" t="str">
+        <x:v>Filesystem creation — DESTRUCTIVE</x:v>
+      </x:c>
+      <x:c r="C9" s="64" t="str">
+        <x:v>Create an XFS filesystem on the verified new blank data volume.</x:v>
+      </x:c>
+      <x:c r="D9" s="64" t="str">
+        <x:v>One-time initial provisioning of the original 1 GiB data volume.</x:v>
+      </x:c>
+      <x:c r="E9" s="64" t="str">
+        <x:v>IRREVERSIBLE if run on the wrong disk. Never run on /dev/nvme0n1 (root) or the restored disk.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="45" customHeight="1">
+      <x:c r="A10" s="63" t="str">
+        <x:v>sudo mkdir -p /data/cloudvault</x:v>
+      </x:c>
+      <x:c r="B10" s="63" t="str">
+        <x:v>Mount point</x:v>
+      </x:c>
+      <x:c r="C10" s="63" t="str">
+        <x:v>Create the persistent data-volume mount directory.</x:v>
+      </x:c>
+      <x:c r="D10" s="63" t="str">
+        <x:v>Before mounting the original data disk.</x:v>
+      </x:c>
+      <x:c r="E10" s="63" t="str">
+        <x:v>Directory creation is safe; filesystem mount is a separate step.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="45" customHeight="1">
+      <x:c r="A11" s="64" t="str">
+        <x:v>sudo mount /dev/nvme1n1 /data/cloudvault</x:v>
+      </x:c>
+      <x:c r="B11" s="64" t="str">
+        <x:v>Mount</x:v>
+      </x:c>
+      <x:c r="C11" s="64" t="str">
+        <x:v>Mount the original XFS data filesystem.</x:v>
+      </x:c>
+      <x:c r="D11" s="64" t="str">
+        <x:v>After confirming device identity and filesystem creation.</x:v>
+      </x:c>
+      <x:c r="E11" s="64" t="str">
+        <x:v>Example device name only; do not mount a random NVMe disk.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="45" customHeight="1">
+      <x:c r="A12" s="63" t="str">
+        <x:v>findmnt /data/cloudvault</x:v>
+      </x:c>
+      <x:c r="B12" s="63" t="str">
+        <x:v>Mount verification</x:v>
+      </x:c>
+      <x:c r="C12" s="63" t="str">
+        <x:v>Show the source device and mount options for the data directory.</x:v>
+      </x:c>
+      <x:c r="D12" s="63" t="str">
+        <x:v>Confirm the original data volume is mounted.</x:v>
+      </x:c>
+      <x:c r="E12" s="63" t="str">
+        <x:v>Check source, target, and filesystem type.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="45" customHeight="1">
+      <x:c r="A13" s="64" t="str">
+        <x:v>df -hT /data/cloudvault</x:v>
+      </x:c>
+      <x:c r="B13" s="64" t="str">
+        <x:v>Capacity verification</x:v>
+      </x:c>
+      <x:c r="C13" s="64" t="str">
+        <x:v>Show mounted filesystem type, size, used, and available space.</x:v>
+      </x:c>
+      <x:c r="D13" s="64" t="str">
+        <x:v>Confirm the expected 1 GiB XFS data volume.</x:v>
+      </x:c>
+      <x:c r="E13" s="64" t="str">
+        <x:v>Useful alongside findmnt and lsblk.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="45" customHeight="1">
+      <x:c r="A14" s="63" t="str">
+        <x:v>echo "CloudVault EBS storage test - Phase 2" | sudo tee /data/cloudvault/ebs-test.txt</x:v>
+      </x:c>
+      <x:c r="B14" s="63" t="str">
+        <x:v>Write test</x:v>
+      </x:c>
+      <x:c r="C14" s="63" t="str">
+        <x:v>Write a small known-content test file to EBS.</x:v>
+      </x:c>
+      <x:c r="D14" s="63" t="str">
+        <x:v>Verify persistence across stop/start and snapshot restore.</x:v>
+      </x:c>
+      <x:c r="E14" s="63" t="str">
+        <x:v>Only write after confirming /data/cloudvault is mounted to the intended volume.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="45" customHeight="1">
+      <x:c r="A15" s="64" t="str">
+        <x:v>cat /data/cloudvault/ebs-test.txt</x:v>
+      </x:c>
+      <x:c r="B15" s="64" t="str">
+        <x:v>Read test</x:v>
+      </x:c>
+      <x:c r="C15" s="64" t="str">
+        <x:v>Read the test file from the original EBS volume.</x:v>
+      </x:c>
+      <x:c r="D15" s="64" t="str">
+        <x:v>Confirm persistence after restarting EC2.</x:v>
+      </x:c>
+      <x:c r="E15" s="64" t="str">
+        <x:v>Expected: CloudVault EBS storage test - Phase 2.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="45" customHeight="1">
+      <x:c r="A16" s="63" t="str">
+        <x:v>sudo cp /etc/fstab /etc/fstab.cloudvault.bak</x:v>
+      </x:c>
+      <x:c r="B16" s="63" t="str">
+        <x:v>Configuration backup</x:v>
+      </x:c>
+      <x:c r="C16" s="63" t="str">
+        <x:v>Back up /etc/fstab before changing persistent mount settings.</x:v>
+      </x:c>
+      <x:c r="D16" s="63" t="str">
+        <x:v>Before adding the data-volume UUID entry.</x:v>
+      </x:c>
+      <x:c r="E16" s="63" t="str">
+        <x:v>A bad fstab entry can affect boot behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="45" customHeight="1">
+      <x:c r="A17" s="64" t="str">
+        <x:v>sudo blkid -s UUID -o value /dev/nvme1n1</x:v>
+      </x:c>
+      <x:c r="B17" s="64" t="str">
+        <x:v>UUID lookup</x:v>
+      </x:c>
+      <x:c r="C17" s="64" t="str">
+        <x:v>Print only the original XFS filesystem UUID.</x:v>
+      </x:c>
+      <x:c r="D17" s="64" t="str">
+        <x:v>Use stable UUID-based mounting rather than a changing NVMe path.</x:v>
+      </x:c>
+      <x:c r="E17" s="64" t="str">
+        <x:v>Verify the serial and device identity first.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="45" customHeight="1">
+      <x:c r="A18" s="63" t="str">
+        <x:v>printf 'UUID=&lt;VERIFIED_UUID&gt; /data/cloudvault xfs defaults,nofail 0 0\n' | sudo tee -a /etc/fstab</x:v>
+      </x:c>
+      <x:c r="B18" s="63" t="str">
+        <x:v>Persistent mount / Example</x:v>
+      </x:c>
+      <x:c r="C18" s="63" t="str">
+        <x:v>Append a UUID-based XFS mount entry to /etc/fstab.</x:v>
+      </x:c>
+      <x:c r="D18" s="63" t="str">
+        <x:v>One-time setup for persistent mounting.</x:v>
+      </x:c>
+      <x:c r="E18" s="63" t="str">
+        <x:v>Replace &lt;VERIFIED_UUID&gt; with actual UUID; do not add a duplicate entry; back up first.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="45" customHeight="1">
+      <x:c r="A19" s="64" t="str">
+        <x:v>sudo findmnt --verify --verbose</x:v>
+      </x:c>
+      <x:c r="B19" s="64" t="str">
+        <x:v>fstab validation</x:v>
+      </x:c>
+      <x:c r="C19" s="64" t="str">
+        <x:v>Validate /etc/fstab mount definitions.</x:v>
+      </x:c>
+      <x:c r="D19" s="64" t="str">
+        <x:v>Immediately after editing fstab and before restarting EC2.</x:v>
+      </x:c>
+      <x:c r="E19" s="64" t="str">
+        <x:v>Verified in lab: success, no errors or warnings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="45" customHeight="1">
+      <x:c r="A20" s="63" t="str">
+        <x:v>sudo mount -a</x:v>
+      </x:c>
+      <x:c r="B20" s="63" t="str">
+        <x:v>Mount validation</x:v>
+      </x:c>
+      <x:c r="C20" s="63" t="str">
+        <x:v>Attempt mounts configured in /etc/fstab.</x:v>
+      </x:c>
+      <x:c r="D20" s="63" t="str">
+        <x:v>Validate the data-volume entry without rebooting.</x:v>
+      </x:c>
+      <x:c r="E20" s="63" t="str">
+        <x:v>Check findmnt afterward; mount -a can affect other fstab entries.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="45" customHeight="1">
+      <x:c r="A21" s="64" t="str">
+        <x:v>sync</x:v>
+      </x:c>
+      <x:c r="B21" s="64" t="str">
+        <x:v>Snapshot preparation</x:v>
+      </x:c>
+      <x:c r="C21" s="64" t="str">
+        <x:v>Flush pending filesystem writes.</x:v>
+      </x:c>
+      <x:c r="D21" s="64" t="str">
+        <x:v>Immediately before requesting the EBS snapshot.</x:v>
+      </x:c>
+      <x:c r="E21" s="64" t="str">
+        <x:v>Improves consistency; application-consistent snapshots may need extra coordination.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="45" customHeight="1">
+      <x:c r="A22" s="63" t="str">
+        <x:v>sudo blkid /dev/nvme2n1</x:v>
+      </x:c>
+      <x:c r="B22" s="63" t="str">
+        <x:v>Restored disk inspection</x:v>
+      </x:c>
+      <x:c r="C22" s="63" t="str">
+        <x:v>Inspect filesystem UUID and type on the restored EBS volume.</x:v>
+      </x:c>
+      <x:c r="D22" s="63" t="str">
+        <x:v>Detect that the restored XFS filesystem duplicates the original UUID.</x:v>
+      </x:c>
+      <x:c r="E22" s="63" t="str">
+        <x:v>Example restored device; verify SERIAL before using it.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="45" customHeight="1">
+      <x:c r="A23" s="64" t="str">
+        <x:v>sudo mkdir -p /data/cloudvault-restored</x:v>
+      </x:c>
+      <x:c r="B23" s="64" t="str">
+        <x:v>Recovery mount point</x:v>
+      </x:c>
+      <x:c r="C23" s="64" t="str">
+        <x:v>Create a separate mount directory for the restored disk.</x:v>
+      </x:c>
+      <x:c r="D23" s="64" t="str">
+        <x:v>Before mounting the restored snapshot copy.</x:v>
+      </x:c>
+      <x:c r="E23" s="64" t="str">
+        <x:v>Keep original and restored volumes mounted at different directories.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="45" customHeight="1">
+      <x:c r="A24" s="63" t="str">
+        <x:v>sudo mount -t xfs -o ro,nouuid,norecovery /dev/nvme2n1 /data/cloudvault-restored</x:v>
+      </x:c>
+      <x:c r="B24" s="63" t="str">
+        <x:v>Safe XFS recovery mount</x:v>
+      </x:c>
+      <x:c r="C24" s="63" t="str">
+        <x:v>Mount the restored XFS filesystem read-only despite duplicate UUID.</x:v>
+      </x:c>
+      <x:c r="D24" s="63" t="str">
+        <x:v>Verify recovery while original XFS filesystem is mounted.</x:v>
+      </x:c>
+      <x:c r="E24" s="63" t="str">
+        <x:v>ro = read-only; nouuid permits duplicate UUID; norecovery avoids journal replay.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="45" customHeight="1">
+      <x:c r="A25" s="64" t="str">
+        <x:v>findmnt /data/cloudvault-restored</x:v>
+      </x:c>
+      <x:c r="B25" s="64" t="str">
+        <x:v>Recovery verification</x:v>
+      </x:c>
+      <x:c r="C25" s="64" t="str">
+        <x:v>Check restored filesystem mount and options.</x:v>
+      </x:c>
+      <x:c r="D25" s="64" t="str">
+        <x:v>Confirm the temporary recovery volume mounted successfully.</x:v>
+      </x:c>
+      <x:c r="E25" s="64" t="str">
+        <x:v>Verify read-only mount and the intended source device.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="45" customHeight="1">
+      <x:c r="A26" s="63" t="str">
+        <x:v>cmp /data/cloudvault/ebs-test.txt /data/cloudvault-restored/ebs-test.txt</x:v>
+      </x:c>
+      <x:c r="B26" s="63" t="str">
+        <x:v>Integrity verification</x:v>
+      </x:c>
+      <x:c r="C26" s="63" t="str">
+        <x:v>Compare original and restored file bytes.</x:v>
+      </x:c>
+      <x:c r="D26" s="63" t="str">
+        <x:v>Verify the snapshot successfully recovered the expected content.</x:v>
+      </x:c>
+      <x:c r="E26" s="63" t="str">
+        <x:v>No output and exit status 0 indicate identical files.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="45" customHeight="1">
+      <x:c r="A27" s="64" t="str">
+        <x:v>sudo umount /data/cloudvault-restored</x:v>
+      </x:c>
+      <x:c r="B27" s="64" t="str">
+        <x:v>Recovery cleanup</x:v>
+      </x:c>
+      <x:c r="C27" s="64" t="str">
+        <x:v>Unmount the temporary restored filesystem.</x:v>
+      </x:c>
+      <x:c r="D27" s="64" t="str">
+        <x:v>Before detaching its EBS volume in AWS.</x:v>
+      </x:c>
+      <x:c r="E27" s="64" t="str">
+        <x:v>Do not detach a mounted filesystem; original remains mounted.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="45" customHeight="1">
+      <x:c r="A28" s="63" t="str">
+        <x:v>findmnt /data/cloudvault-restored</x:v>
+      </x:c>
+      <x:c r="B28" s="63" t="str">
+        <x:v>Cleanup verification</x:v>
+      </x:c>
+      <x:c r="C28" s="63" t="str">
+        <x:v>Check whether the temporary restored mount is still present.</x:v>
+      </x:c>
+      <x:c r="D28" s="63" t="str">
+        <x:v>After unmounting and before detachment.</x:v>
+      </x:c>
+      <x:c r="E28" s="63" t="str">
+        <x:v>No output indicates no mount at that target.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="45" customHeight="1">
+      <x:c r="A29" s="64" t="str">
+        <x:v>aws sts get-caller-identity --query 'Arn' --output text | cut -d/ -f2</x:v>
+      </x:c>
+      <x:c r="B29" s="64" t="str">
+        <x:v>IAM role validation</x:v>
+      </x:c>
+      <x:c r="C29" s="64" t="str">
+        <x:v>Show the instance IAM role name without exposing the full account-specific ARN.</x:v>
+      </x:c>
+      <x:c r="D29" s="64" t="str">
+        <x:v>Verify the EC2 instance uses CloudVaultEC2Role temporary credentials.</x:v>
+      </x:c>
+      <x:c r="E29" s="64" t="str">
+        <x:v>Run inside EC2 SSM Linux shell; never print temporary secret credentials.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="45" customHeight="1">
+      <x:c r="A30" s="63" t="str">
+        <x:v>aws s3api list-objects-v2 --bucket cloudvault-documents-dev01 --prefix documents/</x:v>
+      </x:c>
+      <x:c r="B30" s="63" t="str">
+        <x:v>EC2-to-S3 allowed test</x:v>
+      </x:c>
+      <x:c r="C30" s="63" t="str">
+        <x:v>List objects under the IAM-authorized S3 prefix.</x:v>
+      </x:c>
+      <x:c r="D30" s="63" t="str">
+        <x:v>Validate instance role permissions in the EC2 runtime.</x:v>
+      </x:c>
+      <x:c r="E30" s="63" t="str">
+        <x:v>Expected success for documents/.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="45" customHeight="1">
+      <x:c r="A31" s="64" t="str">
+        <x:v>aws s3api list-objects-v2 --bucket cloudvault-documents-dev01 --prefix private/</x:v>
+      </x:c>
+      <x:c r="B31" s="64" t="str">
+        <x:v>EC2-to-S3 denied test</x:v>
+      </x:c>
+      <x:c r="C31" s="64" t="str">
+        <x:v>Attempt listing a prefix not authorized by the instance IAM policy.</x:v>
+      </x:c>
+      <x:c r="D31" s="64" t="str">
+        <x:v>Validate least-privilege enforcement from EC2.</x:v>
+      </x:c>
+      <x:c r="E31" s="64" t="str">
+        <x:v>Expected AccessDenied; do not broaden policy just to pass a negative test.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="45" customHeight="1">
+      <x:c r="A32" s="63" t="str">
+        <x:v>exit</x:v>
+      </x:c>
+      <x:c r="B32" s="63" t="str">
+        <x:v>Session Manager</x:v>
+      </x:c>
+      <x:c r="C32" s="63" t="str">
+        <x:v>Exit the interactive Linux shell.</x:v>
+      </x:c>
+      <x:c r="D32" s="63" t="str">
+        <x:v>After verifying mounts or before running Windows AWS CLI commands.</x:v>
+      </x:c>
+      <x:c r="E32" s="63" t="str">
+        <x:v>Returns to local PowerShell.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:E1"/>
+    <x:mergeCell ref="A2:E2"/>
+    <x:mergeCell ref="A4:E4"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(phase-2): document EBS persistence and snapshot recovery (#4)
</commit_message>
<xml_diff>
--- a/docs/reference/CloudVault_Command_Notes.xlsx
+++ b/docs/reference/CloudVault_Command_Notes.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git" sheetId="1" r:id="R5fb0f65387df4b9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AWS" sheetId="2" r:id="R38542316415c4cee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PowerShell" sheetId="3" r:id="R63513dbf896047a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git" sheetId="1" r:id="R8beef72692674421"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AWS" sheetId="2" r:id="R886ec38c4a2d4054"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PowerShell" sheetId="3" r:id="Rb66771dc48b44370"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Linux (SSM)" sheetId="4" r:id="Rd0f9613a3de74618"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,7 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="6">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -49,8 +50,35 @@
       <x:color rgb="FF7F6000"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF15314C"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FFA12B22"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="15"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF234560"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -97,6 +125,26 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF163A5F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCE8F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F7FC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF1F8"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -105,7 +153,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="54">
+  <x:cellXfs count="76">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -209,6 +257,56 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -480,9 +578,9 @@
       <x:c r="D1" s="40"/>
       <x:c r="E1" s="40"/>
     </x:row>
-    <x:row r="2" ht="42" customHeight="1">
+    <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="12" t="str">
-        <x:v>Commands used while setting up the CloudVault repository, plus common commit-message standards.</x:v>
+        <x:v>CloudVault Git commands: repository setup, protected-branch workflow, and Phase 2 EBS documentation checkpoint.</x:v>
       </x:c>
       <x:c r="B2" s="12"/>
       <x:c r="C2" s="12"/>
@@ -1307,6 +1405,253 @@
       <x:c r="C59" s="26"/>
       <x:c r="D59" s="26"/>
       <x:c r="E59" s="26"/>
+    </x:row>
+    <x:row r="61" ht="28" customHeight="1">
+      <x:c r="A61" s="56" t="str">
+        <x:v>Phase 2 — EBS Documentation, Branch Review &amp; Pull Request</x:v>
+      </x:c>
+      <x:c r="B61" s="56"/>
+      <x:c r="C61" s="56"/>
+      <x:c r="D61" s="56"/>
+      <x:c r="E61" s="56"/>
+    </x:row>
+    <x:row r="62" ht="26" customHeight="1">
+      <x:c r="A62" s="60" t="str">
+        <x:v>Command</x:v>
+      </x:c>
+      <x:c r="B62" s="60" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="C62" s="60" t="str">
+        <x:v>What it does</x:v>
+      </x:c>
+      <x:c r="D62" s="60" t="str">
+        <x:v>When / Why to use it</x:v>
+      </x:c>
+      <x:c r="E62" s="60" t="str">
+        <x:v>Notes / Cautions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="45" customHeight="1">
+      <x:c r="A63" s="63" t="str">
+        <x:v>git fetch origin</x:v>
+      </x:c>
+      <x:c r="B63" s="63" t="str">
+        <x:v>Sync / Inspection</x:v>
+      </x:c>
+      <x:c r="C63" s="63" t="str">
+        <x:v>Update remote-tracking references without modifying local files.</x:v>
+      </x:c>
+      <x:c r="D63" s="63" t="str">
+        <x:v>Before creating a new documentation branch.</x:v>
+      </x:c>
+      <x:c r="E63" s="63" t="str">
+        <x:v>Fetch first, then check main against origin/main.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="45" customHeight="1">
+      <x:c r="A64" s="64" t="str">
+        <x:v>git pull --ff-only origin main</x:v>
+      </x:c>
+      <x:c r="B64" s="64" t="str">
+        <x:v>Sync / Safe Update</x:v>
+      </x:c>
+      <x:c r="C64" s="64" t="str">
+        <x:v>Fast-forward local main to origin/main without merge commits.</x:v>
+      </x:c>
+      <x:c r="D64" s="64" t="str">
+        <x:v>Use on main if it is behind the remote before branching.</x:v>
+      </x:c>
+      <x:c r="E64" s="64" t="str">
+        <x:v>Fails safely if histories diverged; do not force a merge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="45" customHeight="1">
+      <x:c r="A65" s="63" t="str">
+        <x:v>git switch -c docs/phase-2-ebs-lab</x:v>
+      </x:c>
+      <x:c r="B65" s="63" t="str">
+        <x:v>Branching</x:v>
+      </x:c>
+      <x:c r="C65" s="63" t="str">
+        <x:v>Create and switch to the Phase 2 EBS documentation branch.</x:v>
+      </x:c>
+      <x:c r="D65" s="63" t="str">
+        <x:v>Keep documentation work off protected main.</x:v>
+      </x:c>
+      <x:c r="E65" s="63" t="str">
+        <x:v>Verified feature branch used for this checkpoint.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="45" customHeight="1">
+      <x:c r="A66" s="64" t="str">
+        <x:v>git status --short --branch</x:v>
+      </x:c>
+      <x:c r="B66" s="64" t="str">
+        <x:v>Inspection</x:v>
+      </x:c>
+      <x:c r="C66" s="64" t="str">
+        <x:v>Show current branch and concise working-tree/staging status.</x:v>
+      </x:c>
+      <x:c r="D66" s="64" t="str">
+        <x:v>Before and after editing or staging documentation.</x:v>
+      </x:c>
+      <x:c r="E66" s="64" t="str">
+        <x:v> M means unstaged change; M  means staged change.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="45" customHeight="1">
+      <x:c r="A67" s="63" t="str">
+        <x:v>git branch --show-current</x:v>
+      </x:c>
+      <x:c r="B67" s="63" t="str">
+        <x:v>Inspection</x:v>
+      </x:c>
+      <x:c r="C67" s="63" t="str">
+        <x:v>Print the active local branch name.</x:v>
+      </x:c>
+      <x:c r="D67" s="63" t="str">
+        <x:v>Verify the intended feature branch before committing.</x:v>
+      </x:c>
+      <x:c r="E67" s="63" t="str">
+        <x:v>Expected: docs/phase-2-ebs-lab.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="45" customHeight="1">
+      <x:c r="A68" s="64" t="str">
+        <x:v>git log -1 --format="%h %s"</x:v>
+      </x:c>
+      <x:c r="B68" s="64" t="str">
+        <x:v>Inspection</x:v>
+      </x:c>
+      <x:c r="C68" s="64" t="str">
+        <x:v>Show the latest commit hash and subject.</x:v>
+      </x:c>
+      <x:c r="D68" s="64" t="str">
+        <x:v>Verify the starting main checkpoint.</x:v>
+      </x:c>
+      <x:c r="E68" s="64" t="str">
+        <x:v>Starting checkpoint for this lab: 858378c.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="45" customHeight="1">
+      <x:c r="A69" s="63" t="str">
+        <x:v>git diff --check</x:v>
+      </x:c>
+      <x:c r="B69" s="63" t="str">
+        <x:v>Validation</x:v>
+      </x:c>
+      <x:c r="C69" s="63" t="str">
+        <x:v>Check unstaged changes for whitespace errors.</x:v>
+      </x:c>
+      <x:c r="D69" s="63" t="str">
+        <x:v>After replacing documentation files.</x:v>
+      </x:c>
+      <x:c r="E69" s="63" t="str">
+        <x:v>LF/CRLF conversion warnings on Windows do not by themselves mean errors.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="45" customHeight="1">
+      <x:c r="A70" s="64" t="str">
+        <x:v>git diff --stat</x:v>
+      </x:c>
+      <x:c r="B70" s="64" t="str">
+        <x:v>Review</x:v>
+      </x:c>
+      <x:c r="C70" s="64" t="str">
+        <x:v>Summarize unstaged changes by file.</x:v>
+      </x:c>
+      <x:c r="D70" s="64" t="str">
+        <x:v>Confirm the expected README, diagram, and learning log changed.</x:v>
+      </x:c>
+      <x:c r="E70" s="64" t="str">
+        <x:v>Review actual diffs as needed before staging.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="60" customHeight="1">
+      <x:c r="A71" s="63" t="str">
+        <x:v>git add README.md docs/architecture/cloudvault-current-state.mmd docs/learning-log/phase-2-ec2.md docs/reference/CloudVault_Command_Notes.xlsx</x:v>
+      </x:c>
+      <x:c r="B71" s="63" t="str">
+        <x:v>Staging</x:v>
+      </x:c>
+      <x:c r="C71" s="63" t="str">
+        <x:v>Stage the four Phase 2 documentation/reference files.</x:v>
+      </x:c>
+      <x:c r="D71" s="63" t="str">
+        <x:v>After updating and validating the workbook in the repo.</x:v>
+      </x:c>
+      <x:c r="E71" s="63" t="str">
+        <x:v>Run from repository root; verify the workbook is copied to docs/reference first.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="45" customHeight="1">
+      <x:c r="A72" s="64" t="str">
+        <x:v>git diff --cached --check</x:v>
+      </x:c>
+      <x:c r="B72" s="64" t="str">
+        <x:v>Validation</x:v>
+      </x:c>
+      <x:c r="C72" s="64" t="str">
+        <x:v>Check staged changes for whitespace errors.</x:v>
+      </x:c>
+      <x:c r="D72" s="64" t="str">
+        <x:v>Immediately before committing.</x:v>
+      </x:c>
+      <x:c r="E72" s="64" t="str">
+        <x:v>The --cached flag inspects the staged index.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="45" customHeight="1">
+      <x:c r="A73" s="63" t="str">
+        <x:v>git diff --cached --stat</x:v>
+      </x:c>
+      <x:c r="B73" s="63" t="str">
+        <x:v>Review</x:v>
+      </x:c>
+      <x:c r="C73" s="63" t="str">
+        <x:v>Summarize staged changes by file.</x:v>
+      </x:c>
+      <x:c r="D73" s="63" t="str">
+        <x:v>Confirm the Commands workbook is included with the three documentation files.</x:v>
+      </x:c>
+      <x:c r="E73" s="63" t="str">
+        <x:v>Check git status --short --branch too.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="45" customHeight="1">
+      <x:c r="A74" s="64" t="str">
+        <x:v>git commit -m "docs(phase-2): document EBS persistence and snapshot recovery"</x:v>
+      </x:c>
+      <x:c r="B74" s="64" t="str">
+        <x:v>Commit / Planned</x:v>
+      </x:c>
+      <x:c r="C74" s="64" t="str">
+        <x:v>Commit the reviewed staged changes to the feature branch.</x:v>
+      </x:c>
+      <x:c r="D74" s="64" t="str">
+        <x:v>Only after all four files have been validated.</x:v>
+      </x:c>
+      <x:c r="E74" s="64" t="str">
+        <x:v>Planned next step; not yet executed at this checkpoint.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="45" customHeight="1">
+      <x:c r="A75" s="63" t="str">
+        <x:v>git push -u origin docs/phase-2-ebs-lab</x:v>
+      </x:c>
+      <x:c r="B75" s="63" t="str">
+        <x:v>Remote / Planned</x:v>
+      </x:c>
+      <x:c r="C75" s="63" t="str">
+        <x:v>Push the feature branch and set its upstream.</x:v>
+      </x:c>
+      <x:c r="D75" s="63" t="str">
+        <x:v>After committing, to open a GitHub pull request.</x:v>
+      </x:c>
+      <x:c r="E75" s="63" t="str">
+        <x:v>Planned next step; do not push directly to protected main.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1314,11 +1659,12 @@
     <x:mergeCell ref="A2:E2"/>
     <x:mergeCell ref="A28:E28"/>
     <x:mergeCell ref="A42:E42"/>
+    <x:mergeCell ref="A61:E61"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12418ee50f364b52"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a1216f84d124298"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcfe6e0a3160e4bc0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1070bbf9643f4ef0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1343,9 +1689,9 @@
       <x:c r="D1" s="40"/>
       <x:c r="E1" s="40"/>
     </x:row>
-    <x:row r="2" ht="15" hidden="0" customHeight="1">
+    <x:row r="2" ht="34" hidden="0" customHeight="1">
       <x:c r="A2" s="12" t="str">
-        <x:v>AWS CLI commands used across CloudVault Phase 0 and Phase 1: temporary authentication, identity verification, budgets, IAM, S3 storage, versioning, and least-privilege validation.</x:v>
+        <x:v>CloudVault Phase 0–2 AWS CLI reference: authentication, IAM, S3, EC2, Systems Manager, EBS volumes, snapshots, restoration, and cost control.</x:v>
       </x:c>
       <x:c r="B2" s="12"/>
       <x:c r="C2" s="12"/>
@@ -2762,6 +3108,517 @@
       </x:c>
       <x:c r="E94" s="26" t="str">
         <x:v>Phase 1 S3 usage was effectively $0 at the lab's tiny scale; current-period values are estimated.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="28" customHeight="1">
+      <x:c r="A96" s="56" t="str">
+        <x:v>Phase 2 — EC2 Foundation, Session Manager &amp; Lifecycle</x:v>
+      </x:c>
+      <x:c r="B96" s="56"/>
+      <x:c r="C96" s="56"/>
+      <x:c r="D96" s="56"/>
+      <x:c r="E96" s="56"/>
+    </x:row>
+    <x:row r="97" ht="26" customHeight="1">
+      <x:c r="A97" s="60" t="str">
+        <x:v>Command</x:v>
+      </x:c>
+      <x:c r="B97" s="60" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="C97" s="60" t="str">
+        <x:v>What it does</x:v>
+      </x:c>
+      <x:c r="D97" s="60" t="str">
+        <x:v>When / Why to use it</x:v>
+      </x:c>
+      <x:c r="E97" s="60" t="str">
+        <x:v>Notes / Cautions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="76" customHeight="1">
+      <x:c r="A98" s="63" t="str">
+        <x:v>aws ec2 describe-instances --instance-ids $InstanceId --query "Reservations[].Instances[].{InstanceId:InstanceId,State:State.Name,AZ:Placement.AvailabilityZone,Type:InstanceType}" --output json --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B98" s="63" t="str">
+        <x:v>EC2 / Inventory</x:v>
+      </x:c>
+      <x:c r="C98" s="63" t="str">
+        <x:v>Inspect instance identity, state, type, and Availability Zone.</x:v>
+      </x:c>
+      <x:c r="D98" s="63" t="str">
+        <x:v>Before attaching an EBS volume or starting a lab.</x:v>
+      </x:c>
+      <x:c r="E98" s="63" t="str">
+        <x:v>EBS volumes must be in the same Availability Zone as the EC2 instance.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="60" customHeight="1">
+      <x:c r="A99" s="64" t="str">
+        <x:v>aws ec2 describe-instances --instance-ids $InstanceId --query "Reservations[].Instances[].BlockDeviceMappings" --output json --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B99" s="64" t="str">
+        <x:v>EC2 / Storage</x:v>
+      </x:c>
+      <x:c r="C99" s="64" t="str">
+        <x:v>List the EBS volumes mapped to the instance.</x:v>
+      </x:c>
+      <x:c r="D99" s="64" t="str">
+        <x:v>Distinguish the root volume from the separate data volume.</x:v>
+      </x:c>
+      <x:c r="E99" s="64" t="str">
+        <x:v>Never format or delete the root volume.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="92" customHeight="1">
+      <x:c r="A100" s="63" t="str">
+        <x:v>aws ec2 describe-volumes --volume-ids $DataVolumeId --query "Volumes[].{VolumeId:VolumeId,State:State,Size:Size,Type:VolumeType,Encrypted:Encrypted,AZ:AvailabilityZone,Attachments:Attachments}" --output json --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B100" s="63" t="str">
+        <x:v>EBS / Inspection</x:v>
+      </x:c>
+      <x:c r="C100" s="63" t="str">
+        <x:v>Inspect size, encryption, AZ, state, and attachment information.</x:v>
+      </x:c>
+      <x:c r="D100" s="63" t="str">
+        <x:v>Before and after attaching a data volume.</x:v>
+      </x:c>
+      <x:c r="E100" s="63" t="str">
+        <x:v>Use the exact verified volume ID, not a guessed device name.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="60" customHeight="1">
+      <x:c r="A101" s="64" t="str">
+        <x:v>aws ssm describe-instance-information --filters Key=InstanceIds,Values=$InstanceId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B101" s="64" t="str">
+        <x:v>SSM / Inspection</x:v>
+      </x:c>
+      <x:c r="C101" s="64" t="str">
+        <x:v>Check the instance registration and Session Manager connectivity status.</x:v>
+      </x:c>
+      <x:c r="D101" s="64" t="str">
+        <x:v>Troubleshoot access after an EC2 start.</x:v>
+      </x:c>
+      <x:c r="E101" s="64" t="str">
+        <x:v>The SSM agent needs the instance role and connectivity to Systems Manager endpoints.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="45" customHeight="1">
+      <x:c r="A102" s="63" t="str">
+        <x:v>aws ssm start-session --target $InstanceId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B102" s="63" t="str">
+        <x:v>SSM / Access</x:v>
+      </x:c>
+      <x:c r="C102" s="63" t="str">
+        <x:v>Open a shell on the instance through Systems Manager.</x:v>
+      </x:c>
+      <x:c r="D102" s="63" t="str">
+        <x:v>Perform Linux EBS filesystem commands without SSH.</x:v>
+      </x:c>
+      <x:c r="E102" s="63" t="str">
+        <x:v>Requires Session Manager plugin on Windows; do not open inbound port 22.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="45" customHeight="1">
+      <x:c r="A103" s="64" t="str">
+        <x:v>aws ec2 stop-instances --instance-ids $InstanceId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B103" s="64" t="str">
+        <x:v>EC2 / Cost Control</x:v>
+      </x:c>
+      <x:c r="C103" s="64" t="str">
+        <x:v>Request a normal stop of the instance.</x:v>
+      </x:c>
+      <x:c r="D103" s="64" t="str">
+        <x:v>At the end of the hands-on lab to stop compute charges.</x:v>
+      </x:c>
+      <x:c r="E103" s="64" t="str">
+        <x:v>EBS storage is still billed; do not use force-stop unless troubleshooting requires it.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="45" customHeight="1">
+      <x:c r="A104" s="63" t="str">
+        <x:v>aws ec2 wait instance-stopped --instance-ids $InstanceId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B104" s="63" t="str">
+        <x:v>EC2 / Wait</x:v>
+      </x:c>
+      <x:c r="C104" s="63" t="str">
+        <x:v>Wait until the instance has fully stopped.</x:v>
+      </x:c>
+      <x:c r="D104" s="63" t="str">
+        <x:v>Verify a safe stopping checkpoint before leaving the lab.</x:v>
+      </x:c>
+      <x:c r="E104" s="63" t="str">
+        <x:v>Successful waiter is silent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="45" customHeight="1">
+      <x:c r="A105" s="64" t="str">
+        <x:v>aws ec2 start-instances --instance-ids $InstanceId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B105" s="64" t="str">
+        <x:v>EC2 / Lifecycle</x:v>
+      </x:c>
+      <x:c r="C105" s="64" t="str">
+        <x:v>Start the same existing instance.</x:v>
+      </x:c>
+      <x:c r="D105" s="64" t="str">
+        <x:v>Verify data survives a stop/start cycle.</x:v>
+      </x:c>
+      <x:c r="E105" s="64" t="str">
+        <x:v>Public IPv4 may change; EBS volumes persist.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="45" customHeight="1">
+      <x:c r="A106" s="63" t="str">
+        <x:v>aws ec2 wait instance-running --instance-ids $InstanceId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B106" s="63" t="str">
+        <x:v>EC2 / Wait</x:v>
+      </x:c>
+      <x:c r="C106" s="63" t="str">
+        <x:v>Wait for the instance to reach running state.</x:v>
+      </x:c>
+      <x:c r="D106" s="63" t="str">
+        <x:v>Before reconnecting via Session Manager.</x:v>
+      </x:c>
+      <x:c r="E106" s="63" t="str">
+        <x:v>SSM connectivity may take longer than the EC2 running state.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="92" customHeight="1">
+      <x:c r="A107" s="64" t="str">
+        <x:v>aws ec2 describe-instances --instance-ids $InstanceId --query "Reservations[].Instances[].{InstanceId:InstanceId,State:State.Name,InstanceType:InstanceType,Volumes:BlockDeviceMappings[].Ebs.VolumeId}" --output json --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B107" s="64" t="str">
+        <x:v>EC2 / Final Verification</x:v>
+      </x:c>
+      <x:c r="C107" s="64" t="str">
+        <x:v>Confirm final EC2 state and attached EBS volume IDs.</x:v>
+      </x:c>
+      <x:c r="D107" s="64" t="str">
+        <x:v>Verify the instance is stopped and the original root/data volumes remain.</x:v>
+      </x:c>
+      <x:c r="E107" s="64" t="str">
+        <x:v>Verified end state: stopped t3.micro with an 8 GiB root and 1 GiB data volume.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="28" customHeight="1">
+      <x:c r="A109" s="56" t="str">
+        <x:v>Phase 2 — EBS Provisioning, Snapshot, Recovery &amp; Cleanup</x:v>
+      </x:c>
+      <x:c r="B109" s="56"/>
+      <x:c r="C109" s="56"/>
+      <x:c r="D109" s="56"/>
+      <x:c r="E109" s="56"/>
+    </x:row>
+    <x:row r="110" ht="26" customHeight="1">
+      <x:c r="A110" s="60" t="str">
+        <x:v>Command</x:v>
+      </x:c>
+      <x:c r="B110" s="60" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="C110" s="60" t="str">
+        <x:v>What it does</x:v>
+      </x:c>
+      <x:c r="D110" s="60" t="str">
+        <x:v>When / Why to use it</x:v>
+      </x:c>
+      <x:c r="E110" s="60" t="str">
+        <x:v>Notes / Cautions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="76" customHeight="1">
+      <x:c r="A111" s="63" t="str">
+        <x:v>aws ec2 create-volume --availability-zone ap-southeast-1a --size 1 --volume-type gp3 --encrypted --tag-specifications 'ResourceType=volume,Tags=[{Key=Name,Value=CloudVaultEBSDataDev01}]' --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B111" s="63" t="str">
+        <x:v>EBS / Provisioning</x:v>
+      </x:c>
+      <x:c r="C111" s="63" t="str">
+        <x:v>Create a 1 GiB encrypted gp3 data volume in the EC2 Availability Zone.</x:v>
+      </x:c>
+      <x:c r="D111" s="63" t="str">
+        <x:v>Begin the separate EBS data-volume lab.</x:v>
+      </x:c>
+      <x:c r="E111" s="63" t="str">
+        <x:v>Creating a volume incurs storage cost. Verify the AZ before running; the Name tag is illustrative.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="45" customHeight="1">
+      <x:c r="A112" s="64" t="str">
+        <x:v>aws ec2 wait volume-available --volume-ids $DataVolumeId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B112" s="64" t="str">
+        <x:v>EBS / Wait</x:v>
+      </x:c>
+      <x:c r="C112" s="64" t="str">
+        <x:v>Wait for the newly created volume to be available.</x:v>
+      </x:c>
+      <x:c r="D112" s="64" t="str">
+        <x:v>Before attaching the data volume to EC2.</x:v>
+      </x:c>
+      <x:c r="E112" s="64" t="str">
+        <x:v>Successful waiter is silent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="60" customHeight="1">
+      <x:c r="A113" s="63" t="str">
+        <x:v>aws ec2 attach-volume --volume-id $DataVolumeId --instance-id $InstanceId --device /dev/sdf --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B113" s="63" t="str">
+        <x:v>EBS / Attachment</x:v>
+      </x:c>
+      <x:c r="C113" s="63" t="str">
+        <x:v>Attach the original data volume to the instance.</x:v>
+      </x:c>
+      <x:c r="D113" s="63" t="str">
+        <x:v>Prepare the blank volume for filesystem creation.</x:v>
+      </x:c>
+      <x:c r="E113" s="63" t="str">
+        <x:v>On Nitro instances, the actual Linux name can be /dev/nvme1n1 or another NVMe path; verify SERIAL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="45" customHeight="1">
+      <x:c r="A114" s="64" t="str">
+        <x:v>aws ec2 wait volume-in-use --volume-ids $DataVolumeId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B114" s="64" t="str">
+        <x:v>EBS / Wait</x:v>
+      </x:c>
+      <x:c r="C114" s="64" t="str">
+        <x:v>Wait until AWS reports the data volume is attached/in use.</x:v>
+      </x:c>
+      <x:c r="D114" s="64" t="str">
+        <x:v>Before inspecting it inside the Linux instance.</x:v>
+      </x:c>
+      <x:c r="E114" s="64" t="str">
+        <x:v>Do not format until device serial, size, and existing signatures are verified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="60" customHeight="1">
+      <x:c r="A115" s="63" t="str">
+        <x:v>aws ec2 create-snapshot --volume-id $DataVolumeId --description "CloudVault EBS data recovery lab" --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B115" s="63" t="str">
+        <x:v>EBS / Snapshot</x:v>
+      </x:c>
+      <x:c r="C115" s="63" t="str">
+        <x:v>Create a point-in-time EBS snapshot of the original data volume.</x:v>
+      </x:c>
+      <x:c r="D115" s="63" t="str">
+        <x:v>After writing test data and calling sync in Linux.</x:v>
+      </x:c>
+      <x:c r="E115" s="63" t="str">
+        <x:v>Snapshot storage can incur charges; volume remains attached and usable.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="45" customHeight="1">
+      <x:c r="A116" s="64" t="str">
+        <x:v>aws ec2 wait snapshot-completed --snapshot-ids $SnapshotId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B116" s="64" t="str">
+        <x:v>EBS / Wait</x:v>
+      </x:c>
+      <x:c r="C116" s="64" t="str">
+        <x:v>Wait for the snapshot to complete.</x:v>
+      </x:c>
+      <x:c r="D116" s="64" t="str">
+        <x:v>Before creating a restored EBS volume from it.</x:v>
+      </x:c>
+      <x:c r="E116" s="64" t="str">
+        <x:v>Successful waiter is silent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="76" customHeight="1">
+      <x:c r="A117" s="63" t="str">
+        <x:v>aws ec2 describe-snapshots --snapshot-ids $SnapshotId --query "Snapshots[].{SnapshotId:SnapshotId,State:State,Progress:Progress,Encrypted:Encrypted,VolumeId:VolumeId}" --output json --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B117" s="63" t="str">
+        <x:v>EBS / Snapshot Verification</x:v>
+      </x:c>
+      <x:c r="C117" s="63" t="str">
+        <x:v>Verify snapshot status, progress, encryption, and source volume.</x:v>
+      </x:c>
+      <x:c r="D117" s="63" t="str">
+        <x:v>Confirm completed 100% before restoration.</x:v>
+      </x:c>
+      <x:c r="E117" s="63" t="str">
+        <x:v>Snapshot is a backup of EBS blocks, not a mounted filesystem.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="92" customHeight="1">
+      <x:c r="A118" s="64" t="str">
+        <x:v>aws ec2 create-volume --availability-zone ap-southeast-1a --snapshot-id $SnapshotId --volume-type gp3 --encrypted --tag-specifications 'ResourceType=volume,Tags=[{Key=Name,Value=CloudVaultEBSRestoredDev01}]' --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B118" s="64" t="str">
+        <x:v>EBS / Recovery</x:v>
+      </x:c>
+      <x:c r="C118" s="64" t="str">
+        <x:v>Restore the snapshot to a separate encrypted gp3 volume.</x:v>
+      </x:c>
+      <x:c r="D118" s="64" t="str">
+        <x:v>Test recovery without changing the original volume.</x:v>
+      </x:c>
+      <x:c r="E118" s="64" t="str">
+        <x:v>Use the EC2 instance AZ; the restored XFS filesystem initially shares the original UUID.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="45" customHeight="1">
+      <x:c r="A119" s="63" t="str">
+        <x:v>aws ec2 wait volume-available --volume-ids $RestoredVolumeId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B119" s="63" t="str">
+        <x:v>EBS / Wait</x:v>
+      </x:c>
+      <x:c r="C119" s="63" t="str">
+        <x:v>Wait until the restored volume is available.</x:v>
+      </x:c>
+      <x:c r="D119" s="63" t="str">
+        <x:v>Before attaching the restored volume.</x:v>
+      </x:c>
+      <x:c r="E119" s="63" t="str">
+        <x:v>Successful waiter is silent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="60" customHeight="1">
+      <x:c r="A120" s="64" t="str">
+        <x:v>aws ec2 attach-volume --volume-id $RestoredVolumeId --instance-id $InstanceId --device /dev/sdg --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B120" s="64" t="str">
+        <x:v>EBS / Recovery Attachment</x:v>
+      </x:c>
+      <x:c r="C120" s="64" t="str">
+        <x:v>Attach the restored EBS volume alongside the original.</x:v>
+      </x:c>
+      <x:c r="D120" s="64" t="str">
+        <x:v>Compare recovered test data against the source.</x:v>
+      </x:c>
+      <x:c r="E120" s="64" t="str">
+        <x:v>Confirm the new Linux NVMe serial before mounting; do not format the restored volume.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="76" customHeight="1">
+      <x:c r="A121" s="63" t="str">
+        <x:v>aws ec2 describe-volumes --volume-ids $RestoredVolumeId --query "Volumes[].{VolumeId:VolumeId,State:State,Attachments:Attachments}" --output json --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B121" s="63" t="str">
+        <x:v>EBS / Recovery Verification</x:v>
+      </x:c>
+      <x:c r="C121" s="63" t="str">
+        <x:v>Check the restored volume state and attachment.</x:v>
+      </x:c>
+      <x:c r="D121" s="63" t="str">
+        <x:v>Before or after read-only restore validation.</x:v>
+      </x:c>
+      <x:c r="E121" s="63" t="str">
+        <x:v>The restored volume must be unmounted before detachment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="45" customHeight="1">
+      <x:c r="A122" s="64" t="str">
+        <x:v>aws ec2 detach-volume --volume-id $RestoredVolumeId --instance-id $InstanceId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B122" s="64" t="str">
+        <x:v>EBS / Cleanup</x:v>
+      </x:c>
+      <x:c r="C122" s="64" t="str">
+        <x:v>Normally detach the temporary restored volume.</x:v>
+      </x:c>
+      <x:c r="D122" s="64" t="str">
+        <x:v>After sudo umount and verification inside Linux.</x:v>
+      </x:c>
+      <x:c r="E122" s="64" t="str">
+        <x:v>Avoid --force during normal cleanup; verify this is NOT the original data volume.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="45" customHeight="1">
+      <x:c r="A123" s="63" t="str">
+        <x:v>aws ec2 wait volume-available --volume-ids $RestoredVolumeId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B123" s="63" t="str">
+        <x:v>EBS / Cleanup Verification</x:v>
+      </x:c>
+      <x:c r="C123" s="63" t="str">
+        <x:v>Wait until the detached restored volume is available.</x:v>
+      </x:c>
+      <x:c r="D123" s="63" t="str">
+        <x:v>Before deleting the temporary restored volume.</x:v>
+      </x:c>
+      <x:c r="E123" s="63" t="str">
+        <x:v>Successful waiter is silent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="45" customHeight="1">
+      <x:c r="A124" s="64" t="str">
+        <x:v>aws ec2 delete-volume --volume-id $RestoredVolumeId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B124" s="65" t="str">
+        <x:v>EBS / Cleanup — Destructive</x:v>
+      </x:c>
+      <x:c r="C124" s="64" t="str">
+        <x:v>Permanently delete the temporary restored EBS volume.</x:v>
+      </x:c>
+      <x:c r="D124" s="64" t="str">
+        <x:v>After successful data comparison and detachment.</x:v>
+      </x:c>
+      <x:c r="E124" s="64" t="str">
+        <x:v>IRREVERSIBLE. Never substitute $DataVolumeId or the root volume ID.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="45" customHeight="1">
+      <x:c r="A125" s="63" t="str">
+        <x:v>aws ec2 describe-volumes --volume-ids $RestoredVolumeId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B125" s="63" t="str">
+        <x:v>EBS / Cleanup Verification</x:v>
+      </x:c>
+      <x:c r="C125" s="63" t="str">
+        <x:v>Check whether the deleted restored volume still exists.</x:v>
+      </x:c>
+      <x:c r="D125" s="63" t="str">
+        <x:v>Confirm successful deletion.</x:v>
+      </x:c>
+      <x:c r="E125" s="63" t="str">
+        <x:v>InvalidVolume.NotFound is the expected result after deletion.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="45" customHeight="1">
+      <x:c r="A126" s="64" t="str">
+        <x:v>aws ec2 delete-snapshot --snapshot-id $SnapshotId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B126" s="65" t="str">
+        <x:v>EBS / Cleanup — Destructive</x:v>
+      </x:c>
+      <x:c r="C126" s="64" t="str">
+        <x:v>Permanently delete the temporary recovery snapshot.</x:v>
+      </x:c>
+      <x:c r="D126" s="64" t="str">
+        <x:v>After restoring and verifying data and deleting the restored volume.</x:v>
+      </x:c>
+      <x:c r="E126" s="64" t="str">
+        <x:v>IRREVERSIBLE. Deleting a snapshot removes this recovery point; original EBS remains.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127" ht="45" customHeight="1">
+      <x:c r="A127" s="63" t="str">
+        <x:v>aws ec2 describe-snapshots --snapshot-ids $SnapshotId --profile cloudvault --region ap-southeast-1</x:v>
+      </x:c>
+      <x:c r="B127" s="63" t="str">
+        <x:v>EBS / Cleanup Verification</x:v>
+      </x:c>
+      <x:c r="C127" s="63" t="str">
+        <x:v>Check whether the deleted snapshot still exists.</x:v>
+      </x:c>
+      <x:c r="D127" s="63" t="str">
+        <x:v>Confirm successful snapshot cleanup.</x:v>
+      </x:c>
+      <x:c r="E127" s="63" t="str">
+        <x:v>InvalidSnapshot.NotFound is the expected result after deletion.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2773,10 +3630,12 @@
     <x:mergeCell ref="A27:E27"/>
     <x:mergeCell ref="A29:E29"/>
     <x:mergeCell ref="A35:E35"/>
+    <x:mergeCell ref="A96:E96"/>
+    <x:mergeCell ref="A109:E109"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19b013e8bd424d4a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7b2ee5fd39b4d0e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2801,9 +3660,9 @@
       <x:c r="D1" s="40"/>
       <x:c r="E1" s="40"/>
     </x:row>
-    <x:row r="2" ht="15" hidden="0" customHeight="1">
+    <x:row r="2" ht="34" hidden="0" customHeight="1">
       <x:c r="A2" s="12" t="str">
-        <x:v>PowerShell and Windows shell commands used while installing/troubleshooting AWS CLI and Git and managing the CloudVault project.</x:v>
+        <x:v>Windows PowerShell reference for CloudVault setup, validation, Phase 2 EBS resource variables, and documentation.</x:v>
       </x:c>
       <x:c r="B2" s="12"/>
       <x:c r="C2" s="12"/>
@@ -3831,75 +4690,167 @@
       <x:c r="D69" s="26"/>
       <x:c r="E69" s="26"/>
     </x:row>
-    <x:row r="70" ht="15" hidden="0" customHeight="1">
-      <x:c r="A70" s="26"/>
-      <x:c r="B70" s="26"/>
-      <x:c r="C70" s="26"/>
-      <x:c r="D70" s="26"/>
-      <x:c r="E70" s="26"/>
-    </x:row>
-    <x:row r="71" ht="15" hidden="0" customHeight="1">
-      <x:c r="A71" s="26"/>
-      <x:c r="B71" s="26"/>
-      <x:c r="C71" s="26"/>
-      <x:c r="D71" s="26"/>
-      <x:c r="E71" s="26"/>
-    </x:row>
-    <x:row r="72" ht="15" hidden="0" customHeight="1">
-      <x:c r="A72" s="26"/>
-      <x:c r="B72" s="26"/>
-      <x:c r="C72" s="26"/>
-      <x:c r="D72" s="26"/>
-      <x:c r="E72" s="26"/>
-    </x:row>
-    <x:row r="73" ht="15" hidden="0" customHeight="1">
-      <x:c r="A73" s="26"/>
-      <x:c r="B73" s="26"/>
-      <x:c r="C73" s="26"/>
-      <x:c r="D73" s="26"/>
-      <x:c r="E73" s="26"/>
-    </x:row>
-    <x:row r="74" ht="15" hidden="0" customHeight="1">
-      <x:c r="A74" s="26"/>
-      <x:c r="B74" s="26"/>
-      <x:c r="C74" s="26"/>
-      <x:c r="D74" s="26"/>
-      <x:c r="E74" s="26"/>
-    </x:row>
-    <x:row r="75" ht="15" hidden="0" customHeight="1">
-      <x:c r="A75" s="26"/>
-      <x:c r="B75" s="26"/>
-      <x:c r="C75" s="26"/>
-      <x:c r="D75" s="26"/>
-      <x:c r="E75" s="26"/>
-    </x:row>
-    <x:row r="76" ht="15" hidden="0" customHeight="1">
-      <x:c r="A76" s="26"/>
-      <x:c r="B76" s="26"/>
-      <x:c r="C76" s="26"/>
-      <x:c r="D76" s="26"/>
-      <x:c r="E76" s="26"/>
-    </x:row>
-    <x:row r="77" ht="15" hidden="0" customHeight="1">
-      <x:c r="A77" s="26"/>
-      <x:c r="B77" s="26"/>
-      <x:c r="C77" s="26"/>
-      <x:c r="D77" s="26"/>
-      <x:c r="E77" s="26"/>
-    </x:row>
-    <x:row r="78" ht="15" hidden="0" customHeight="1">
-      <x:c r="A78" s="26"/>
-      <x:c r="B78" s="26"/>
-      <x:c r="C78" s="26"/>
-      <x:c r="D78" s="26"/>
-      <x:c r="E78" s="26"/>
-    </x:row>
-    <x:row r="79" ht="15" hidden="0" customHeight="1">
-      <x:c r="A79" s="26"/>
-      <x:c r="B79" s="26"/>
-      <x:c r="C79" s="26"/>
-      <x:c r="D79" s="26"/>
-      <x:c r="E79" s="26"/>
+    <x:row r="70" ht="28" hidden="0" customHeight="1">
+      <x:c r="A70" s="68" t="str">
+        <x:v>Phase 2 — EBS Variables &amp; Documentation Inspection</x:v>
+      </x:c>
+      <x:c r="B70" s="68"/>
+      <x:c r="C70" s="68"/>
+      <x:c r="D70" s="68"/>
+      <x:c r="E70" s="68"/>
+    </x:row>
+    <x:row r="71" ht="26" hidden="0" customHeight="1">
+      <x:c r="A71" s="60" t="str">
+        <x:v>Command</x:v>
+      </x:c>
+      <x:c r="B71" s="60" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="C71" s="60" t="str">
+        <x:v>What it does</x:v>
+      </x:c>
+      <x:c r="D71" s="60" t="str">
+        <x:v>When / Why to use it</x:v>
+      </x:c>
+      <x:c r="E71" s="60" t="str">
+        <x:v>Notes / Cautions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="45" hidden="0" customHeight="1">
+      <x:c r="A72" s="63" t="str">
+        <x:v>$InstanceId = "REPLACE_WITH_VERIFIED_INSTANCE_ID"</x:v>
+      </x:c>
+      <x:c r="B72" s="63" t="str">
+        <x:v>Variables / EC2</x:v>
+      </x:c>
+      <x:c r="C72" s="63" t="str">
+        <x:v>Store the verified EC2 instance ID in the current PowerShell session.</x:v>
+      </x:c>
+      <x:c r="D72" s="63" t="str">
+        <x:v>Before EC2 and SSM commands that use $InstanceId.</x:v>
+      </x:c>
+      <x:c r="E72" s="63" t="str">
+        <x:v>Variables do not persist across new terminal sessions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="45" hidden="0" customHeight="1">
+      <x:c r="A73" s="64" t="str">
+        <x:v>$DataVolumeId = "REPLACE_WITH_ORIGINAL_DATA_VOLUME_ID"</x:v>
+      </x:c>
+      <x:c r="B73" s="64" t="str">
+        <x:v>Variables / EBS</x:v>
+      </x:c>
+      <x:c r="C73" s="64" t="str">
+        <x:v>Store the original data volume ID.</x:v>
+      </x:c>
+      <x:c r="D73" s="64" t="str">
+        <x:v>Before creating snapshots or inspecting the original disk.</x:v>
+      </x:c>
+      <x:c r="E73" s="64" t="str">
+        <x:v>NEVER confuse the original data volume with the disposable restored volume.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="45" hidden="0" customHeight="1">
+      <x:c r="A74" s="63" t="str">
+        <x:v>$SnapshotId = "REPLACE_WITH_SNAPSHOT_ID"</x:v>
+      </x:c>
+      <x:c r="B74" s="63" t="str">
+        <x:v>Variables / EBS</x:v>
+      </x:c>
+      <x:c r="C74" s="63" t="str">
+        <x:v>Store the temporary EBS snapshot ID.</x:v>
+      </x:c>
+      <x:c r="D74" s="63" t="str">
+        <x:v>Before snapshot status, restore, and cleanup commands.</x:v>
+      </x:c>
+      <x:c r="E74" s="63" t="str">
+        <x:v>The snapshot was deleted at the end of the lab.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="45" hidden="0" customHeight="1">
+      <x:c r="A75" s="64" t="str">
+        <x:v>$RestoredVolumeId = "REPLACE_WITH_RESTORED_VOLUME_ID"</x:v>
+      </x:c>
+      <x:c r="B75" s="64" t="str">
+        <x:v>Variables / EBS</x:v>
+      </x:c>
+      <x:c r="C75" s="64" t="str">
+        <x:v>Store the temporary restored EBS volume ID.</x:v>
+      </x:c>
+      <x:c r="D75" s="64" t="str">
+        <x:v>Before inspecting, detaching, or deleting the restored volume.</x:v>
+      </x:c>
+      <x:c r="E75" s="64" t="str">
+        <x:v>The restored volume was deleted at the end of the lab.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="45" hidden="0" customHeight="1">
+      <x:c r="A76" s="63" t="str">
+        <x:v>Get-Content .\docs\learning-log\phase-2-ec2.md</x:v>
+      </x:c>
+      <x:c r="B76" s="63" t="str">
+        <x:v>Documentation / Inspection</x:v>
+      </x:c>
+      <x:c r="C76" s="63" t="str">
+        <x:v>Display the current Phase 2 learning log.</x:v>
+      </x:c>
+      <x:c r="D76" s="63" t="str">
+        <x:v>Before editing or verifying the EBS lab notes.</x:v>
+      </x:c>
+      <x:c r="E76" s="63" t="str">
+        <x:v>Run from the CloudVault repository root.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="45" hidden="0" customHeight="1">
+      <x:c r="A77" s="64" t="str">
+        <x:v>Get-Content .\docs\architecture\cloudvault-current-state.mmd</x:v>
+      </x:c>
+      <x:c r="B77" s="64" t="str">
+        <x:v>Documentation / Inspection</x:v>
+      </x:c>
+      <x:c r="C77" s="64" t="str">
+        <x:v>Display the current Mermaid architecture source.</x:v>
+      </x:c>
+      <x:c r="D77" s="64" t="str">
+        <x:v>Before updating the deployed-resource and recovery-workflow diagram.</x:v>
+      </x:c>
+      <x:c r="E77" s="64" t="str">
+        <x:v>A source-text check does not replace visual Mermaid rendering.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="45" hidden="0" customHeight="1">
+      <x:c r="A78" s="63" t="str">
+        <x:v>Get-Content .\README.md</x:v>
+      </x:c>
+      <x:c r="B78" s="63" t="str">
+        <x:v>Documentation / Inspection</x:v>
+      </x:c>
+      <x:c r="C78" s="63" t="str">
+        <x:v>Display the project README.</x:v>
+      </x:c>
+      <x:c r="D78" s="63" t="str">
+        <x:v>Before updating the Phase 2 progress and resource status.</x:v>
+      </x:c>
+      <x:c r="E78" s="63" t="str">
+        <x:v>Run from the repository root.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="45" hidden="0" customHeight="1">
+      <x:c r="A79" s="64" t="str">
+        <x:v>Copy-Item .\CloudVault_Command_Notes_Phase2_Updated.xlsx .\docs\reference\CloudVault_Command_Notes.xlsx</x:v>
+      </x:c>
+      <x:c r="B79" s="64" t="str">
+        <x:v>Documentation / Workbook</x:v>
+      </x:c>
+      <x:c r="C79" s="64" t="str">
+        <x:v>Copy the updated workbook into the tracked reference location.</x:v>
+      </x:c>
+      <x:c r="D79" s="64" t="str">
+        <x:v>After downloading this updated workbook into the repository root.</x:v>
+      </x:c>
+      <x:c r="E79" s="64" t="str">
+        <x:v>If the downloaded filename or location differs, adjust the source path; overwrites destination.</x:v>
+      </x:c>
     </x:row>
     <x:row r="80" ht="15" hidden="0" customHeight="1">
       <x:c r="A80" s="26"/>
@@ -3984,10 +4935,535 @@
     <x:mergeCell ref="A2:E2"/>
     <x:mergeCell ref="A27:E27"/>
     <x:mergeCell ref="A29:E29"/>
+    <x:mergeCell ref="A70:E70"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec23640550714bee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b49ef0ca5c843f2"/>
   </x:tableParts>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="55" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="42" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="43" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="46" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="71" t="str">
+        <x:v>Linux / SSM Command Reference</x:v>
+      </x:c>
+      <x:c r="B1" s="71"/>
+      <x:c r="C1" s="71"/>
+      <x:c r="D1" s="71"/>
+      <x:c r="E1" s="71"/>
+    </x:row>
+    <x:row r="2" ht="36" customHeight="1">
+      <x:c r="A2" s="75" t="str">
+        <x:v>CloudVault Phase 2 — commands run inside the Amazon Linux 2023 Session Manager shell. Verify NVMe serials before disk operations.</x:v>
+      </x:c>
+      <x:c r="B2" s="75"/>
+      <x:c r="C2" s="75"/>
+      <x:c r="D2" s="75"/>
+      <x:c r="E2" s="75"/>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="A4" s="56" t="str">
+        <x:v>Phase 2 — EC2 Linux Storage, Snapshot Validation &amp; S3 Tests</x:v>
+      </x:c>
+      <x:c r="B4" s="56"/>
+      <x:c r="C4" s="56"/>
+      <x:c r="D4" s="56"/>
+      <x:c r="E4" s="56"/>
+    </x:row>
+    <x:row r="5" ht="26" customHeight="1">
+      <x:c r="A5" s="60" t="str">
+        <x:v>Command</x:v>
+      </x:c>
+      <x:c r="B5" s="60" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="C5" s="60" t="str">
+        <x:v>What it does</x:v>
+      </x:c>
+      <x:c r="D5" s="60" t="str">
+        <x:v>When / Why to use it</x:v>
+      </x:c>
+      <x:c r="E5" s="60" t="str">
+        <x:v>Notes / Cautions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="45" customHeight="1">
+      <x:c r="A6" s="63" t="str">
+        <x:v>lsblk -o NAME,SIZE,TYPE,SERIAL,FSTYPE,MOUNTPOINTS</x:v>
+      </x:c>
+      <x:c r="B6" s="63" t="str">
+        <x:v>Device identification</x:v>
+      </x:c>
+      <x:c r="C6" s="63" t="str">
+        <x:v>List block devices, serials, filesystem types, and mounts.</x:v>
+      </x:c>
+      <x:c r="D6" s="63" t="str">
+        <x:v>Identify original and restored Nitro NVMe EBS devices before touching them.</x:v>
+      </x:c>
+      <x:c r="E6" s="63" t="str">
+        <x:v>Match the EBS volume ID to the NVMe SERIAL; device numbering can change.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="45" customHeight="1">
+      <x:c r="A7" s="64" t="str">
+        <x:v>sudo blkid /dev/nvme1n1</x:v>
+      </x:c>
+      <x:c r="B7" s="64" t="str">
+        <x:v>Filesystem inspection</x:v>
+      </x:c>
+      <x:c r="C7" s="64" t="str">
+        <x:v>Read filesystem UUID and type for the identified original data disk.</x:v>
+      </x:c>
+      <x:c r="D7" s="64" t="str">
+        <x:v>Before adding an /etc/fstab entry.</x:v>
+      </x:c>
+      <x:c r="E7" s="64" t="str">
+        <x:v>Example device path from this lab; verify the actual device first.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="45" customHeight="1">
+      <x:c r="A8" s="63" t="str">
+        <x:v>sudo wipefs -n /dev/nvme1n1</x:v>
+      </x:c>
+      <x:c r="B8" s="63" t="str">
+        <x:v>Non-destructive inspection</x:v>
+      </x:c>
+      <x:c r="C8" s="63" t="str">
+        <x:v>List filesystem signatures without erasing them.</x:v>
+      </x:c>
+      <x:c r="D8" s="63" t="str">
+        <x:v>Before formatting a newly attached blank disk.</x:v>
+      </x:c>
+      <x:c r="E8" s="63" t="str">
+        <x:v>The -n option is a dry run. Never use wipefs to clear an unverified disk.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="45" customHeight="1">
+      <x:c r="A9" s="64" t="str">
+        <x:v>sudo mkfs.xfs /dev/nvme1n1</x:v>
+      </x:c>
+      <x:c r="B9" s="65" t="str">
+        <x:v>Filesystem creation — DESTRUCTIVE</x:v>
+      </x:c>
+      <x:c r="C9" s="64" t="str">
+        <x:v>Create an XFS filesystem on the verified new blank data volume.</x:v>
+      </x:c>
+      <x:c r="D9" s="64" t="str">
+        <x:v>One-time initial provisioning of the original 1 GiB data volume.</x:v>
+      </x:c>
+      <x:c r="E9" s="64" t="str">
+        <x:v>IRREVERSIBLE if run on the wrong disk. Never run on /dev/nvme0n1 (root) or the restored disk.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="45" customHeight="1">
+      <x:c r="A10" s="63" t="str">
+        <x:v>sudo mkdir -p /data/cloudvault</x:v>
+      </x:c>
+      <x:c r="B10" s="63" t="str">
+        <x:v>Mount point</x:v>
+      </x:c>
+      <x:c r="C10" s="63" t="str">
+        <x:v>Create the persistent data-volume mount directory.</x:v>
+      </x:c>
+      <x:c r="D10" s="63" t="str">
+        <x:v>Before mounting the original data disk.</x:v>
+      </x:c>
+      <x:c r="E10" s="63" t="str">
+        <x:v>Directory creation is safe; filesystem mount is a separate step.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="45" customHeight="1">
+      <x:c r="A11" s="64" t="str">
+        <x:v>sudo mount /dev/nvme1n1 /data/cloudvault</x:v>
+      </x:c>
+      <x:c r="B11" s="64" t="str">
+        <x:v>Mount</x:v>
+      </x:c>
+      <x:c r="C11" s="64" t="str">
+        <x:v>Mount the original XFS data filesystem.</x:v>
+      </x:c>
+      <x:c r="D11" s="64" t="str">
+        <x:v>After confirming device identity and filesystem creation.</x:v>
+      </x:c>
+      <x:c r="E11" s="64" t="str">
+        <x:v>Example device name only; do not mount a random NVMe disk.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="45" customHeight="1">
+      <x:c r="A12" s="63" t="str">
+        <x:v>findmnt /data/cloudvault</x:v>
+      </x:c>
+      <x:c r="B12" s="63" t="str">
+        <x:v>Mount verification</x:v>
+      </x:c>
+      <x:c r="C12" s="63" t="str">
+        <x:v>Show the source device and mount options for the data directory.</x:v>
+      </x:c>
+      <x:c r="D12" s="63" t="str">
+        <x:v>Confirm the original data volume is mounted.</x:v>
+      </x:c>
+      <x:c r="E12" s="63" t="str">
+        <x:v>Check source, target, and filesystem type.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="45" customHeight="1">
+      <x:c r="A13" s="64" t="str">
+        <x:v>df -hT /data/cloudvault</x:v>
+      </x:c>
+      <x:c r="B13" s="64" t="str">
+        <x:v>Capacity verification</x:v>
+      </x:c>
+      <x:c r="C13" s="64" t="str">
+        <x:v>Show mounted filesystem type, size, used, and available space.</x:v>
+      </x:c>
+      <x:c r="D13" s="64" t="str">
+        <x:v>Confirm the expected 1 GiB XFS data volume.</x:v>
+      </x:c>
+      <x:c r="E13" s="64" t="str">
+        <x:v>Useful alongside findmnt and lsblk.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="45" customHeight="1">
+      <x:c r="A14" s="63" t="str">
+        <x:v>echo "CloudVault EBS storage test - Phase 2" | sudo tee /data/cloudvault/ebs-test.txt</x:v>
+      </x:c>
+      <x:c r="B14" s="63" t="str">
+        <x:v>Write test</x:v>
+      </x:c>
+      <x:c r="C14" s="63" t="str">
+        <x:v>Write a small known-content test file to EBS.</x:v>
+      </x:c>
+      <x:c r="D14" s="63" t="str">
+        <x:v>Verify persistence across stop/start and snapshot restore.</x:v>
+      </x:c>
+      <x:c r="E14" s="63" t="str">
+        <x:v>Only write after confirming /data/cloudvault is mounted to the intended volume.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="45" customHeight="1">
+      <x:c r="A15" s="64" t="str">
+        <x:v>cat /data/cloudvault/ebs-test.txt</x:v>
+      </x:c>
+      <x:c r="B15" s="64" t="str">
+        <x:v>Read test</x:v>
+      </x:c>
+      <x:c r="C15" s="64" t="str">
+        <x:v>Read the test file from the original EBS volume.</x:v>
+      </x:c>
+      <x:c r="D15" s="64" t="str">
+        <x:v>Confirm persistence after restarting EC2.</x:v>
+      </x:c>
+      <x:c r="E15" s="64" t="str">
+        <x:v>Expected: CloudVault EBS storage test - Phase 2.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="45" customHeight="1">
+      <x:c r="A16" s="63" t="str">
+        <x:v>sudo cp /etc/fstab /etc/fstab.cloudvault.bak</x:v>
+      </x:c>
+      <x:c r="B16" s="63" t="str">
+        <x:v>Configuration backup</x:v>
+      </x:c>
+      <x:c r="C16" s="63" t="str">
+        <x:v>Back up /etc/fstab before changing persistent mount settings.</x:v>
+      </x:c>
+      <x:c r="D16" s="63" t="str">
+        <x:v>Before adding the data-volume UUID entry.</x:v>
+      </x:c>
+      <x:c r="E16" s="63" t="str">
+        <x:v>A bad fstab entry can affect boot behavior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="45" customHeight="1">
+      <x:c r="A17" s="64" t="str">
+        <x:v>sudo blkid -s UUID -o value /dev/nvme1n1</x:v>
+      </x:c>
+      <x:c r="B17" s="64" t="str">
+        <x:v>UUID lookup</x:v>
+      </x:c>
+      <x:c r="C17" s="64" t="str">
+        <x:v>Print only the original XFS filesystem UUID.</x:v>
+      </x:c>
+      <x:c r="D17" s="64" t="str">
+        <x:v>Use stable UUID-based mounting rather than a changing NVMe path.</x:v>
+      </x:c>
+      <x:c r="E17" s="64" t="str">
+        <x:v>Verify the serial and device identity first.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="45" customHeight="1">
+      <x:c r="A18" s="63" t="str">
+        <x:v>printf 'UUID=&lt;VERIFIED_UUID&gt; /data/cloudvault xfs defaults,nofail 0 0\n' | sudo tee -a /etc/fstab</x:v>
+      </x:c>
+      <x:c r="B18" s="63" t="str">
+        <x:v>Persistent mount / Example</x:v>
+      </x:c>
+      <x:c r="C18" s="63" t="str">
+        <x:v>Append a UUID-based XFS mount entry to /etc/fstab.</x:v>
+      </x:c>
+      <x:c r="D18" s="63" t="str">
+        <x:v>One-time setup for persistent mounting.</x:v>
+      </x:c>
+      <x:c r="E18" s="63" t="str">
+        <x:v>Replace &lt;VERIFIED_UUID&gt; with actual UUID; do not add a duplicate entry; back up first.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="45" customHeight="1">
+      <x:c r="A19" s="64" t="str">
+        <x:v>sudo findmnt --verify --verbose</x:v>
+      </x:c>
+      <x:c r="B19" s="64" t="str">
+        <x:v>fstab validation</x:v>
+      </x:c>
+      <x:c r="C19" s="64" t="str">
+        <x:v>Validate /etc/fstab mount definitions.</x:v>
+      </x:c>
+      <x:c r="D19" s="64" t="str">
+        <x:v>Immediately after editing fstab and before restarting EC2.</x:v>
+      </x:c>
+      <x:c r="E19" s="64" t="str">
+        <x:v>Verified in lab: success, no errors or warnings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="45" customHeight="1">
+      <x:c r="A20" s="63" t="str">
+        <x:v>sudo mount -a</x:v>
+      </x:c>
+      <x:c r="B20" s="63" t="str">
+        <x:v>Mount validation</x:v>
+      </x:c>
+      <x:c r="C20" s="63" t="str">
+        <x:v>Attempt mounts configured in /etc/fstab.</x:v>
+      </x:c>
+      <x:c r="D20" s="63" t="str">
+        <x:v>Validate the data-volume entry without rebooting.</x:v>
+      </x:c>
+      <x:c r="E20" s="63" t="str">
+        <x:v>Check findmnt afterward; mount -a can affect other fstab entries.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="45" customHeight="1">
+      <x:c r="A21" s="64" t="str">
+        <x:v>sync</x:v>
+      </x:c>
+      <x:c r="B21" s="64" t="str">
+        <x:v>Snapshot preparation</x:v>
+      </x:c>
+      <x:c r="C21" s="64" t="str">
+        <x:v>Flush pending filesystem writes.</x:v>
+      </x:c>
+      <x:c r="D21" s="64" t="str">
+        <x:v>Immediately before requesting the EBS snapshot.</x:v>
+      </x:c>
+      <x:c r="E21" s="64" t="str">
+        <x:v>Improves consistency; application-consistent snapshots may need extra coordination.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="45" customHeight="1">
+      <x:c r="A22" s="63" t="str">
+        <x:v>sudo blkid /dev/nvme2n1</x:v>
+      </x:c>
+      <x:c r="B22" s="63" t="str">
+        <x:v>Restored disk inspection</x:v>
+      </x:c>
+      <x:c r="C22" s="63" t="str">
+        <x:v>Inspect filesystem UUID and type on the restored EBS volume.</x:v>
+      </x:c>
+      <x:c r="D22" s="63" t="str">
+        <x:v>Detect that the restored XFS filesystem duplicates the original UUID.</x:v>
+      </x:c>
+      <x:c r="E22" s="63" t="str">
+        <x:v>Example restored device; verify SERIAL before using it.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="45" customHeight="1">
+      <x:c r="A23" s="64" t="str">
+        <x:v>sudo mkdir -p /data/cloudvault-restored</x:v>
+      </x:c>
+      <x:c r="B23" s="64" t="str">
+        <x:v>Recovery mount point</x:v>
+      </x:c>
+      <x:c r="C23" s="64" t="str">
+        <x:v>Create a separate mount directory for the restored disk.</x:v>
+      </x:c>
+      <x:c r="D23" s="64" t="str">
+        <x:v>Before mounting the restored snapshot copy.</x:v>
+      </x:c>
+      <x:c r="E23" s="64" t="str">
+        <x:v>Keep original and restored volumes mounted at different directories.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="45" customHeight="1">
+      <x:c r="A24" s="63" t="str">
+        <x:v>sudo mount -t xfs -o ro,nouuid,norecovery /dev/nvme2n1 /data/cloudvault-restored</x:v>
+      </x:c>
+      <x:c r="B24" s="63" t="str">
+        <x:v>Safe XFS recovery mount</x:v>
+      </x:c>
+      <x:c r="C24" s="63" t="str">
+        <x:v>Mount the restored XFS filesystem read-only despite duplicate UUID.</x:v>
+      </x:c>
+      <x:c r="D24" s="63" t="str">
+        <x:v>Verify recovery while original XFS filesystem is mounted.</x:v>
+      </x:c>
+      <x:c r="E24" s="63" t="str">
+        <x:v>ro = read-only; nouuid permits duplicate UUID; norecovery avoids journal replay.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="45" customHeight="1">
+      <x:c r="A25" s="64" t="str">
+        <x:v>findmnt /data/cloudvault-restored</x:v>
+      </x:c>
+      <x:c r="B25" s="64" t="str">
+        <x:v>Recovery verification</x:v>
+      </x:c>
+      <x:c r="C25" s="64" t="str">
+        <x:v>Check restored filesystem mount and options.</x:v>
+      </x:c>
+      <x:c r="D25" s="64" t="str">
+        <x:v>Confirm the temporary recovery volume mounted successfully.</x:v>
+      </x:c>
+      <x:c r="E25" s="64" t="str">
+        <x:v>Verify read-only mount and the intended source device.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="45" customHeight="1">
+      <x:c r="A26" s="63" t="str">
+        <x:v>cmp /data/cloudvault/ebs-test.txt /data/cloudvault-restored/ebs-test.txt</x:v>
+      </x:c>
+      <x:c r="B26" s="63" t="str">
+        <x:v>Integrity verification</x:v>
+      </x:c>
+      <x:c r="C26" s="63" t="str">
+        <x:v>Compare original and restored file bytes.</x:v>
+      </x:c>
+      <x:c r="D26" s="63" t="str">
+        <x:v>Verify the snapshot successfully recovered the expected content.</x:v>
+      </x:c>
+      <x:c r="E26" s="63" t="str">
+        <x:v>No output and exit status 0 indicate identical files.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="45" customHeight="1">
+      <x:c r="A27" s="64" t="str">
+        <x:v>sudo umount /data/cloudvault-restored</x:v>
+      </x:c>
+      <x:c r="B27" s="64" t="str">
+        <x:v>Recovery cleanup</x:v>
+      </x:c>
+      <x:c r="C27" s="64" t="str">
+        <x:v>Unmount the temporary restored filesystem.</x:v>
+      </x:c>
+      <x:c r="D27" s="64" t="str">
+        <x:v>Before detaching its EBS volume in AWS.</x:v>
+      </x:c>
+      <x:c r="E27" s="64" t="str">
+        <x:v>Do not detach a mounted filesystem; original remains mounted.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="45" customHeight="1">
+      <x:c r="A28" s="63" t="str">
+        <x:v>findmnt /data/cloudvault-restored</x:v>
+      </x:c>
+      <x:c r="B28" s="63" t="str">
+        <x:v>Cleanup verification</x:v>
+      </x:c>
+      <x:c r="C28" s="63" t="str">
+        <x:v>Check whether the temporary restored mount is still present.</x:v>
+      </x:c>
+      <x:c r="D28" s="63" t="str">
+        <x:v>After unmounting and before detachment.</x:v>
+      </x:c>
+      <x:c r="E28" s="63" t="str">
+        <x:v>No output indicates no mount at that target.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="45" customHeight="1">
+      <x:c r="A29" s="64" t="str">
+        <x:v>aws sts get-caller-identity --query 'Arn' --output text | cut -d/ -f2</x:v>
+      </x:c>
+      <x:c r="B29" s="64" t="str">
+        <x:v>IAM role validation</x:v>
+      </x:c>
+      <x:c r="C29" s="64" t="str">
+        <x:v>Show the instance IAM role name without exposing the full account-specific ARN.</x:v>
+      </x:c>
+      <x:c r="D29" s="64" t="str">
+        <x:v>Verify the EC2 instance uses CloudVaultEC2Role temporary credentials.</x:v>
+      </x:c>
+      <x:c r="E29" s="64" t="str">
+        <x:v>Run inside EC2 SSM Linux shell; never print temporary secret credentials.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="45" customHeight="1">
+      <x:c r="A30" s="63" t="str">
+        <x:v>aws s3api list-objects-v2 --bucket cloudvault-documents-dev01 --prefix documents/</x:v>
+      </x:c>
+      <x:c r="B30" s="63" t="str">
+        <x:v>EC2-to-S3 allowed test</x:v>
+      </x:c>
+      <x:c r="C30" s="63" t="str">
+        <x:v>List objects under the IAM-authorized S3 prefix.</x:v>
+      </x:c>
+      <x:c r="D30" s="63" t="str">
+        <x:v>Validate instance role permissions in the EC2 runtime.</x:v>
+      </x:c>
+      <x:c r="E30" s="63" t="str">
+        <x:v>Expected success for documents/.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="45" customHeight="1">
+      <x:c r="A31" s="64" t="str">
+        <x:v>aws s3api list-objects-v2 --bucket cloudvault-documents-dev01 --prefix private/</x:v>
+      </x:c>
+      <x:c r="B31" s="64" t="str">
+        <x:v>EC2-to-S3 denied test</x:v>
+      </x:c>
+      <x:c r="C31" s="64" t="str">
+        <x:v>Attempt listing a prefix not authorized by the instance IAM policy.</x:v>
+      </x:c>
+      <x:c r="D31" s="64" t="str">
+        <x:v>Validate least-privilege enforcement from EC2.</x:v>
+      </x:c>
+      <x:c r="E31" s="64" t="str">
+        <x:v>Expected AccessDenied; do not broaden policy just to pass a negative test.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="45" customHeight="1">
+      <x:c r="A32" s="63" t="str">
+        <x:v>exit</x:v>
+      </x:c>
+      <x:c r="B32" s="63" t="str">
+        <x:v>Session Manager</x:v>
+      </x:c>
+      <x:c r="C32" s="63" t="str">
+        <x:v>Exit the interactive Linux shell.</x:v>
+      </x:c>
+      <x:c r="D32" s="63" t="str">
+        <x:v>After verifying mounts or before running Windows AWS CLI commands.</x:v>
+      </x:c>
+      <x:c r="E32" s="63" t="str">
+        <x:v>Returns to local PowerShell.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:E1"/>
+    <x:mergeCell ref="A2:E2"/>
+    <x:mergeCell ref="A4:E4"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>